<commit_message>
[CC-002] Crear VERSION y REGLAS_INDICADORES en Excel maestro
- Excel maestro: nuevas hojas REGLAS_INDICADORES (21 columnas, 0 reglas)
  y VERSION (10 columnas; solo la fila "previa a 2.0.0 — sin versión
  formal"). Las 11 hojas existentes no cambian.
- docs/methodology/00-index.md: estado de transición actualizado.
- docs/registro-cambios.md: CC-002 en FUENTE SINCRONIZADA.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q6jJJ6yS7zpSoTqztmBBAw
</commit_message>
<xml_diff>
--- a/docs/excel/Base de Datos Valpo Verde.xlsx
+++ b/docs/excel/Base de Datos Valpo Verde.xlsx
@@ -24,6 +24,8 @@
     <sheet name="DICCIONARIO_CAMPOS" sheetId="14" r:id="rId9"/>
     <sheet name="MATRICES_CALCULO" sheetId="15" r:id="rId10"/>
     <sheet name="INDICES" sheetId="17" r:id="rId11"/>
+    <sheet name="REGLAS_INDICADORES" sheetId="18" r:id="rId15"/>
+    <sheet name="VERSION" sheetId="19" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="Descompactación">LISTAS!$I$2:$I$3</definedName>
@@ -4394,6 +4396,281 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:U1"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+    <col min="7" max="7" width="60" customWidth="1"/>
+    <col min="8" max="8" width="30" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
+    <col min="10" max="10" width="9" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="12" max="12" width="12" customWidth="1"/>
+    <col min="13" max="13" width="9" customWidth="1"/>
+    <col min="14" max="14" width="13" customWidth="1"/>
+    <col min="15" max="15" width="12" customWidth="1"/>
+    <col min="16" max="16" width="12" customWidth="1"/>
+    <col min="17" max="17" width="14" customWidth="1"/>
+    <col min="18" max="18" width="9" customWidth="1"/>
+    <col min="19" max="19" width="30" customWidth="1"/>
+    <col min="20" max="20" width="24" customWidth="1"/>
+    <col min="21" max="21" width="40" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">id_regla</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">componente</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">codigo_indicador</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">indicador</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tipo_regla</t>
+        </is>
+      </c>
+      <c r="F1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">orden</t>
+        </is>
+      </c>
+      <c r="G1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">condicion</t>
+        </is>
+      </c>
+      <c r="H1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">campos_utilizados</t>
+        </is>
+      </c>
+      <c r="I1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">resultado</t>
+        </is>
+      </c>
+      <c r="J1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">puntaje</t>
+        </is>
+      </c>
+      <c r="K1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">regla_agregadora</t>
+        </is>
+      </c>
+      <c r="L1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">max_indicador</t>
+        </is>
+      </c>
+      <c r="M1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">residual</t>
+        </is>
+      </c>
+      <c r="N1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">estado_regla</t>
+        </is>
+      </c>
+      <c r="O1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">version_desde</t>
+        </is>
+      </c>
+      <c r="P1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">version_hasta</t>
+        </is>
+      </c>
+      <c r="Q1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">reemplazada_por</t>
+        </is>
+      </c>
+      <c r="R1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cc</t>
+        </is>
+      </c>
+      <c r="S1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fundamento_fuente</t>
+        </is>
+      </c>
+      <c r="T1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">diagrama_ref</t>
+        </is>
+      </c>
+      <c r="U1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">observaciones</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="9">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:B5000">
+      <formula1>"Raíces y cuello,Tronco,Copa y ramas,Infraestructura"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E2:E5000">
+      <formula1>"clasificación,ajuste,aplicabilidad"</formula1>
+    </dataValidation>
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" sqref="F2:F5000">
+      <formula1>1</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I2:I5000">
+      <formula1>"Despreciable,Sin afectación,Leve,Moderada,Severa,No determinado,No aplica,Mantener clasificación,Mínimo Moderada"</formula1>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" sqref="J2:J5000">
+      <formula1>0</formula1>
+      <formula2>3</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="K2:K5000">
+      <formula1>"R01,R02,R03,M04,ninguna"</formula1>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" sqref="L2:L5000">
+      <formula1>0</formula1>
+      <formula2>3</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="M2:M5000">
+      <formula1>"Sí,No"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="N2:N5000">
+      <formula1>"vigente,pendiente,reemplazada,descartada"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="13" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="17" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="15" customWidth="1"/>
+    <col min="7" max="7" width="17" customWidth="1"/>
+    <col min="8" max="8" width="24" customWidth="1"/>
+    <col min="9" max="9" width="16" customWidth="1"/>
+    <col min="10" max="10" width="80" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">version_paquete</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rule_version</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">estado</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fecha_publicacion</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cc_incluidos</t>
+        </is>
+      </c>
+      <c r="F1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">aprobado_por</t>
+        </is>
+      </c>
+      <c r="G1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fecha_aprobacion</t>
+        </is>
+      </c>
+      <c r="H1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tag_git</t>
+        </is>
+      </c>
+      <c r="I1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">version_anterior</t>
+        </is>
+      </c>
+      <c r="J1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">observaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">previa a 2.0.0</t>
+        </is>
+      </c>
+      <c r="C2" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sin versión formal</t>
+        </is>
+      </c>
+      <c r="E2" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-002</t>
+        </is>
+      </c>
+      <c r="J2" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Excel maestro sin versión formal (contenido subido el 2026-10-04, commit 24e8cae). NO constituye el paquete metodológico 2.0.0 ni una versión publicada y no define rule_version. Contiene inconsistencias internas detectadas en la auditoría de diagramas (p. ej. rangos de R02 y R03 distintos entre MATRICES_CALCULO y DICCIONARIO_CAMPOS). Las hojas REGLAS_INDICADORES y VERSION fueron agregadas por CC-002, sin reglas cargadas.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C1000">
+      <formula1>"en preparación,publicada,reemplazada,sin versión formal"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F2:F1000">
+      <formula1>"marybaxmann,Valen-j211"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:DX1"/>

</xml_diff>

<commit_message>
[CC-004] Normalizar catálogos LISTAS y referencias del diccionario
- LISTAS: tabla normalizada P:X (12 catálogos, 70 valores vigentes):
  tipo_ot, accion, subtipo_accion, confirmacion_cavidad_interna y 8
  escalas. Bloque A1:N9 y 14 rangos con nombre intactos, rotulados como
  técnicos y derivados (retiro en CC-012).
- DICCIONARIO_CAMPOS: 19 celdas de "Unidad / valores" y 10 frases de
  enumeración en "Validación" remiten a LISTAS:<id_catalogo>.
- VERSION: fila 2.0.0 en preparación (cc_incluidos CC-004), sin
  rule_version.
- docs/methodology/convenciones-catalogos.md (nuevo).
- workflow.md §14.9: controles de sincronización de catálogos.
- registro-cambios.md: ficha CC-004 (FUENTE SINCRONIZADA); anotaciones en
  CC-007 y CC-018.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q6jJJ6yS7zpSoTqztmBBAw
</commit_message>
<xml_diff>
--- a/docs/excel/Base de Datos Valpo Verde.xlsx
+++ b/docs/excel/Base de Datos Valpo Verde.xlsx
@@ -4569,7 +4569,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -4655,6 +4655,33 @@
       <c r="J2" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">Excel maestro sin versión formal (contenido subido el 2026-10-04, commit 24e8cae). NO constituye el paquete metodológico 2.0.0 ni una versión publicada y no define rule_version. Contiene inconsistencias internas detectadas en la auditoría de diagramas (p. ej. rangos de R02 y R03 distintos entre MATRICES_CALCULO y DICCIONARIO_CAMPOS). Las hojas REGLAS_INDICADORES y VERSION fueron agregadas por CC-002, sin reglas cargadas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2.0.0</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">en preparación</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+      <c r="I3" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">previa a 2.0.0</t>
+        </is>
+      </c>
+      <c r="J3" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paquete metodológico en construcción. NO publicado; no define rule_version. Acumula los CC aprobados que se incorporen al paquete 2.0.0. CC-004 no publica la metodología 2.0.0.</t>
         </is>
       </c>
     </row>
@@ -5772,14 +5799,21 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:X71"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="8.88671875" customWidth="1"/>
+    <col min="16" max="16" width="34" customWidth="1"/>
+    <col min="17" max="17" width="32" customWidth="1"/>
+    <col min="18" max="18" width="40" customWidth="1"/>
+    <col min="19" max="19" width="8" customWidth="1"/>
+    <col min="20" max="21" width="22" customWidth="1"/>
+    <col min="22" max="23" width="12" customWidth="1"/>
+    <col min="24" max="24" width="80" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>171</v>
       </c>
@@ -5822,8 +5856,53 @@
       <c r="N1" t="s">
         <v>209</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">id_catalogo</t>
+        </is>
+      </c>
+      <c r="Q1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">codigo</t>
+        </is>
+      </c>
+      <c r="R1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">etiqueta</t>
+        </is>
+      </c>
+      <c r="S1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">orden</t>
+        </is>
+      </c>
+      <c r="T1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">catalogo_padre</t>
+        </is>
+      </c>
+      <c r="U1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">codigo_padre</t>
+        </is>
+      </c>
+      <c r="V1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">estado_valor</t>
+        </is>
+      </c>
+      <c r="W1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cc</t>
+        </is>
+      </c>
+      <c r="X1" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">observaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>133</v>
       </c>
@@ -5860,8 +5939,33 @@
       <c r="N2" t="s">
         <v>219</v>
       </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P2" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tipo_ot</t>
+        </is>
+      </c>
+      <c r="Q2" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">inspeccion</t>
+        </is>
+      </c>
+      <c r="R2" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Inspección</t>
+        </is>
+      </c>
+      <c r="V2" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W2" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>200</v>
       </c>
@@ -5898,8 +6002,33 @@
       <c r="N3" t="s">
         <v>227</v>
       </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P3" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tipo_ot</t>
+        </is>
+      </c>
+      <c r="Q3" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mantenimiento</t>
+        </is>
+      </c>
+      <c r="R3" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mantenimiento</t>
+        </is>
+      </c>
+      <c r="V3" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W3" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>178</v>
       </c>
@@ -5924,8 +6053,43 @@
       <c r="N4" t="s">
         <v>231</v>
       </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P4" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accion</t>
+        </is>
+      </c>
+      <c r="Q4" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">evaluacion_inicial</t>
+        </is>
+      </c>
+      <c r="R4" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evaluación inicial</t>
+        </is>
+      </c>
+      <c r="T4" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tipo_ot</t>
+        </is>
+      </c>
+      <c r="U4" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">inspeccion</t>
+        </is>
+      </c>
+      <c r="V4" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W4" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>202</v>
       </c>
@@ -5941,8 +6105,43 @@
       <c r="N5" t="s">
         <v>235</v>
       </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P5" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accion</t>
+        </is>
+      </c>
+      <c r="Q5" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">reevaluacion</t>
+        </is>
+      </c>
+      <c r="R5" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reevaluación</t>
+        </is>
+      </c>
+      <c r="T5" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tipo_ot</t>
+        </is>
+      </c>
+      <c r="U5" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">inspeccion</t>
+        </is>
+      </c>
+      <c r="V5" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W5" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>206</v>
       </c>
@@ -5952,29 +6151,2384 @@
       <c r="N6" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P6" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accion</t>
+        </is>
+      </c>
+      <c r="Q6" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">evaluacion_instrumental</t>
+        </is>
+      </c>
+      <c r="R6" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evaluación instrumental</t>
+        </is>
+      </c>
+      <c r="T6" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tipo_ot</t>
+        </is>
+      </c>
+      <c r="U6" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">inspeccion</t>
+        </is>
+      </c>
+      <c r="V6" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W6" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" spans="1:24" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>238</v>
       </c>
       <c r="M7" t="s">
         <v>239</v>
       </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P7" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accion</t>
+        </is>
+      </c>
+      <c r="Q7" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">monitoreo</t>
+        </is>
+      </c>
+      <c r="R7" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Monitoreo</t>
+        </is>
+      </c>
+      <c r="T7" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tipo_ot</t>
+        </is>
+      </c>
+      <c r="U7" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">inspeccion</t>
+        </is>
+      </c>
+      <c r="V7" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W7" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" spans="1:24" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>240</v>
       </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="P8" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accion</t>
+        </is>
+      </c>
+      <c r="Q8" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">poda</t>
+        </is>
+      </c>
+      <c r="R8" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Poda</t>
+        </is>
+      </c>
+      <c r="T8" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tipo_ot</t>
+        </is>
+      </c>
+      <c r="U8" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mantenimiento</t>
+        </is>
+      </c>
+      <c r="V8" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W8" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>207</v>
+      </c>
+      <c r="P9" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accion</t>
+        </is>
+      </c>
+      <c r="Q9" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">riego</t>
+        </is>
+      </c>
+      <c r="R9" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Riego</t>
+        </is>
+      </c>
+      <c r="T9" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tipo_ot</t>
+        </is>
+      </c>
+      <c r="U9" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mantenimiento</t>
+        </is>
+      </c>
+      <c r="V9" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W9" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="P10" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accion</t>
+        </is>
+      </c>
+      <c r="Q10" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">descompactacion</t>
+        </is>
+      </c>
+      <c r="R10" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Descompactación</t>
+        </is>
+      </c>
+      <c r="T10" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tipo_ot</t>
+        </is>
+      </c>
+      <c r="U10" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mantenimiento</t>
+        </is>
+      </c>
+      <c r="V10" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W10" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BLOQUE TÉCNICO A1:N9 — derivado para los menús actuales del Excel. No editar. No es fuente de valores. La fuente es la tabla P:X. Será regenerado y retirado por CC-012.</t>
+        </is>
+      </c>
+      <c r="P11" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accion</t>
+        </is>
+      </c>
+      <c r="Q11" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">manejo_fitosanitario</t>
+        </is>
+      </c>
+      <c r="R11" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manejo fitosanitario</t>
+        </is>
+      </c>
+      <c r="T11" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tipo_ot</t>
+        </is>
+      </c>
+      <c r="U11" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mantenimiento</t>
+        </is>
+      </c>
+      <c r="V11" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W11" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="P12" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accion</t>
+        </is>
+      </c>
+      <c r="Q12" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tala_retiro</t>
+        </is>
+      </c>
+      <c r="R12" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tala / retiro</t>
+        </is>
+      </c>
+      <c r="T12" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tipo_ot</t>
+        </is>
+      </c>
+      <c r="U12" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mantenimiento</t>
+        </is>
+      </c>
+      <c r="V12" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W12" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="P13" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accion</t>
+        </is>
+      </c>
+      <c r="Q13" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">reparacion_alcorque</t>
+        </is>
+      </c>
+      <c r="R13" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reparación de alcorque</t>
+        </is>
+      </c>
+      <c r="T13" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tipo_ot</t>
+        </is>
+      </c>
+      <c r="U13" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mantenimiento</t>
+        </is>
+      </c>
+      <c r="V13" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W13" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="P14" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accion</t>
+        </is>
+      </c>
+      <c r="Q14" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">soporte_tutorado</t>
+        </is>
+      </c>
+      <c r="R14" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Soporte / tutorado</t>
+        </is>
+      </c>
+      <c r="T14" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tipo_ot</t>
+        </is>
+      </c>
+      <c r="U14" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mantenimiento</t>
+        </is>
+      </c>
+      <c r="V14" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W14" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="P15" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accion</t>
+        </is>
+      </c>
+      <c r="Q15" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">otra_intervencion</t>
+        </is>
+      </c>
+      <c r="R15" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Otra intervención</t>
+        </is>
+      </c>
+      <c r="T15" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tipo_ot</t>
+        </is>
+      </c>
+      <c r="U15" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mantenimiento</t>
+        </is>
+      </c>
+      <c r="V15" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W15" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="P16" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">subtipo_accion</t>
+        </is>
+      </c>
+      <c r="Q16" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">seguimiento</t>
+        </is>
+      </c>
+      <c r="R16" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Seguimiento</t>
+        </is>
+      </c>
+      <c r="T16" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accion</t>
+        </is>
+      </c>
+      <c r="U16" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">reevaluacion</t>
+        </is>
+      </c>
+      <c r="V16" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W16" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="P17" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">subtipo_accion</t>
+        </is>
+      </c>
+      <c r="Q17" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">post_intervencion</t>
+        </is>
+      </c>
+      <c r="R17" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Post intervención</t>
+        </is>
+      </c>
+      <c r="T17" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accion</t>
+        </is>
+      </c>
+      <c r="U17" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">reevaluacion</t>
+        </is>
+      </c>
+      <c r="V17" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W17" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="P18" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">subtipo_accion</t>
+        </is>
+      </c>
+      <c r="Q18" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tomografia_sonica</t>
+        </is>
+      </c>
+      <c r="R18" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tomografía sónica</t>
+        </is>
+      </c>
+      <c r="T18" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accion</t>
+        </is>
+      </c>
+      <c r="U18" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">evaluacion_instrumental</t>
+        </is>
+      </c>
+      <c r="V18" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W18" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="P19" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">subtipo_accion</t>
+        </is>
+      </c>
+      <c r="Q19" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">resistografia</t>
+        </is>
+      </c>
+      <c r="R19" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Resistografía</t>
+        </is>
+      </c>
+      <c r="T19" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accion</t>
+        </is>
+      </c>
+      <c r="U19" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">evaluacion_instrumental</t>
+        </is>
+      </c>
+      <c r="V19" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W19" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="P20" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">subtipo_accion</t>
+        </is>
+      </c>
+      <c r="Q20" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">otra</t>
+        </is>
+      </c>
+      <c r="R20" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Otra</t>
+        </is>
+      </c>
+      <c r="T20" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accion</t>
+        </is>
+      </c>
+      <c r="U20" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">evaluacion_instrumental</t>
+        </is>
+      </c>
+      <c r="V20" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W20" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+      <c r="X20" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Requiere especificar en observaciones (obligatorio).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="P21" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">subtipo_accion</t>
+        </is>
+      </c>
+      <c r="Q21" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fitosanitario</t>
+        </is>
+      </c>
+      <c r="R21" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fitosanitario</t>
+        </is>
+      </c>
+      <c r="T21" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accion</t>
+        </is>
+      </c>
+      <c r="U21" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">monitoreo</t>
+        </is>
+      </c>
+      <c r="V21" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W21" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="P22" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">subtipo_accion</t>
+        </is>
+      </c>
+      <c r="Q22" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">estructural</t>
+        </is>
+      </c>
+      <c r="R22" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estructural</t>
+        </is>
+      </c>
+      <c r="T22" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accion</t>
+        </is>
+      </c>
+      <c r="U22" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">monitoreo</t>
+        </is>
+      </c>
+      <c r="V22" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W22" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="P23" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">subtipo_accion</t>
+        </is>
+      </c>
+      <c r="Q23" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vitalidad</t>
+        </is>
+      </c>
+      <c r="R23" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vitalidad</t>
+        </is>
+      </c>
+      <c r="T23" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accion</t>
+        </is>
+      </c>
+      <c r="U23" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">monitoreo</t>
+        </is>
+      </c>
+      <c r="V23" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W23" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="P24" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">subtipo_accion</t>
+        </is>
+      </c>
+      <c r="Q24" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sanitaria</t>
+        </is>
+      </c>
+      <c r="R24" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sanitaria</t>
+        </is>
+      </c>
+      <c r="T24" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accion</t>
+        </is>
+      </c>
+      <c r="U24" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">poda</t>
+        </is>
+      </c>
+      <c r="V24" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W24" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="P25" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">subtipo_accion</t>
+        </is>
+      </c>
+      <c r="Q25" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">formacion</t>
+        </is>
+      </c>
+      <c r="R25" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Formación</t>
+        </is>
+      </c>
+      <c r="T25" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accion</t>
+        </is>
+      </c>
+      <c r="U25" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">poda</t>
+        </is>
+      </c>
+      <c r="V25" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W25" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="P26" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">subtipo_accion</t>
+        </is>
+      </c>
+      <c r="Q26" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">despeje</t>
+        </is>
+      </c>
+      <c r="R26" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Despeje</t>
+        </is>
+      </c>
+      <c r="T26" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accion</t>
+        </is>
+      </c>
+      <c r="U26" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">poda</t>
+        </is>
+      </c>
+      <c r="V26" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W26" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="P27" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">subtipo_accion</t>
+        </is>
+      </c>
+      <c r="Q27" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">reduccion</t>
+        </is>
+      </c>
+      <c r="R27" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reducción</t>
+        </is>
+      </c>
+      <c r="T27" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accion</t>
+        </is>
+      </c>
+      <c r="U27" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">poda</t>
+        </is>
+      </c>
+      <c r="V27" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W27" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="P28" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">subtipo_accion</t>
+        </is>
+      </c>
+      <c r="Q28" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">programado</t>
+        </is>
+      </c>
+      <c r="R28" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Programado</t>
+        </is>
+      </c>
+      <c r="T28" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accion</t>
+        </is>
+      </c>
+      <c r="U28" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">riego</t>
+        </is>
+      </c>
+      <c r="V28" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W28" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="P29" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">subtipo_accion</t>
+        </is>
+      </c>
+      <c r="Q29" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">emergencia</t>
+        </is>
+      </c>
+      <c r="R29" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Emergencia</t>
+        </is>
+      </c>
+      <c r="T29" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accion</t>
+        </is>
+      </c>
+      <c r="U29" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">riego</t>
+        </is>
+      </c>
+      <c r="V29" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W29" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="P30" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">subtipo_accion</t>
+        </is>
+      </c>
+      <c r="Q30" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">manual</t>
+        </is>
+      </c>
+      <c r="R30" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="T30" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accion</t>
+        </is>
+      </c>
+      <c r="U30" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">descompactacion</t>
+        </is>
+      </c>
+      <c r="V30" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W30" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="P31" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">subtipo_accion</t>
+        </is>
+      </c>
+      <c r="Q31" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mecanica</t>
+        </is>
+      </c>
+      <c r="R31" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mecánica</t>
+        </is>
+      </c>
+      <c r="T31" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accion</t>
+        </is>
+      </c>
+      <c r="U31" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">descompactacion</t>
+        </is>
+      </c>
+      <c r="V31" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W31" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="P32" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">subtipo_accion</t>
+        </is>
+      </c>
+      <c r="Q32" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">preventivo</t>
+        </is>
+      </c>
+      <c r="R32" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Preventivo</t>
+        </is>
+      </c>
+      <c r="T32" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accion</t>
+        </is>
+      </c>
+      <c r="U32" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">manejo_fitosanitario</t>
+        </is>
+      </c>
+      <c r="V32" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W32" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="P33" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">subtipo_accion</t>
+        </is>
+      </c>
+      <c r="Q33" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">correctivo</t>
+        </is>
+      </c>
+      <c r="R33" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Correctivo</t>
+        </is>
+      </c>
+      <c r="T33" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accion</t>
+        </is>
+      </c>
+      <c r="U33" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">manejo_fitosanitario</t>
+        </is>
+      </c>
+      <c r="V33" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W33" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="P34" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">subtipo_accion</t>
+        </is>
+      </c>
+      <c r="Q34" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tala</t>
+        </is>
+      </c>
+      <c r="R34" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tala</t>
+        </is>
+      </c>
+      <c r="T34" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accion</t>
+        </is>
+      </c>
+      <c r="U34" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tala_retiro</t>
+        </is>
+      </c>
+      <c r="V34" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W34" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="P35" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">subtipo_accion</t>
+        </is>
+      </c>
+      <c r="Q35" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">retiro_tocon</t>
+        </is>
+      </c>
+      <c r="R35" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Retiro de tocón</t>
+        </is>
+      </c>
+      <c r="T35" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accion</t>
+        </is>
+      </c>
+      <c r="U35" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tala_retiro</t>
+        </is>
+      </c>
+      <c r="V35" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W35" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="P36" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">subtipo_accion</t>
+        </is>
+      </c>
+      <c r="Q36" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">retiro_residuos</t>
+        </is>
+      </c>
+      <c r="R36" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Retiro de residuos</t>
+        </is>
+      </c>
+      <c r="T36" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">accion</t>
+        </is>
+      </c>
+      <c r="U36" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tala_retiro</t>
+        </is>
+      </c>
+      <c r="V36" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W36" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="P37" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">confirmacion_cavidad_interna</t>
+        </is>
+      </c>
+      <c r="Q37" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">si</t>
+        </is>
+      </c>
+      <c r="R37" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sí</t>
+        </is>
+      </c>
+      <c r="V37" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W37" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="P38" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">confirmacion_cavidad_interna</t>
+        </is>
+      </c>
+      <c r="Q38" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no</t>
+        </is>
+      </c>
+      <c r="R38" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="V38" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W38" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="P39" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">confirmacion_cavidad_interna</t>
+        </is>
+      </c>
+      <c r="Q39" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">requiere_evaluacion_instrumental</t>
+        </is>
+      </c>
+      <c r="R39" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Requiere evaluación instrumental</t>
+        </is>
+      </c>
+      <c r="V39" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W39" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="P40" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">escala_probabilidad_falla</t>
+        </is>
+      </c>
+      <c r="Q40" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">improbable</t>
+        </is>
+      </c>
+      <c r="R40" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Improbable</t>
+        </is>
+      </c>
+      <c r="S40" s="13">
+        <v>1</v>
+      </c>
+      <c r="V40" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W40" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+      <c r="X40" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Representación. Autoridad: R01–R03 (resultado); M02 (entrada). LISTAS no define la lógica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="P41" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">escala_probabilidad_falla</t>
+        </is>
+      </c>
+      <c r="Q41" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">posible</t>
+        </is>
+      </c>
+      <c r="R41" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Posible</t>
+        </is>
+      </c>
+      <c r="S41" s="13">
+        <v>2</v>
+      </c>
+      <c r="V41" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W41" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+      <c r="X41" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Representación. Autoridad: R01–R03 (resultado); M02 (entrada). LISTAS no define la lógica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="P42" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">escala_probabilidad_falla</t>
+        </is>
+      </c>
+      <c r="Q42" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">probable</t>
+        </is>
+      </c>
+      <c r="R42" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Probable</t>
+        </is>
+      </c>
+      <c r="S42" s="13">
+        <v>3</v>
+      </c>
+      <c r="V42" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W42" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+      <c r="X42" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Representación. Autoridad: R01–R03 (resultado); M02 (entrada). LISTAS no define la lógica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="P43" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">escala_probabilidad_falla</t>
+        </is>
+      </c>
+      <c r="Q43" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">inminente</t>
+        </is>
+      </c>
+      <c r="R43" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Inminente</t>
+        </is>
+      </c>
+      <c r="S43" s="13">
+        <v>4</v>
+      </c>
+      <c r="V43" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W43" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+      <c r="X43" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Representación. Autoridad: R01–R03 (resultado); M02 (entrada). LISTAS no define la lógica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="P44" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">escala_nivel_riesgo</t>
+        </is>
+      </c>
+      <c r="Q44" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bajo</t>
+        </is>
+      </c>
+      <c r="R44" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bajo</t>
+        </is>
+      </c>
+      <c r="S44" s="13">
+        <v>1</v>
+      </c>
+      <c r="V44" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W44" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+      <c r="X44" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Representación. Autoridad: M03 (resultado); R04; M05 (entrada). LISTAS no define la lógica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="P45" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">escala_nivel_riesgo</t>
+        </is>
+      </c>
+      <c r="Q45" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">moderado</t>
+        </is>
+      </c>
+      <c r="R45" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moderado</t>
+        </is>
+      </c>
+      <c r="S45" s="13">
+        <v>2</v>
+      </c>
+      <c r="V45" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W45" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+      <c r="X45" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Representación. Autoridad: M03 (resultado); R04; M05 (entrada). LISTAS no define la lógica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="P46" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">escala_nivel_riesgo</t>
+        </is>
+      </c>
+      <c r="Q46" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">alto</t>
+        </is>
+      </c>
+      <c r="R46" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alto</t>
+        </is>
+      </c>
+      <c r="S46" s="13">
+        <v>3</v>
+      </c>
+      <c r="V46" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W46" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+      <c r="X46" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Representación. Autoridad: M03 (resultado); R04; M05 (entrada). LISTAS no define la lógica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="P47" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">escala_nivel_riesgo</t>
+        </is>
+      </c>
+      <c r="Q47" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">extremo</t>
+        </is>
+      </c>
+      <c r="R47" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extremo</t>
+        </is>
+      </c>
+      <c r="S47" s="13">
+        <v>4</v>
+      </c>
+      <c r="V47" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W47" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+      <c r="X47" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Representación. Autoridad: M03 (resultado); R04; M05 (entrada). LISTAS no define la lógica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="P48" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">escala_consecuencia</t>
+        </is>
+      </c>
+      <c r="Q48" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">despreciable</t>
+        </is>
+      </c>
+      <c r="R48" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Despreciable</t>
+        </is>
+      </c>
+      <c r="S48" s="13">
+        <v>1</v>
+      </c>
+      <c r="V48" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W48" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+      <c r="X48" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Representación. Autoridad: M03 (entrada). LISTAS no define la lógica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="P49" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">escala_consecuencia</t>
+        </is>
+      </c>
+      <c r="Q49" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">menor</t>
+        </is>
+      </c>
+      <c r="R49" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Menor</t>
+        </is>
+      </c>
+      <c r="S49" s="13">
+        <v>2</v>
+      </c>
+      <c r="V49" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W49" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+      <c r="X49" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Representación. Autoridad: M03 (entrada). LISTAS no define la lógica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="P50" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">escala_consecuencia</t>
+        </is>
+      </c>
+      <c r="Q50" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">significativa</t>
+        </is>
+      </c>
+      <c r="R50" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Significativa</t>
+        </is>
+      </c>
+      <c r="S50" s="13">
+        <v>3</v>
+      </c>
+      <c r="V50" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W50" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+      <c r="X50" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Representación. Autoridad: M03 (entrada). LISTAS no define la lógica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="P51" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">escala_consecuencia</t>
+        </is>
+      </c>
+      <c r="Q51" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">severa</t>
+        </is>
+      </c>
+      <c r="R51" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Severa</t>
+        </is>
+      </c>
+      <c r="S51" s="13">
+        <v>4</v>
+      </c>
+      <c r="V51" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W51" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+      <c r="X51" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Representación. Autoridad: M03 (entrada). LISTAS no define la lógica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="P52" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">escala_probabilidad_impacto</t>
+        </is>
+      </c>
+      <c r="Q52" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">muy_baja</t>
+        </is>
+      </c>
+      <c r="R52" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Muy baja</t>
+        </is>
+      </c>
+      <c r="S52" s="13">
+        <v>1</v>
+      </c>
+      <c r="V52" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W52" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+      <c r="X52" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Representación. Autoridad: M01 (resultado); M02 (entrada). LISTAS no define la lógica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="P53" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">escala_probabilidad_impacto</t>
+        </is>
+      </c>
+      <c r="Q53" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">baja</t>
+        </is>
+      </c>
+      <c r="R53" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Baja</t>
+        </is>
+      </c>
+      <c r="S53" s="13">
+        <v>2</v>
+      </c>
+      <c r="V53" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W53" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+      <c r="X53" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Representación. Autoridad: M01 (resultado); M02 (entrada). LISTAS no define la lógica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="P54" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">escala_probabilidad_impacto</t>
+        </is>
+      </c>
+      <c r="Q54" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">media</t>
+        </is>
+      </c>
+      <c r="R54" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Media</t>
+        </is>
+      </c>
+      <c r="S54" s="13">
+        <v>3</v>
+      </c>
+      <c r="V54" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W54" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+      <c r="X54" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Representación. Autoridad: M01 (resultado); M02 (entrada). LISTAS no define la lógica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="P55" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">escala_probabilidad_impacto</t>
+        </is>
+      </c>
+      <c r="Q55" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">alta</t>
+        </is>
+      </c>
+      <c r="R55" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alta</t>
+        </is>
+      </c>
+      <c r="S55" s="13">
+        <v>4</v>
+      </c>
+      <c r="V55" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W55" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+      <c r="X55" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Representación. Autoridad: M01 (resultado); M02 (entrada). LISTAS no define la lógica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="P56" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">escala_zona_objetivo</t>
+        </is>
+      </c>
+      <c r="Q56" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bajo_copa</t>
+        </is>
+      </c>
+      <c r="R56" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bajo la copa</t>
+        </is>
+      </c>
+      <c r="S56" s="13">
+        <v>1</v>
+      </c>
+      <c r="V56" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W56" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+      <c r="X56" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Representación. Autoridad: M01 (entrada). LISTAS no define la lógica. Las filas de M01 usan la forma corta de la etiqueta. Se alinearán en la sincronización del paquete 2.0.0. MATRICES_CALCULO no se modifica en CC-004.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="P57" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">escala_zona_objetivo</t>
+        </is>
+      </c>
+      <c r="Q57" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">limite_copa_1x_altura</t>
+        </is>
+      </c>
+      <c r="R57" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entre el límite de la copa y 1× la altura del árbol</t>
+        </is>
+      </c>
+      <c r="S57" s="13">
+        <v>2</v>
+      </c>
+      <c r="V57" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W57" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+      <c r="X57" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Representación. Autoridad: M01 (entrada). LISTAS no define la lógica. Las filas de M01 usan la forma corta de la etiqueta. Se alinearán en la sincronización del paquete 2.0.0. MATRICES_CALCULO no se modifica en CC-004.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="P58" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">escala_zona_objetivo</t>
+        </is>
+      </c>
+      <c r="Q58" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">entre_1x_1_5x_altura</t>
+        </is>
+      </c>
+      <c r="R58" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entre 1× y 1,5× la altura del árbol</t>
+        </is>
+      </c>
+      <c r="S58" s="13">
+        <v>3</v>
+      </c>
+      <c r="V58" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W58" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+      <c r="X58" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Representación. Autoridad: M01 (entrada). LISTAS no define la lógica. Las filas de M01 usan la forma corta de la etiqueta. Se alinearán en la sincronización del paquete 2.0.0. MATRICES_CALCULO no se modifica en CC-004.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="P59" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">escala_zona_objetivo</t>
+        </is>
+      </c>
+      <c r="Q59" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mas_alla_1_5x_altura</t>
+        </is>
+      </c>
+      <c r="R59" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Más allá de 1,5× la altura del árbol</t>
+        </is>
+      </c>
+      <c r="S59" s="13">
+        <v>4</v>
+      </c>
+      <c r="V59" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W59" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+      <c r="X59" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Representación. Autoridad: M01 (entrada). LISTAS no define la lógica. Las filas de M01 usan la forma corta de la etiqueta. Se alinearán en la sincronización del paquete 2.0.0. MATRICES_CALCULO no se modifica en CC-004.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="P60" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">escala_tasa_ocupacion</t>
+        </is>
+      </c>
+      <c r="Q60" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rara</t>
+        </is>
+      </c>
+      <c r="R60" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rara</t>
+        </is>
+      </c>
+      <c r="S60" s="13">
+        <v>1</v>
+      </c>
+      <c r="V60" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W60" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+      <c r="X60" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Representación. Autoridad: M01 (entrada). LISTAS no define la lógica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="P61" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">escala_tasa_ocupacion</t>
+        </is>
+      </c>
+      <c r="Q61" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ocasional</t>
+        </is>
+      </c>
+      <c r="R61" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ocasional</t>
+        </is>
+      </c>
+      <c r="S61" s="13">
+        <v>2</v>
+      </c>
+      <c r="V61" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W61" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+      <c r="X61" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Representación. Autoridad: M01 (entrada). LISTAS no define la lógica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="P62" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">escala_tasa_ocupacion</t>
+        </is>
+      </c>
+      <c r="Q62" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">frecuente</t>
+        </is>
+      </c>
+      <c r="R62" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Frecuente</t>
+        </is>
+      </c>
+      <c r="S62" s="13">
+        <v>3</v>
+      </c>
+      <c r="V62" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W62" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+      <c r="X62" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Representación. Autoridad: M01 (entrada). LISTAS no define la lógica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="P63" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">escala_tasa_ocupacion</t>
+        </is>
+      </c>
+      <c r="Q63" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">constante</t>
+        </is>
+      </c>
+      <c r="R63" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Constante</t>
+        </is>
+      </c>
+      <c r="S63" s="13">
+        <v>4</v>
+      </c>
+      <c r="V63" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W63" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+      <c r="X63" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Representación. Autoridad: M01 (entrada). LISTAS no define la lógica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="P64" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">escala_clasificacion_infraestructura</t>
+        </is>
+      </c>
+      <c r="Q64" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bajo</t>
+        </is>
+      </c>
+      <c r="R64" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bajo</t>
+        </is>
+      </c>
+      <c r="S64" s="13">
+        <v>1</v>
+      </c>
+      <c r="V64" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W64" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+      <c r="X64" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Representación. Autoridad: M04 (resultado); M05 (entrada). LISTAS no define la lógica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="P65" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">escala_clasificacion_infraestructura</t>
+        </is>
+      </c>
+      <c r="Q65" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">moderado</t>
+        </is>
+      </c>
+      <c r="R65" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moderado</t>
+        </is>
+      </c>
+      <c r="S65" s="13">
+        <v>2</v>
+      </c>
+      <c r="V65" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W65" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+      <c r="X65" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Representación. Autoridad: M04 (resultado); M05 (entrada). LISTAS no define la lógica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="P66" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">escala_clasificacion_infraestructura</t>
+        </is>
+      </c>
+      <c r="Q66" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">alto</t>
+        </is>
+      </c>
+      <c r="R66" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alto</t>
+        </is>
+      </c>
+      <c r="S66" s="13">
+        <v>3</v>
+      </c>
+      <c r="V66" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W66" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+      <c r="X66" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Representación. Autoridad: M04 (resultado); M05 (entrada). LISTAS no define la lógica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="P67" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">escala_clasificacion_infraestructura</t>
+        </is>
+      </c>
+      <c r="Q67" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">critico</t>
+        </is>
+      </c>
+      <c r="R67" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Crítico</t>
+        </is>
+      </c>
+      <c r="S67" s="13">
+        <v>4</v>
+      </c>
+      <c r="V67" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W67" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+      <c r="X67" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Representación. Autoridad: M04 (resultado); M05 (entrada). LISTAS no define la lógica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="P68" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">escala_prioridad</t>
+        </is>
+      </c>
+      <c r="Q68" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">baja</t>
+        </is>
+      </c>
+      <c r="R68" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Baja</t>
+        </is>
+      </c>
+      <c r="S68" s="13">
+        <v>1</v>
+      </c>
+      <c r="V68" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W68" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+      <c r="X68" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Representación. Autoridad: M05 (resultado). LISTAS no define la lógica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="P69" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">escala_prioridad</t>
+        </is>
+      </c>
+      <c r="Q69" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">media</t>
+        </is>
+      </c>
+      <c r="R69" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Media</t>
+        </is>
+      </c>
+      <c r="S69" s="13">
+        <v>2</v>
+      </c>
+      <c r="V69" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W69" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+      <c r="X69" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Representación. Autoridad: M05 (resultado). LISTAS no define la lógica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="P70" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">escala_prioridad</t>
+        </is>
+      </c>
+      <c r="Q70" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">alta</t>
+        </is>
+      </c>
+      <c r="R70" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alta</t>
+        </is>
+      </c>
+      <c r="S70" s="13">
+        <v>3</v>
+      </c>
+      <c r="V70" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W70" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+      <c r="X70" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Representación. Autoridad: M05 (resultado). LISTAS no define la lógica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="P71" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">escala_prioridad</t>
+        </is>
+      </c>
+      <c r="Q71" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">critica</t>
+        </is>
+      </c>
+      <c r="R71" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Crítica</t>
+        </is>
+      </c>
+      <c r="S71" s="13">
+        <v>4</v>
+      </c>
+      <c r="V71" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vigente</t>
+        </is>
+      </c>
+      <c r="W71" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-004</t>
+        </is>
+      </c>
+      <c r="X71" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Representación. Autoridad: M05 (resultado). LISTAS no define la lógica.</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B2:B8">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="V2:V5000">
+      <formula1>"vigente,reemplazado,descartado"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -7087,8 +9641,10 @@
       <c r="G32" s="9" t="s">
         <v>282</v>
       </c>
-      <c r="H32" s="9" t="s">
-        <v>379</v>
+      <c r="H32" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LISTAS:confirmacion_cavidad_interna</t>
+        </is>
       </c>
       <c r="I32" s="9" t="s">
         <v>335</v>
@@ -7521,8 +10077,10 @@
       <c r="G44" s="10" t="s">
         <v>282</v>
       </c>
-      <c r="H44" s="10" t="s">
-        <v>379</v>
+      <c r="H44" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LISTAS:confirmacion_cavidad_interna</t>
+        </is>
       </c>
       <c r="I44" s="10" t="s">
         <v>335</v>
@@ -10684,8 +13242,10 @@
       <c r="G133" s="9" t="s">
         <v>282</v>
       </c>
-      <c r="H133" s="10" t="s">
-        <v>664</v>
+      <c r="H133" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LISTAS:escala_zona_objetivo</t>
+        </is>
       </c>
       <c r="I133" s="10" t="s">
         <v>334</v>
@@ -10718,8 +13278,10 @@
       <c r="G134" s="10" t="s">
         <v>282</v>
       </c>
-      <c r="H134" s="10" t="s">
-        <v>666</v>
+      <c r="H134" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LISTAS:escala_tasa_ocupacion</t>
+        </is>
       </c>
       <c r="I134" s="10" t="s">
         <v>334</v>
@@ -10752,8 +13314,10 @@
       <c r="G135" s="37" t="s">
         <v>282</v>
       </c>
-      <c r="H135" s="37" t="s">
-        <v>310</v>
+      <c r="H135" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LISTAS:escala_probabilidad_impacto</t>
+        </is>
       </c>
       <c r="I135" s="37" t="s">
         <v>334</v>
@@ -10762,8 +13326,10 @@
         <v>682</v>
       </c>
       <c r="K135" s="37"/>
-      <c r="L135" s="37" t="s">
-        <v>683</v>
+      <c r="L135" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Resultado automático según M01. Valores permitidos: LISTAS:escala_probabilidad_impacto. No editable manualmente.</t>
+        </is>
       </c>
     </row>
     <row r="136" spans="1:12" s="20" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -10788,8 +13354,10 @@
       <c r="G136" s="19" t="s">
         <v>282</v>
       </c>
-      <c r="H136" s="19" t="s">
-        <v>684</v>
+      <c r="H136" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LISTAS:escala_consecuencia</t>
+        </is>
       </c>
       <c r="I136" s="19" t="s">
         <v>334</v>
@@ -10822,8 +13390,10 @@
       <c r="G137" s="19" t="s">
         <v>282</v>
       </c>
-      <c r="H137" s="19" t="s">
-        <v>684</v>
+      <c r="H137" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LISTAS:escala_consecuencia</t>
+        </is>
       </c>
       <c r="I137" s="19" t="s">
         <v>334</v>
@@ -10856,8 +13426,10 @@
       <c r="G138" s="19" t="s">
         <v>282</v>
       </c>
-      <c r="H138" s="19" t="s">
-        <v>684</v>
+      <c r="H138" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LISTAS:escala_consecuencia</t>
+        </is>
       </c>
       <c r="I138" s="19" t="s">
         <v>334</v>
@@ -10890,8 +13462,10 @@
       <c r="G139" s="41" t="s">
         <v>282</v>
       </c>
-      <c r="H139" s="41" t="s">
-        <v>309</v>
+      <c r="H139" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LISTAS:escala_probabilidad_falla</t>
+        </is>
       </c>
       <c r="I139" s="41" t="s">
         <v>334</v>
@@ -10900,8 +13474,10 @@
         <v>708</v>
       </c>
       <c r="K139" s="41"/>
-      <c r="L139" s="41" t="s">
-        <v>709</v>
+      <c r="L139" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Resultado automático no editable. Puntaje total válido 0–9. Resultado permitido: LISTAS:escala_probabilidad_falla.</t>
+        </is>
       </c>
     </row>
     <row r="140" spans="1:12" s="42" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -10926,8 +13502,10 @@
       <c r="G140" s="41" t="s">
         <v>282</v>
       </c>
-      <c r="H140" s="41" t="s">
-        <v>309</v>
+      <c r="H140" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LISTAS:escala_probabilidad_falla</t>
+        </is>
       </c>
       <c r="I140" s="41" t="s">
         <v>334</v>
@@ -10936,8 +13514,10 @@
         <v>719</v>
       </c>
       <c r="K140" s="41"/>
-      <c r="L140" s="41" t="s">
-        <v>709</v>
+      <c r="L140" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Resultado automático no editable. Puntaje total válido 0–9. Resultado permitido: LISTAS:escala_probabilidad_falla.</t>
+        </is>
       </c>
     </row>
     <row r="141" spans="1:12" s="42" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -10962,8 +13542,10 @@
       <c r="G141" s="41" t="s">
         <v>282</v>
       </c>
-      <c r="H141" s="41" t="s">
-        <v>309</v>
+      <c r="H141" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LISTAS:escala_probabilidad_falla</t>
+        </is>
       </c>
       <c r="I141" s="41" t="s">
         <v>334</v>
@@ -10972,8 +13554,10 @@
         <v>728</v>
       </c>
       <c r="K141" s="41"/>
-      <c r="L141" s="41" t="s">
-        <v>709</v>
+      <c r="L141" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Resultado automático no editable. Puntaje total válido 0–9. Resultado permitido: LISTAS:escala_probabilidad_falla.</t>
+        </is>
       </c>
     </row>
     <row r="142" spans="1:12" s="38" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -10998,8 +13582,10 @@
       <c r="G142" s="37" t="s">
         <v>282</v>
       </c>
-      <c r="H142" s="37" t="s">
-        <v>312</v>
+      <c r="H142" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LISTAS:escala_nivel_riesgo</t>
+        </is>
       </c>
       <c r="I142" s="41" t="s">
         <v>334</v>
@@ -11008,8 +13594,10 @@
         <v>746</v>
       </c>
       <c r="K142" s="37"/>
-      <c r="L142" s="37" t="s">
-        <v>752</v>
+      <c r="L142" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Valor calculado automáticamente y no editable. Valores permitidos: LISTAS:escala_nivel_riesgo. Requiere valores válidos en probabilidad_falla_raices_cuello, probabilidad_impacto y consecuencia_raices_cuello</t>
+        </is>
       </c>
     </row>
     <row r="143" spans="1:12" s="38" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -11034,8 +13622,10 @@
       <c r="G143" s="37" t="s">
         <v>282</v>
       </c>
-      <c r="H143" s="37" t="s">
-        <v>312</v>
+      <c r="H143" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LISTAS:escala_nivel_riesgo</t>
+        </is>
       </c>
       <c r="I143" s="41" t="s">
         <v>334</v>
@@ -11044,8 +13634,10 @@
         <v>747</v>
       </c>
       <c r="K143" s="37"/>
-      <c r="L143" s="37" t="s">
-        <v>753</v>
+      <c r="L143" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Valor calculado automáticamente y no editable. Valores permitidos: LISTAS:escala_nivel_riesgo. Requiere valores válidos en probabilidad_falla_tronco, probabilidad_impacto y consecuencia_tronco</t>
+        </is>
       </c>
     </row>
     <row r="144" spans="1:12" s="38" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -11070,8 +13662,10 @@
       <c r="G144" s="37" t="s">
         <v>282</v>
       </c>
-      <c r="H144" s="37" t="s">
-        <v>312</v>
+      <c r="H144" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LISTAS:escala_nivel_riesgo</t>
+        </is>
       </c>
       <c r="I144" s="41" t="s">
         <v>334</v>
@@ -11080,8 +13674,10 @@
         <v>748</v>
       </c>
       <c r="K144" s="37"/>
-      <c r="L144" s="37" t="s">
-        <v>754</v>
+      <c r="L144" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Valor calculado automáticamente y no editable. Valores permitidos: LISTAS:escala_nivel_riesgo. Requiere valores válidos en probabilidad_falla_copa_ramas, probabilidad_impacto y consecuencia_copa_ramas</t>
+        </is>
       </c>
     </row>
     <row r="145" spans="1:12" s="20" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -11138,8 +13734,10 @@
       <c r="G146" s="37" t="s">
         <v>282</v>
       </c>
-      <c r="H146" s="37" t="s">
-        <v>771</v>
+      <c r="H146" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LISTAS:escala_clasificacion_infraestructura</t>
+        </is>
       </c>
       <c r="I146" s="41" t="s">
         <v>334</v>
@@ -11148,8 +13746,10 @@
         <v>770</v>
       </c>
       <c r="K146" s="37"/>
-      <c r="L146" s="37" t="s">
-        <v>773</v>
+      <c r="L146" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Valor calculado automáticamente y no editable. Valores permitidos: LISTAS:escala_clasificacion_infraestructura.</t>
+        </is>
       </c>
     </row>
     <row r="147" spans="1:12" s="38" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -11174,8 +13774,10 @@
       <c r="G147" s="37" t="s">
         <v>282</v>
       </c>
-      <c r="H147" s="37" t="s">
-        <v>312</v>
+      <c r="H147" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LISTAS:escala_nivel_riesgo</t>
+        </is>
       </c>
       <c r="I147" s="41" t="s">
         <v>334</v>
@@ -11184,8 +13786,10 @@
         <v>781</v>
       </c>
       <c r="K147" s="37"/>
-      <c r="L147" s="37" t="s">
-        <v>782</v>
+      <c r="L147" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Valor calculado automáticamente y no editable. Valores permitidos: LISTAS:escala_nivel_riesgo. Requiere clasificaciones válidas de los componentes evaluados.</t>
+        </is>
       </c>
     </row>
     <row r="148" spans="1:12" s="23" customFormat="1" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -11210,8 +13814,10 @@
       <c r="G148" s="22" t="s">
         <v>282</v>
       </c>
-      <c r="H148" s="22" t="s">
-        <v>791</v>
+      <c r="H148" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LISTAS:escala_prioridad</t>
+        </is>
       </c>
       <c r="I148" s="41" t="s">
         <v>334</v>
@@ -11220,8 +13826,10 @@
         <v>792</v>
       </c>
       <c r="K148" s="22"/>
-      <c r="L148" s="22" t="s">
-        <v>793</v>
+      <c r="L148" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Valor calculado automáticamente y no editable. Valores permitidos: LISTAS:escala_prioridad. Requiere valores válidos en clasificacion_riesgo y clasificacion_infraestructura.</t>
+        </is>
       </c>
     </row>
     <row r="149" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -11246,8 +13854,10 @@
       <c r="G149" s="8" t="s">
         <v>870</v>
       </c>
-      <c r="H149" s="8" t="s">
-        <v>871</v>
+      <c r="H149" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LISTAS:accion (filtrado por tipo_ot)</t>
+        </is>
       </c>
       <c r="I149" s="8" t="s">
         <v>334</v>
@@ -11281,8 +13891,10 @@
       <c r="G150" s="8" t="s">
         <v>870</v>
       </c>
-      <c r="H150" s="8" t="s">
-        <v>876</v>
+      <c r="H150" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LISTAS:subtipo_accion (filtrado por accion; vacío si la acción no tiene subtipos)</t>
+        </is>
       </c>
       <c r="I150" s="8" t="s">
         <v>335</v>

</xml_diff>

<commit_message>
[CC-020] Corrección previa al merge: fustes sin altura fija y huso sin 19S
- configuracion_fustes: definición neutral respecto de la altura;
  validación PENDIENTE sin categorías candidatas.
- numero_fustes y dap_fustes_cm: sin 1,30 m como criterio; criterio/altura
  de referencia PENDIENTE.
- huso: zona UTM asociada a la coordenada registrada, sin zona fija;
  obligatoriedad UTM, datum, huso y coordenada original PENDIENTES.
- registro-cambios: SHA-256 del Excel e historial de CC-020.

Sin fórmula de DAP equivalente. §14.12 sin cambios. Sin cambios de software.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/excel/Base de Datos Valpo Verde.xlsx
+++ b/docs/excel/Base de Datos Valpo Verde.xlsx
@@ -9062,11 +9062,15 @@
       <c r="D11" s="19" t="s">
         <v>251</v>
       </c>
-      <c r="E11" s="18" t="s">
-        <v>16</v>
-      </c>
-      <c r="F11" s="19" t="s">
-        <v>317</v>
+      <c r="E11" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Según el CRS de captura configurado para el proyecto; mecanismo pendiente (ADR-010 v2.0).</t>
+        </is>
+      </c>
+      <c r="F11" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Zona UTM y hemisferio asociados a la coordenada UTM registrada. No se asume una zona única para la plataforma.</t>
+        </is>
       </c>
       <c r="G11" s="19" t="s">
         <v>266</v>
@@ -9083,7 +9087,7 @@
       <c r="K11" s="19"/>
       <c r="L11" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Este, Norte, huso, hemisferio y datum deben ser coherentes. No fijar SRID sin verificar configuración del proyecto. PENDIENTE (CC-020): huso y datum siguen abiertos (ADR-010 v2.0); el valor fijo 19S no se aplica como regla, porque la plataforma no asume una única zona UTM. Obligatoriedad anterior: Obligatorio.</t>
+          <t xml:space="preserve">Este, Norte, huso, hemisferio y datum deben ser coherentes. No fijar SRID sin verificar configuración del proyecto. PENDIENTE (CC-020 / ADR-010 v2.0): obligatoriedad de la captura UTM, datum, huso y conservación de la coordenada original de levantamiento por definir. Obligatoriedad anterior: Obligatorio. La ubicación canónica obligatoria del árbol es ubicacion_wgs84.</t>
         </is>
       </c>
       <c r="N11" s="19" t="inlineStr">
@@ -9491,7 +9495,7 @@
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Configuración de los fustes del ejemplar a 1,30 m sobre el terreno. Se registra en cada medición porque condiciona la medición del DAP en esa fecha.</t>
+          <t xml:space="preserve">Configuración de los fustes del ejemplar. Se registra en cada medición porque condiciona la medición del DAP en esa fecha.</t>
         </is>
       </c>
       <c r="G19" s="10" t="s">
@@ -9509,7 +9513,7 @@
       <c r="K19" s="9"/>
       <c r="L19" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obligatorio en la medición inicial (CC-020). PENDIENTE (CC-020): categorías en estudio (monofuste, bifurcado, multifuste) y su relación con numero_fustes y con el cálculo del DAP; no implementar un dominio cerrado hasta su aprobación. Obligatoriedad en mediciones posteriores: pendiente.</t>
+          <t xml:space="preserve">Obligatorio en la medición inicial (CC-020). PENDIENTE (CC-020): categorías definitivas, criterio/altura de referencia y relación con numero_fustes y cálculo del DAP por definir. No implementar un dominio cerrado hasta su aprobación. Obligatoriedad en mediciones posteriores: pendiente.</t>
         </is>
       </c>
       <c r="N19" s="9" t="inlineStr">
@@ -9536,8 +9540,10 @@
       <c r="E20" s="13" t="s">
         <v>313</v>
       </c>
-      <c r="F20" s="9" t="s">
-        <v>329</v>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Número de fustes del ejemplar considerados en la medición.</t>
+        </is>
       </c>
       <c r="G20" s="10" t="s">
         <v>330</v>
@@ -9556,7 +9562,7 @@
       </c>
       <c r="L20" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Válido cuando se registra un número entero ≥ 2. PENDIENTE (CC-020): relación con las categorías de configuración de fustes por definir.</t>
+          <t xml:space="preserve">Válido cuando se registra un número entero ≥ 2. PENDIENTE (CC-020): criterio/altura de referencia para determinar el número de fustes aplicables. Relación con las categorías de configuración de fustes por definir.</t>
         </is>
       </c>
       <c r="N20" s="10" t="inlineStr">
@@ -9585,7 +9591,7 @@
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Diámetros individuales a 1,30 m de cada fuste medido. Son los datos primarios de un ejemplar con más de un fuste y se conservan aunque el DAP equivalente no esté calculado.</t>
+          <t xml:space="preserve">Diámetros individuales de los fustes considerados en la medición. Son los datos primarios de un ejemplar con más de un fuste y se conservan aunque el DAP equivalente no esté calculado.</t>
         </is>
       </c>
       <c r="G21" s="10" t="s">
@@ -9605,7 +9611,7 @@
       </c>
       <c r="L21" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obligatorio en la medición inicial cuando el ejemplar tiene más de un fuste (CC-020). La cantidad de diámetros registrados debe coincidir con numero_fustes; cada valor debe ser &gt; 0.</t>
+          <t xml:space="preserve">Obligatorio en la medición inicial cuando el ejemplar tiene más de un fuste (CC-020). La cantidad de diámetros registrados debe coincidir con numero_fustes; cada valor debe ser &gt; 0. PENDIENTE (CC-020): criterio/altura de referencia que determina los fustes aplicables.</t>
         </is>
       </c>
       <c r="N21" s="10" t="inlineStr">

</xml_diff>

<commit_message>
[CC-029] docs: M05 con prioridad No determinado cuando el riesgo es No determinado
Si clasificacion_riesgo = No determinado, clasificacion_prioridad = No
determinado (mismo criterio que CC-024). Actualiza el Excel maestro
(DICCIONARIO_CAMPOS H172, J172, L172; MATRICES_CALCULO AW5; VERSION E4),
registra la ficha CC-029 y actualiza HANDOFF (próximo libre: CC-030).
Sin cambios de código, migraciones, RLS ni Supabase.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/excel/Base de Datos Valpo Verde.xlsx
+++ b/docs/excel/Base de Datos Valpo Verde.xlsx
@@ -6561,8 +6561,10 @@
       <c r="AV5" t="s">
         <v>937</v>
       </c>
-      <c r="AW5" t="s">
-        <v>940</v>
+      <c r="AW5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cruzar clasificacion_riesgo × clasificacion_infraestructura y devolver la categoría correspondiente de M05. Si clasificacion_infraestructura = No aplica, usar la columna Bajo. Todo riesgo Extremo entrega prioridad Crítica. Si clasificacion_riesgo = No determinado, clasificacion_prioridad = No determinado.</t>
+        </is>
       </c>
     </row>
     <row r="6" spans="1:52" x14ac:dyDescent="0.3">
@@ -11537,7 +11539,7 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">CC-024, CC-026, CC-027, CC-028</t>
+          <t xml:space="preserve">CC-024, CC-026, CC-027, CC-028, CC-029</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
@@ -19686,19 +19688,23 @@
       <c r="G172" s="15" t="s">
         <v>357</v>
       </c>
-      <c r="H172" s="15" t="s">
-        <v>709</v>
+      <c r="H172" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Baja / Media / Alta / Crítica / No determinado</t>
+        </is>
       </c>
       <c r="I172" s="25" t="s">
         <v>324</v>
       </c>
-      <c r="J172" s="15" t="s">
-        <v>710</v>
+      <c r="J172" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M05: cruzar clasificacion_riesgo (Bajo/Moderado/Alto/Extremo) × clasificacion_infraestructura (Bajo/Moderado/Alto/Crítico). Si clasificacion_infraestructura = No aplica, usar la columna Bajo. Todo riesgo Extremo → Crítica. Si clasificacion_riesgo = No determinado, clasificacion_prioridad = No determinado. Orientación: Baja = seguimiento rutinario; Media = intervención programada; Alta = intervención prioritaria en el corto plazo; Crítica = atención urgente.</t>
+        </is>
       </c>
       <c r="K172" s="15"/>
       <c r="L172" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Valor calculado automáticamente. El Inspector puede ajustarlo registrando justificacion_ajuste_clasificacion; la plataforma conserva el valor calculado, el valor ajustado, el Inspector y la fecha del ajuste. Valores permitidos: Baja / Media / Alta / Crítica. Requiere valores válidos en clasificacion_riesgo y clasificacion_infraestructura. Si se ajusta clasificacion_riesgo o clasificacion_infraestructura, calcular con el valor ajustado.</t>
+          <t xml:space="preserve">Valor calculado automáticamente. El Inspector puede ajustarlo registrando justificacion_ajuste_clasificacion; la plataforma conserva el valor calculado, el valor ajustado, el Inspector y la fecha del ajuste. Valores permitidos: Baja / Media / Alta / Crítica / No determinado. Requiere valores válidos en clasificacion_riesgo y clasificacion_infraestructura. Si se ajusta clasificacion_riesgo o clasificacion_infraestructura, calcular con el valor ajustado.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[CC-039] docs: catálogo botánico en CATALOGO_ESPECIES y edad estimada del árbol
- origen_biogeografico pasa de ARBOLES a CATALOGO_ESPECIES (una vez por
  especie, categorías excluyentes); se recupera por especie_cientifica.
- Nuevos persistencia_follaje (Perennifolia / Caducifolia / Semicaducifolia)
  y tipo_hoja (Latifoliada / Acicular / Escuamiforme / Palmera) en el catálogo.
- Nuevo rango_edad_estimada_anios en ARBOLES (tramos de 5 años).
- Excel maestro: DICCIONARIO_CAMPOS, cabeceras, INDICES D9/D10/F9/F10,
  REGLAS_GENERALES B16/C16 y VERSION E4. Ficha CC-039, AM-11 y HANDOFF.
Sin cambios de código, migraciones, RLS ni Supabase.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/excel/Base de Datos Valpo Verde.xlsx
+++ b/docs/excel/Base de Datos Valpo Verde.xlsx
@@ -5261,62 +5261,62 @@
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t xml:space="preserve">origen_biogeografico</t>
+          <t xml:space="preserve">multifustal</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t xml:space="preserve">multifustal</t>
+          <t xml:space="preserve">numero_fustes</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t xml:space="preserve">numero_fustes</t>
+          <t xml:space="preserve">dap_fustes_cm</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t xml:space="preserve">dap_fustes_cm</t>
+          <t xml:space="preserve">dap_cm</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t xml:space="preserve">dap_cm</t>
+          <t xml:space="preserve">altura_total_m</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t xml:space="preserve">altura_total_m</t>
+          <t xml:space="preserve">diametro_copa_ns_m</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
         <is>
-          <t xml:space="preserve">diametro_copa_ns_m</t>
+          <t xml:space="preserve">diametro_copa_eo_m</t>
         </is>
       </c>
       <c r="U1" t="inlineStr">
         <is>
-          <t xml:space="preserve">diametro_copa_eo_m</t>
+          <t xml:space="preserve">diametro_copa_m</t>
         </is>
       </c>
       <c r="V1" t="inlineStr">
         <is>
-          <t xml:space="preserve">diametro_copa_m</t>
+          <t xml:space="preserve">altura_primera_rama_m</t>
         </is>
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t xml:space="preserve">altura_primera_rama_m</t>
+          <t xml:space="preserve">altura_base_copa_viva_m</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t xml:space="preserve">altura_base_copa_viva_m</t>
+          <t xml:space="preserve">clase_edad</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
         <is>
-          <t xml:space="preserve">clase_edad</t>
+          <t xml:space="preserve">rango_edad_estimada_anios</t>
         </is>
       </c>
       <c r="Z1" t="inlineStr">
@@ -5327,7 +5327,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Y2:Y1048576" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="X2:X1048576" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Joven,Semimaduro,Tempranamente maduro,Maduro,Sobremaduro"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5584,14 +5584,16 @@
       </c>
       <c r="D9" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">ARBOLES.id_arbol; ARBOLES.id_proyecto; ARBOLES.id_sector; ARBOLES.sector; ARBOLES.origen_biogeografico; estado_presencia derivado.</t>
+          <t xml:space="preserve">ARBOLES.id_arbol; ARBOLES.id_proyecto; ARBOLES.id_sector; ARBOLES.sector; ARBOLES.especie_cientifica; CATALOGO_ESPECIES.origen_biogeografico (vinculado mediante especie_cientifica); estado_presencia derivado.</t>
         </is>
       </c>
       <c r="E9" s="30" t="s">
         <v>1253</v>
       </c>
-      <c r="F9" s="30" t="s">
-        <v>1255</v>
+      <c r="F9" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PN = (N_nativos / N_presentes) × 100. N_nativos = número de árboles presentes cuya especie tiene CATALOGO_ESPECIES.origen_biogeografico = Nativa o Endémica; N_presentes = Número total de Árboles presentes en el ámbito seleccionado. Contar individuos únicos. Fuente: inventario de SIVU.</t>
+        </is>
       </c>
       <c r="G9" s="30" t="s">
         <v>1254</v>
@@ -5616,14 +5618,16 @@
       </c>
       <c r="D10" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">ARBOLES.id_arbol; ARBOLES.id_proyecto; ARBOLES.id_sector; ARBOLES.sector; ARBOLES.origen_biogeografico; estado_presencia derivado.</t>
+          <t xml:space="preserve">ARBOLES.id_arbol; ARBOLES.id_proyecto; ARBOLES.id_sector; ARBOLES.sector; ARBOLES.especie_cientifica; CATALOGO_ESPECIES.origen_biogeografico (vinculado mediante especie_cientifica); estado_presencia derivado.</t>
         </is>
       </c>
       <c r="E10" s="30" t="s">
         <v>1253</v>
       </c>
-      <c r="F10" s="30" t="s">
-        <v>1260</v>
+      <c r="F10" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PI = (N_introducidos / N_presentes) × 100. N_introducidos = número de árboles presentes cuya especie tiene CATALOGO_ESPECIES.origen_biogeografico = Introducida; N_presentes = Número total de Árboles presentes en el ámbito seleccionado. Contar individuos únicos, independientemente de sus fustes o inspecciones. Fuente: inventario de SIVU.</t>
+        </is>
       </c>
       <c r="G10" s="30" t="s">
         <v>1254</v>
@@ -6243,18 +6247,39 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0724DCB-01ED-4E1E-B9D5-08D0DCF7F3F6}">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:3" ht="15" x14ac:dyDescent="0.35">
-      <c r="A1" s="61" t="s">
-        <v>10</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1208</v>
-      </c>
-      <c r="C1" s="61" t="s">
-        <v>1209</v>
+    <row r="1" spans="1:6" ht="15" x14ac:dyDescent="0.35">
+      <c r="A1" s="61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">especie_cientifica</t>
+        </is>
+      </c>
+      <c r="B1" s="61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">genero</t>
+        </is>
+      </c>
+      <c r="C1" s="61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">familia</t>
+        </is>
+      </c>
+      <c r="D1" s="61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">origen_biogeografico</t>
+        </is>
+      </c>
+      <c r="E1" s="61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">persistencia_follaje</t>
+        </is>
+      </c>
+      <c r="F1" s="61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tipo_hoja</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -7457,12 +7482,12 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">El Usuario municipal solo ingresa en el alta el nombre común o científico, la ubicación y, opcionalmente, el origen biogeográfico. Crea las OT y define requiere_revision_inspector en las OT de Mantenimiento.</t>
+          <t xml:space="preserve">El Usuario municipal solo ingresa en el alta el nombre común o científico y la ubicación. Crea las OT y define requiere_revision_inspector en las OT de Mantenimiento.</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">especie_cientifica; nombre_comun; origen_biogeografico; sector; ubicacion_descriptiva; utm_este; utm_norte; requiere_revision_inspector</t>
+          <t xml:space="preserve">especie_cientifica; nombre_comun; sector; ubicacion_descriptiva; utm_este; utm_norte; requiere_revision_inspector</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
@@ -11539,7 +11564,7 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">CC-024, CC-026, CC-027, CC-028, CC-029</t>
+          <t xml:space="preserve">CC-024, CC-026, CC-027, CC-028, CC-029, CC-039</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
@@ -13028,7 +13053,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M260"/>
+  <dimension ref="A1:M263"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="24" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7" style="41" customWidth="1"/>
@@ -13561,44 +13586,40 @@
         <v>1420</v>
       </c>
     </row>
-    <row r="15" spans="1:12" s="46" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="44" t="s">
+    <row r="15" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="10" t="s">
         <v>317</v>
       </c>
-      <c r="B15" s="48" t="s">
-        <v>12</v>
-      </c>
-      <c r="C15" s="45" t="s">
+      <c r="B15" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" s="7" t="s">
         <v>276</v>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Inspector / Usuario municipal</t>
-        </is>
-      </c>
-      <c r="E15" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Asignación por el Inspector según la distribución natural de la especie identificada.</t>
-        </is>
-      </c>
-      <c r="F15" s="45" t="s">
-        <v>1068</v>
+          <t xml:space="preserve">Inspector</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="s">
+        <v>342</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>356</v>
       </c>
       <c r="G15" s="8" t="s">
         <v>357</v>
       </c>
-      <c r="H15" s="45" t="s">
-        <v>355</v>
-      </c>
-      <c r="I15" s="45" t="s">
+      <c r="H15" s="7" t="s">
+        <v>358</v>
+      </c>
+      <c r="I15" s="7" t="s">
         <v>324</v>
       </c>
-      <c r="J15" s="45"/>
-      <c r="K15" s="45"/>
-      <c r="L15" s="45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Debe ser coherente con especie_cientifica. La clasificación debe considerar la distribución natural de la especie respecto de Chile, no el lugar de plantación ni el origen del ejemplar. En el alta municipal es opcional; el Inspector lo confirma o corrige mediante OT.</t>
-        </is>
+      <c r="J15" s="7"/>
+      <c r="K15" s="7"/>
+      <c r="L15" s="7" t="s">
+        <v>359</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -13606,7 +13627,7 @@
         <v>317</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C16" s="7" t="s">
         <v>276</v>
@@ -13620,21 +13641,23 @@
         <v>342</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>324</v>
+        <v>363</v>
       </c>
       <c r="J16" s="7"/>
-      <c r="K16" s="7"/>
-      <c r="L16" s="7" t="s">
-        <v>359</v>
+      <c r="K16" s="7" t="s">
+        <v>364</v>
+      </c>
+      <c r="L16" s="8" t="s">
+        <v>365</v>
       </c>
     </row>
     <row r="17" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -13642,7 +13665,7 @@
         <v>317</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C17" s="7" t="s">
         <v>276</v>
@@ -13656,13 +13679,13 @@
         <v>342</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>360</v>
+        <v>366</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>362</v>
+        <v>368</v>
       </c>
       <c r="I17" s="7" t="s">
         <v>363</v>
@@ -13672,107 +13695,105 @@
         <v>364</v>
       </c>
       <c r="L17" s="8" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="10" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" s="35" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="17" t="s">
         <v>317</v>
       </c>
-      <c r="B18" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="C18" s="7" t="s">
+      <c r="B18" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="18" t="s">
+        <v>370</v>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sistema / Inspector</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="s">
+        <v>345</v>
+      </c>
+      <c r="F18" s="18" t="s">
+        <v>371</v>
+      </c>
+      <c r="G18" s="18" t="s">
+        <v>347</v>
+      </c>
+      <c r="H18" s="18" t="s">
+        <v>368</v>
+      </c>
+      <c r="I18" s="18" t="s">
+        <v>324</v>
+      </c>
+      <c r="J18" s="18" t="s">
+        <v>372</v>
+      </c>
+      <c r="K18" s="18"/>
+      <c r="L18" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Valor numérico &gt; 0. No admite texto. Si no puede medirse, mantener la evaluación preguardada; no registrar 0. Si multifustal = No, el valor debe ser ingresado manualmente; si multifustal = Sí, debe ser calculado automáticamente por la plataforma.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="10" t="s">
+        <v>317</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>1386</v>
+      </c>
+      <c r="C19" s="7" t="s">
         <v>276</v>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Inspector</t>
         </is>
       </c>
-      <c r="E18" s="11" t="s">
-        <v>342</v>
-      </c>
-      <c r="F18" s="7" t="s">
-        <v>366</v>
-      </c>
-      <c r="G18" s="8" t="s">
-        <v>367</v>
-      </c>
-      <c r="H18" s="7" t="s">
-        <v>368</v>
-      </c>
-      <c r="I18" s="7" t="s">
-        <v>363</v>
-      </c>
-      <c r="J18" s="7"/>
-      <c r="K18" s="7" t="s">
-        <v>364</v>
-      </c>
-      <c r="L18" s="8" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12" s="35" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="17" t="s">
-        <v>317</v>
-      </c>
-      <c r="B19" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="C19" s="18" t="s">
-        <v>370</v>
-      </c>
-      <c r="D19" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sistema / Inspector</t>
-        </is>
-      </c>
-      <c r="E19" s="17" t="s">
+      <c r="E19" s="10" t="s">
         <v>345</v>
       </c>
-      <c r="F19" s="18" t="s">
-        <v>371</v>
-      </c>
-      <c r="G19" s="18" t="s">
+      <c r="F19" s="7" t="s">
+        <v>374</v>
+      </c>
+      <c r="G19" s="7" t="s">
         <v>347</v>
       </c>
-      <c r="H19" s="18" t="s">
-        <v>368</v>
-      </c>
-      <c r="I19" s="18" t="s">
+      <c r="H19" s="7" t="s">
+        <v>348</v>
+      </c>
+      <c r="I19" s="7" t="s">
         <v>324</v>
       </c>
-      <c r="J19" s="18" t="s">
-        <v>372</v>
-      </c>
-      <c r="K19" s="18"/>
-      <c r="L19" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Valor numérico &gt; 0. No admite texto. Si no puede medirse, mantener la evaluación preguardada; no registrar 0. Si multifustal = No, el valor debe ser ingresado manualmente; si multifustal = Sí, debe ser calculado automáticamente por la plataforma.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J19" s="7"/>
+      <c r="K19" s="7"/>
+      <c r="L19" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Valor numérico &gt; 0. No admite texto. Si no puede medirse, mantener la evaluación preguardada; no registrar 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" spans="1:12" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="10" t="s">
         <v>317</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>1386</v>
+        <v>1388</v>
       </c>
       <c r="C20" s="7" t="s">
         <v>276</v>
       </c>
-      <c r="D20" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Inspector</t>
-        </is>
+      <c r="D20" s="7" t="s">
+        <v>259</v>
       </c>
       <c r="E20" s="10" t="s">
         <v>345</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>374</v>
+        <v>1421</v>
       </c>
       <c r="G20" s="7" t="s">
         <v>347</v>
@@ -13781,14 +13802,16 @@
         <v>348</v>
       </c>
       <c r="I20" s="7" t="s">
-        <v>324</v>
-      </c>
-      <c r="J20" s="7"/>
-      <c r="K20" s="7"/>
-      <c r="L20" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Valor numérico &gt; 0. No admite texto. Si no puede medirse, mantener la evaluación preguardada; no registrar 0.</t>
-        </is>
+        <v>1422</v>
+      </c>
+      <c r="J20" s="7" t="s">
+        <v>1151</v>
+      </c>
+      <c r="K20" s="7" t="s">
+        <v>1423</v>
+      </c>
+      <c r="L20" s="8" t="s">
+        <v>1424</v>
       </c>
     </row>
     <row r="21" spans="1:12" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -13796,7 +13819,7 @@
         <v>317</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>1388</v>
+        <v>1389</v>
       </c>
       <c r="C21" s="7" t="s">
         <v>276</v>
@@ -13808,7 +13831,7 @@
         <v>345</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>1421</v>
+        <v>1425</v>
       </c>
       <c r="G21" s="7" t="s">
         <v>347</v>
@@ -13834,19 +13857,19 @@
         <v>317</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>1389</v>
+        <v>17</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>276</v>
+        <v>419</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>259</v>
+        <v>319</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>345</v>
+        <v>1426</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>1425</v>
+        <v>1427</v>
       </c>
       <c r="G22" s="7" t="s">
         <v>347</v>
@@ -13855,54 +13878,54 @@
         <v>348</v>
       </c>
       <c r="I22" s="7" t="s">
-        <v>1422</v>
+        <v>363</v>
       </c>
       <c r="J22" s="7" t="s">
+        <v>1428</v>
+      </c>
+      <c r="K22" s="7" t="s">
+        <v>1429</v>
+      </c>
+      <c r="L22" s="8" t="s">
+        <v>1430</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>317</v>
+      </c>
+      <c r="B23" t="s">
+        <v>18</v>
+      </c>
+      <c r="C23" s="65" t="s">
+        <v>276</v>
+      </c>
+      <c r="D23" t="s">
+        <v>259</v>
+      </c>
+      <c r="E23" t="s">
+        <v>345</v>
+      </c>
+      <c r="F23" t="s">
+        <v>1390</v>
+      </c>
+      <c r="G23" t="s">
+        <v>347</v>
+      </c>
+      <c r="H23" t="s">
+        <v>348</v>
+      </c>
+      <c r="I23" t="s">
+        <v>1431</v>
+      </c>
+      <c r="J23" t="s">
         <v>1151</v>
       </c>
-      <c r="K22" s="7" t="s">
-        <v>1423</v>
-      </c>
-      <c r="L22" s="8" t="s">
-        <v>1424</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="10" t="s">
-        <v>317</v>
-      </c>
-      <c r="B23" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="C23" s="7" t="s">
-        <v>419</v>
-      </c>
-      <c r="D23" s="7" t="s">
-        <v>319</v>
-      </c>
-      <c r="E23" s="10" t="s">
-        <v>1426</v>
-      </c>
-      <c r="F23" s="7" t="s">
-        <v>1427</v>
-      </c>
-      <c r="G23" s="7" t="s">
-        <v>347</v>
-      </c>
-      <c r="H23" s="7" t="s">
-        <v>348</v>
-      </c>
-      <c r="I23" s="7" t="s">
-        <v>363</v>
-      </c>
-      <c r="J23" s="7" t="s">
-        <v>1428</v>
-      </c>
-      <c r="K23" s="7" t="s">
-        <v>1429</v>
-      </c>
-      <c r="L23" s="8" t="s">
-        <v>1430</v>
+      <c r="K23" t="s">
+        <v>1391</v>
+      </c>
+      <c r="L23" t="s">
+        <v>1432</v>
       </c>
     </row>
     <row r="24" spans="1:12" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
@@ -13910,7 +13933,7 @@
         <v>317</v>
       </c>
       <c r="B24" t="s">
-        <v>18</v>
+        <v>1387</v>
       </c>
       <c r="C24" s="65" t="s">
         <v>276</v>
@@ -13922,7 +13945,7 @@
         <v>345</v>
       </c>
       <c r="F24" t="s">
-        <v>1390</v>
+        <v>1392</v>
       </c>
       <c r="G24" t="s">
         <v>347</v>
@@ -13937,84 +13960,108 @@
         <v>1151</v>
       </c>
       <c r="K24" t="s">
-        <v>1391</v>
+        <v>1433</v>
       </c>
       <c r="L24" t="s">
-        <v>1432</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
+        <v>1434</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" s="51" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="49" t="s">
         <v>317</v>
       </c>
-      <c r="B25" t="s">
-        <v>1387</v>
-      </c>
-      <c r="C25" s="65" t="s">
+      <c r="B25" s="49" t="s">
+        <v>19</v>
+      </c>
+      <c r="C25" s="50" t="s">
         <v>276</v>
       </c>
-      <c r="D25" t="s">
-        <v>259</v>
-      </c>
-      <c r="E25" t="s">
-        <v>345</v>
-      </c>
-      <c r="F25" t="s">
-        <v>1392</v>
-      </c>
-      <c r="G25" t="s">
-        <v>347</v>
-      </c>
-      <c r="H25" t="s">
-        <v>348</v>
-      </c>
-      <c r="I25" t="s">
-        <v>1431</v>
-      </c>
-      <c r="J25" t="s">
-        <v>1151</v>
-      </c>
-      <c r="K25" t="s">
-        <v>1433</v>
-      </c>
-      <c r="L25" t="s">
-        <v>1434</v>
+      <c r="D25" s="50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Inspector</t>
+        </is>
+      </c>
+      <c r="E25" s="49" t="s">
+        <v>342</v>
+      </c>
+      <c r="F25" s="50" t="s">
+        <v>376</v>
+      </c>
+      <c r="G25" s="50" t="s">
+        <v>357</v>
+      </c>
+      <c r="H25" s="50" t="s">
+        <v>377</v>
+      </c>
+      <c r="I25" s="50" t="s">
+        <v>324</v>
+      </c>
+      <c r="J25" s="50"/>
+      <c r="K25" s="50"/>
+      <c r="L25" s="50" t="s">
+        <v>378</v>
       </c>
     </row>
     <row r="26" spans="1:12" s="51" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="49" t="s">
-        <v>317</v>
-      </c>
-      <c r="B26" s="49" t="s">
-        <v>19</v>
-      </c>
-      <c r="C26" s="50" t="s">
-        <v>276</v>
+      <c r="A26" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARBOLES</t>
+        </is>
+      </c>
+      <c r="B26" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rango_edad_estimada_anios</t>
+        </is>
+      </c>
+      <c r="C26" s="50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estimado</t>
+        </is>
       </c>
       <c r="D26" s="50" t="inlineStr">
         <is>
           <t xml:space="preserve">Inspector</t>
         </is>
       </c>
-      <c r="E26" s="49" t="s">
-        <v>342</v>
-      </c>
-      <c r="F26" s="50" t="s">
-        <v>376</v>
-      </c>
-      <c r="G26" s="50" t="s">
-        <v>357</v>
-      </c>
-      <c r="H26" s="50" t="s">
-        <v>377</v>
-      </c>
-      <c r="I26" s="50" t="s">
-        <v>324</v>
-      </c>
-      <c r="J26" s="50"/>
-      <c r="K26" s="50"/>
-      <c r="L26" s="50" t="s">
-        <v>378</v>
+      <c r="E26" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estimación a partir de especie_cientifica, dap_cm, altura_total_m, características de crecimiento de la especie, fotografías con regla topográfica y antecedentes disponibles.</t>
+        </is>
+      </c>
+      <c r="F26" s="50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Intervalo de edad cronológica estimada del ejemplar, en años, independiente de su etapa de desarrollo.</t>
+        </is>
+      </c>
+      <c r="G26" s="50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Categoría</t>
+        </is>
+      </c>
+      <c r="H26" s="50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0–5 / 6–10 / 11–15 / 16–20 / 21–25 / 26–30 / 31–35 / 36–40 / 41–45 / 46–50 / 51–55 / 56–60 / 61–65 / 66–70 / 71–75 / 76–80 / 81–85 / 86–90 / 91–95 / 96–100 / Más de 100 años</t>
+        </is>
+      </c>
+      <c r="I26" s="50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Obligatorio (pendiente de validar su factibilidad)</t>
+        </is>
+      </c>
+      <c r="J26" s="50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estimación; no calcular a partir de clase_edad ni únicamente a partir de dap_cm.</t>
+        </is>
+      </c>
+      <c r="K26" s="50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">En la inspección de Evaluación inicial o de Levantamiento del árbol.</t>
+        </is>
+      </c>
+      <c r="L26" s="50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Seleccionar un único intervalo. No establecer equivalencias automáticas entre clase_edad y la edad cronológica. No utilizar únicamente el DAP como determinante de la edad. La estimación corresponde a la fecha_inspeccion en que se registró; conservar el historial por inspección.</t>
+        </is>
       </c>
     </row>
     <row r="27" spans="1:12" s="51" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -22978,74 +23025,74 @@
     <row r="257" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A257" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">PROYECTOS</t>
+          <t xml:space="preserve">CATALOGO_ESPECIES</t>
         </is>
       </c>
       <c r="B257" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">id_proyecto</t>
+          <t xml:space="preserve">origen_biogeografico</t>
         </is>
       </c>
       <c r="C257" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Generado por plataforma</t>
+          <t xml:space="preserve">Manual</t>
         </is>
       </c>
       <c r="D257" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sistema</t>
+          <t xml:space="preserve">Inspector</t>
         </is>
       </c>
       <c r="E257" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Asignación automática al crear el proyecto.</t>
+          <t xml:space="preserve">Asignación según la distribución natural de la especie respecto de Chile, consultando el Catálogo de las plantas vasculares de Chile (Rodríguez et al., 2018) o su versión en línea vigente.</t>
         </is>
       </c>
       <c r="F257" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Identificador único y estable del proyecto, que separa inventarios, delimitación territorial y acceso de usuarios.</t>
+          <t xml:space="preserve">Clasificación de la especie según su procedencia biogeográfica respecto del territorio chileno. Endémica: especie nativa cuya distribución natural está restringida a Chile. Nativa: especie nativa de Chile cuya distribución natural no se restringe al país. Introducida: especie exótica presente en Chile fuera de su distribución natural.</t>
         </is>
       </c>
       <c r="G257" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Identificador (texto)</t>
+          <t xml:space="preserve">Categoría</t>
         </is>
       </c>
       <c r="H257" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">No aplica</t>
+          <t xml:space="preserve">Nativa / Endémica / Introducida</t>
         </is>
       </c>
       <c r="I257" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obligatorio</t>
+          <t xml:space="preserve">Obligatorio para completar la clasificación del catálogo</t>
         </is>
       </c>
       <c r="J257" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Asignación automática única.</t>
+          <t xml:space="preserve">La plataforma lo vincula al árbol mediante especie_cientifica.</t>
         </is>
       </c>
       <c r="K257" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Al crear el proyecto.</t>
+          <t xml:space="preserve">Al completar o actualizar la clasificación de la especie.</t>
         </is>
       </c>
       <c r="L257" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">No editable. Solo el Administrador puede crear proyectos.</t>
+          <t xml:space="preserve">Categorías excluyentes: una especie endémica no se registra como Nativa. Considerar la distribución natural de la especie respecto de Chile, no el lugar de plantación ni el origen del ejemplar. Si aún no se conoce, dejar nulo; no inventarlo ni bloquear el registro del árbol. Se muestra en la ficha del árbol mediante especie_cientifica; no se ingresa por ejemplar ni se duplica en ARBOLES. Si el árbol no tiene especie_cientifica vigente, se informa como Origen no determinado.</t>
         </is>
       </c>
     </row>
     <row r="258" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A258" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">PROYECTOS</t>
+          <t xml:space="preserve">CATALOGO_ESPECIES</t>
         </is>
       </c>
       <c r="B258" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">nombre_proyecto</t>
+          <t xml:space="preserve">persistencia_follaje</t>
         </is>
       </c>
       <c r="C258" s="33" t="inlineStr">
@@ -23055,169 +23102,355 @@
       </c>
       <c r="D258" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Administrador</t>
+          <t xml:space="preserve">Inspector</t>
         </is>
       </c>
       <c r="E258" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ingreso del nombre al crear o editar el proyecto.</t>
+          <t xml:space="preserve">Asignación según fuentes botánicas de referencia al incorporar o completar la especie en el catálogo.</t>
         </is>
       </c>
       <c r="F258" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nombre visible del proyecto.</t>
+          <t xml:space="preserve">Comportamiento habitual del follaje de la especie a lo largo del año. Perennifolia: conserva follaje funcional durante todo el año, con renovación gradual. Caducifolia: pierde la totalidad del follaje durante la estación desfavorable. Semicaducifolia: pierde parcialmente el follaje, o lo pierde por un período breve, según las condiciones climáticas del año.</t>
         </is>
       </c>
       <c r="G258" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Texto</t>
+          <t xml:space="preserve">Categoría</t>
         </is>
       </c>
       <c r="H258" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">No aplica</t>
+          <t xml:space="preserve">Perennifolia / Caducifolia / Semicaducifolia</t>
         </is>
       </c>
       <c r="I258" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obligatorio</t>
+          <t xml:space="preserve">Obligatorio para completar la clasificación del catálogo</t>
         </is>
       </c>
       <c r="J258" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">No aplica.</t>
+          <t xml:space="preserve">La plataforma la vincula al árbol mediante especie_cientifica.</t>
         </is>
       </c>
       <c r="K258" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Al crear o editar el proyecto.</t>
+          <t xml:space="preserve">Al completar o actualizar la clasificación de la especie.</t>
         </is>
       </c>
       <c r="L258" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">No vacío. Su modificación no altera id_proyecto.</t>
+          <t xml:space="preserve">Corresponde al comportamiento habitual de la especie, no a la condición observada en el ejemplar. Si las fuentes describen un comportamiento variable, registrar el habitual en las condiciones climáticas de Valparaíso. Si aún no se conoce, dejar nulo; no inventarla ni bloquear el registro del árbol. No duplicar en ARBOLES. Si el árbol no tiene especie_cientifica vigente, no mostrar valor.</t>
         </is>
       </c>
     </row>
     <row r="259" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A259" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">MIEMBROS_PROYECTO</t>
+          <t xml:space="preserve">CATALOGO_ESPECIES</t>
         </is>
       </c>
       <c r="B259" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">id_proyecto</t>
+          <t xml:space="preserve">tipo_hoja</t>
         </is>
       </c>
       <c r="C259" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vinculado por plataforma</t>
+          <t xml:space="preserve">Manual</t>
         </is>
       </c>
       <c r="D259" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Administrador</t>
+          <t xml:space="preserve">Inspector</t>
         </is>
       </c>
       <c r="E259" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Selección del proyecto al asignar un miembro.</t>
+          <t xml:space="preserve">Asignación según fuentes botánicas de referencia al incorporar o completar la especie en el catálogo.</t>
         </is>
       </c>
       <c r="F259" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proyecto al que se asigna el usuario.</t>
+          <t xml:space="preserve">Morfología predominante de las hojas adultas de la especie. Latifoliada: lámina ancha y plana. Acicular: hoja alargada y angosta, en forma de aguja. Escuamiforme: hoja reducida a escamas adosadas a la ramilla. Palmera: hoja de palmera, palmada o pinnada.</t>
         </is>
       </c>
       <c r="G259" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Identificador (texto)</t>
+          <t xml:space="preserve">Categoría</t>
         </is>
       </c>
       <c r="H259" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">No aplica</t>
+          <t xml:space="preserve">Latifoliada / Acicular / Escuamiforme / Palmera</t>
         </is>
       </c>
       <c r="I259" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obligatorio</t>
+          <t xml:space="preserve">Obligatorio para completar la clasificación del catálogo</t>
         </is>
       </c>
       <c r="J259" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">No aplica.</t>
+          <t xml:space="preserve">La plataforma lo vincula al árbol mediante especie_cientifica.</t>
         </is>
       </c>
       <c r="K259" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Al asignar un usuario a un proyecto.</t>
+          <t xml:space="preserve">Al completar o actualizar la clasificación de la especie.</t>
         </is>
       </c>
       <c r="L259" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Referencia válida a PROYECTOS. Un usuario puede pertenecer a varios proyectos; no repetir la misma combinación id_proyecto e id_usuario.</t>
+          <t xml:space="preserve">Seleccionar una única categoría según el follaje adulto; no considerar el follaje juvenil. Si la morfología no coincide exactamente con una categoría, asignar la más cercana: las estructuras planas que cumplen función foliar, como los filodios, se clasifican como Latifoliada; las hojas reducidas a escamas sobre ramillas verdes se clasifican como Escuamiforme. Si aún no se conoce, dejar nulo; no inventarlo ni bloquear el registro del árbol. No duplicar en ARBOLES. Si el árbol no tiene especie_cientifica vigente, no mostrar valor.</t>
         </is>
       </c>
     </row>
     <row r="260" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A260" s="41" t="inlineStr">
         <is>
+          <t xml:space="preserve">PROYECTOS</t>
+        </is>
+      </c>
+      <c r="B260" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">id_proyecto</t>
+        </is>
+      </c>
+      <c r="C260" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Generado por plataforma</t>
+        </is>
+      </c>
+      <c r="D260" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sistema</t>
+        </is>
+      </c>
+      <c r="E260" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Asignación automática al crear el proyecto.</t>
+        </is>
+      </c>
+      <c r="F260" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Identificador único y estable del proyecto, que separa inventarios, delimitación territorial y acceso de usuarios.</t>
+        </is>
+      </c>
+      <c r="G260" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Identificador (texto)</t>
+        </is>
+      </c>
+      <c r="H260" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No aplica</t>
+        </is>
+      </c>
+      <c r="I260" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Obligatorio</t>
+        </is>
+      </c>
+      <c r="J260" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Asignación automática única.</t>
+        </is>
+      </c>
+      <c r="K260" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Al crear el proyecto.</t>
+        </is>
+      </c>
+      <c r="L260" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No editable. Solo el Administrador puede crear proyectos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="261" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A261" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PROYECTOS</t>
+        </is>
+      </c>
+      <c r="B261" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nombre_proyecto</t>
+        </is>
+      </c>
+      <c r="C261" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="D261" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Administrador</t>
+        </is>
+      </c>
+      <c r="E261" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ingreso del nombre al crear o editar el proyecto.</t>
+        </is>
+      </c>
+      <c r="F261" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nombre visible del proyecto.</t>
+        </is>
+      </c>
+      <c r="G261" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Texto</t>
+        </is>
+      </c>
+      <c r="H261" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No aplica</t>
+        </is>
+      </c>
+      <c r="I261" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Obligatorio</t>
+        </is>
+      </c>
+      <c r="J261" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No aplica.</t>
+        </is>
+      </c>
+      <c r="K261" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Al crear o editar el proyecto.</t>
+        </is>
+      </c>
+      <c r="L261" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No vacío. Su modificación no altera id_proyecto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="262" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A262" s="41" t="inlineStr">
+        <is>
           <t xml:space="preserve">MIEMBROS_PROYECTO</t>
         </is>
       </c>
-      <c r="B260" s="41" t="inlineStr">
+      <c r="B262" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">id_proyecto</t>
+        </is>
+      </c>
+      <c r="C262" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vinculado por plataforma</t>
+        </is>
+      </c>
+      <c r="D262" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Administrador</t>
+        </is>
+      </c>
+      <c r="E262" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Selección del proyecto al asignar un miembro.</t>
+        </is>
+      </c>
+      <c r="F262" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proyecto al que se asigna el usuario.</t>
+        </is>
+      </c>
+      <c r="G262" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Identificador (texto)</t>
+        </is>
+      </c>
+      <c r="H262" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No aplica</t>
+        </is>
+      </c>
+      <c r="I262" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Obligatorio</t>
+        </is>
+      </c>
+      <c r="J262" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No aplica.</t>
+        </is>
+      </c>
+      <c r="K262" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Al asignar un usuario a un proyecto.</t>
+        </is>
+      </c>
+      <c r="L262" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Referencia válida a PROYECTOS. Un usuario puede pertenecer a varios proyectos; no repetir la misma combinación id_proyecto e id_usuario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="263" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A263" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIEMBROS_PROYECTO</t>
+        </is>
+      </c>
+      <c r="B263" s="41" t="inlineStr">
         <is>
           <t xml:space="preserve">id_usuario</t>
         </is>
       </c>
-      <c r="C260" s="33" t="inlineStr">
+      <c r="C263" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">Vinculado por plataforma</t>
         </is>
       </c>
-      <c r="D260" s="33" t="inlineStr">
+      <c r="D263" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">Administrador</t>
         </is>
       </c>
-      <c r="E260" s="41" t="inlineStr">
+      <c r="E263" s="41" t="inlineStr">
         <is>
           <t xml:space="preserve">Selección del usuario al asignarlo al proyecto.</t>
         </is>
       </c>
-      <c r="F260" s="33" t="inlineStr">
+      <c r="F263" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">Usuario con acceso al proyecto.</t>
         </is>
       </c>
-      <c r="G260" s="33" t="inlineStr">
+      <c r="G263" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">Identificador (texto)</t>
         </is>
       </c>
-      <c r="H260" s="33" t="inlineStr">
+      <c r="H263" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">No aplica</t>
         </is>
       </c>
-      <c r="I260" s="33" t="inlineStr">
+      <c r="I263" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">Obligatorio</t>
         </is>
       </c>
-      <c r="J260" s="33" t="inlineStr">
+      <c r="J263" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">No aplica.</t>
         </is>
       </c>
-      <c r="K260" s="33" t="inlineStr">
+      <c r="K263" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">Al asignar un usuario a un proyecto.</t>
         </is>
       </c>
-      <c r="L260" s="33" t="inlineStr">
+      <c r="L263" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">Referencia válida a USUARIOS con activo = Sí. El rol del usuario se mantiene en USUARIOS.Rol.</t>
         </is>

</xml_diff>

<commit_message>
[AM-10] Excel: textos de CC-031, CC-032, CC-036 y CC-037; edad estimada opcional; defoliación estacional
Aplica en el Excel maestro los textos propuestos en las fichas:
- CC-031: estado_registro con Anulado; filas nuevas motivo_anulacion,
  anulado_por y fecha_anulacion (DICCIONARIO_CAMPOS e INSPECCION); regla
  nueva en REGLAS_GENERALES (fila 26).
- CC-032: utm_este y utm_norte (E y L).
- CC-036: nombre_reportante, rut_reportante y resultado_revision.
- CC-037: REGLAS_GENERALES B25 y fecha_proxima_inspeccion /
  fecha_proximo_monitoreo (L).
Además, decisiones de la autora del 2026-10-20: rango_edad_estimada_anios
Opcional (CC-039) y referencia estacional de la defoliación en caducifolias
(AM-11). Agrega la fila 2.0.0 de VERSION con estado "aprobación de
publicación pendiente".

Solo el Excel. Sin cambios de código, migraciones, RLS ni Supabase.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/excel/Base de Datos Valpo Verde.xlsx
+++ b/docs/excel/Base de Datos Valpo Verde.xlsx
@@ -7135,7 +7135,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -7680,7 +7680,7 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">SIVU sugiere, según nivel_riesgo, el rango de la próxima inspección técnica y del próximo monitoreo: Bajo 24 meses y 12 meses; Moderado 12 meses y 3 a 6 meses; Alto 1 a 3 meses y 2 a 4 semanas; Extremo reevaluación dentro de 1 a 4 semanas y monitoreo inmediato y continuo mientras persista el peligro. Al llegar el inicio de cada rango, la fecha se envía al calendario del módulo para agendarla. El Inspector puede ajustarla registrando justificacion_ajuste_fecha.</t>
+          <t xml:space="preserve">SIVU sugiere, según nivel_riesgo, el rango de la próxima inspección técnica y del próximo monitoreo: Bajo 24 meses y 12 meses; Moderado 12 meses y 3 a 6 meses; Alto 1 a 3 meses y 2 a 4 semanas; Extremo reevaluación dentro de 1 a 4 semanas y monitoreo inmediato y continuo mientras persista el peligro. SIVU no agenda automáticamente: al llegar el inicio de cada rango, muestra un recordatorio en la lista de próximas inspecciones y monitoreos del proyecto, con el inicio y el término del rango, desde la cual el Usuario municipal crea y programa la OT. El Inspector puede ajustar la fecha registrando justificacion_ajuste_fecha.</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
@@ -7691,6 +7691,28 @@
       <c r="D25" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">INSPECCION</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Historial y vigencia</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mientras una inspección está Preguardado, el Inspector puede modificar todos sus datos. Una inspección Finalizado no se modifica: si contiene un error, el Inspector la anula registrando motivo_anulacion. La inspección anulada se conserva en el historial y deja de considerarse para la vigencia. Los datos correctos se registran en una nueva inspección: en la misma OT si todavía no está completada; si lo está, en una nueva OT. Solo el Inspector anula inspecciones.</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">estado_registro; motivo_anulacion; anulado_por; fecha_anulacion</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INSPECCION; ARBOLES; REGISTRO_EVALUACION; ORDENES DE TRABAJO</t>
         </is>
       </c>
     </row>
@@ -11435,7 +11457,7 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -11585,6 +11607,38 @@
       <c r="J4" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Contenido del Excel auditado el 2026-10-18 (incluye REGLAS_GENERALES y REGLAS_INDICADORES con 98 reglas). Por CC-028 es la única fuente metodológica del proyecto y reemplaza al Excel anterior; prevalece sobre CC-008, CC-009 y CC-020 en lo que los contradiga (conflictos P1–P9 de CC-026). NO publica la versión 2.0.0 ni define rule_version (C1 pendiente).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2.0.0</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2.0</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">aprobación de publicación pendiente</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-024, CC-026, CC-027, CC-028, CC-029, CC-030, CC-031, CC-032, CC-034, CC-035, CC-036, CC-037, CC-039</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2.0.0 en preparación (fuente única desde CC-028)</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Incluye AM-10: textos de CC-031, CC-032, CC-036 y CC-037; rango_edad_estimada_anios opcional (CC-039) y referencia estacional de la defoliación en caducifolias (AM-11). El Excel maestro es la única fuente (CC-028) y los diagramas no forman parte del paquete (CC-030). INDICES sigue en propuesta (DM-09). Todas las reglas de REGLAS_INDICADORES son vigentes en esta versión (PR-011 v3.0). Al publicar, la autora completa fecha_publicacion, aprobado_por, fecha_aprobacion y tag_git, y cambia el estado a publicada.</t>
         </is>
       </c>
     </row>
@@ -12418,7 +12472,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:S1"/>
+  <dimension ref="A1:V1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.6640625" customWidth="1"/>
@@ -12428,7 +12482,7 @@
     <col min="14" max="14" width="25.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="12" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:22" ht="12" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">id_inspeccion</t>
@@ -12522,6 +12576,21 @@
       <c r="S1" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">estado_registro</t>
+        </is>
+      </c>
+      <c r="T1" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">motivo_anulacion</t>
+        </is>
+      </c>
+      <c r="U1" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">anulado_por</t>
+        </is>
+      </c>
+      <c r="V1" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fecha_anulacion</t>
         </is>
       </c>
     </row>
@@ -13053,7 +13122,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M263"/>
+  <dimension ref="A1:M266"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="24" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7" style="41" customWidth="1"/>
@@ -13381,7 +13450,7 @@
       </c>
       <c r="E9" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ingreso manual de la coordenada del árbol obtenida en terreno.</t>
+          <t xml:space="preserve">Ingreso manual de la coordenada del árbol obtenida en terreno. Como ayuda, al marcar el punto en el mapa del formulario la plataforma rellena utm_este y utm_norte, que siguen siendo editables.</t>
         </is>
       </c>
       <c r="F9" s="7" t="s">
@@ -13398,8 +13467,10 @@
       </c>
       <c r="J9" s="7"/>
       <c r="K9" s="7"/>
-      <c r="L9" s="7" t="s">
-        <v>349</v>
+      <c r="L9" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Coordenada UTM huso 19S, datum WGS84 (EPSG:32719). Este y Norte deben ser coherentes con el huso y el datum fijos. Si proviene del punto marcado en el mapa, la plataforma la convierte a UTM y puede editarse antes de guardar.</t>
+        </is>
       </c>
     </row>
     <row r="10" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -13417,7 +13488,7 @@
       </c>
       <c r="E10" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ingreso manual de la coordenada del árbol obtenida en terreno.</t>
+          <t xml:space="preserve">Ingreso manual de la coordenada del árbol obtenida en terreno. Como ayuda, al marcar el punto en el mapa del formulario la plataforma rellena utm_este y utm_norte, que siguen siendo editables.</t>
         </is>
       </c>
       <c r="F10" s="8" t="s">
@@ -13434,8 +13505,10 @@
       </c>
       <c r="J10" s="8"/>
       <c r="K10" s="8"/>
-      <c r="L10" s="8" t="s">
-        <v>349</v>
+      <c r="L10" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Coordenada UTM huso 19S, datum WGS84 (EPSG:32719). Norte y Este deben ser coherentes con el huso y el datum fijos. Si proviene del punto marcado en el mapa, la plataforma la convierte a UTM y puede editarse antes de guardar.</t>
+        </is>
       </c>
     </row>
     <row r="11" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -14045,7 +14118,7 @@
       </c>
       <c r="I26" s="50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obligatorio (pendiente de validar su factibilidad)</t>
+          <t xml:space="preserve">Opcional</t>
         </is>
       </c>
       <c r="J26" s="50" t="inlineStr">
@@ -14060,7 +14133,7 @@
       </c>
       <c r="L26" s="50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Seleccionar un único intervalo. No establecer equivalencias automáticas entre clase_edad y la edad cronológica. No utilizar únicamente el DAP como determinante de la edad. La estimación corresponde a la fecha_inspeccion en que se registró; conservar el historial por inspección.</t>
+          <t xml:space="preserve">Seleccionar un único intervalo. No establecer equivalencias automáticas entre clase_edad y la edad cronológica. No utilizar únicamente el DAP como determinante de la edad. La estimación corresponde a la fecha_inspeccion en que se registró; conservar el historial por inspección. Opcional mientras no se valide la factibilidad de su estimación; no se exige para finalizar la inspección.</t>
         </is>
       </c>
     </row>
@@ -16235,8 +16308,10 @@
         <v>525</v>
       </c>
       <c r="K83" s="7"/>
-      <c r="L83" s="7" t="s">
-        <v>526</v>
+      <c r="L83" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Valor numérico entre 0 y 100 %. 0 % representa ausencia de pérdida de follaje respecto del árbol de referencia. La estimación debe realizarse sobre la copa evaluable y respecto de una condición de referencia comparable. En especies con persistencia_follaje = Caducifolia o Semicaducifolia (CATALOGO_ESPECIES) evaluadas en receso vegetativo, la referencia es la copa de la misma especie en esa condición estacional: la pérdida estacional de hojas no se registra como defoliación.</t>
+        </is>
       </c>
     </row>
     <row r="84" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -19972,11 +20047,15 @@
       <c r="D178" s="33" t="s">
         <v>1071</v>
       </c>
-      <c r="E178" s="41" t="s">
-        <v>1072</v>
-      </c>
-      <c r="F178" s="33" t="s">
-        <v>1073</v>
+      <c r="E178" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mediante el ingreso del nombre de la persona que comunica la incidencia en el formulario ciudadano público, al que se accede por el código QR del árbol.</t>
+        </is>
+      </c>
+      <c r="F178" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nombre de la persona natural que informa una situación relacionada con el arbolado urbano o su interacción con la infraestructura. Es un dato personal: solo lo ve el Usuario municipal y se conserva únicamente mientras se revisa la incidencia.</t>
+        </is>
       </c>
       <c r="G178" s="33" t="s">
         <v>343</v>
@@ -19984,12 +20063,14 @@
       <c r="H178" s="33" t="s">
         <v>1074</v>
       </c>
-      <c r="I178" s="33" t="s">
-        <v>324</v>
+      <c r="I178" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Obligatorio al reportar</t>
+        </is>
       </c>
       <c r="L178" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aceptar caracteres alfabéticos, espacios y tildes. Limitar a 100 caracteres.</t>
+          <t xml:space="preserve">Aceptar caracteres alfabéticos, espacios y tildes. Limitar a 100 caracteres. Visible solo para el Usuario municipal. Se elimina junto con rut_reportante cuando resultado_revision = Validada o Descartada; con Requiere antecedentes se conserva hasta el resultado final.</t>
         </is>
       </c>
     </row>
@@ -20006,11 +20087,15 @@
       <c r="D179" s="33" t="s">
         <v>1071</v>
       </c>
-      <c r="E179" s="41" t="s">
-        <v>1076</v>
-      </c>
-      <c r="F179" s="33" t="s">
-        <v>1077</v>
+      <c r="E179" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mediante el ingreso del RUT de la persona que comunica la incidencia en el formulario ciudadano público, al que se accede por el código QR del árbol.</t>
+        </is>
+      </c>
+      <c r="F179" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Identificador tributario de la persona natural que reporta. Es un dato personal: solo lo ve el Usuario municipal y se conserva únicamente mientras se revisa la incidencia.</t>
+        </is>
       </c>
       <c r="G179" s="33" t="s">
         <v>343</v>
@@ -20018,12 +20103,14 @@
       <c r="H179" s="33" t="s">
         <v>1078</v>
       </c>
-      <c r="I179" s="33" t="s">
-        <v>324</v>
+      <c r="I179" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Obligatorio al reportar</t>
+        </is>
       </c>
       <c r="L179" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Validar estructura y dígito verificador del RUT.</t>
+          <t xml:space="preserve">Validar estructura y dígito verificador del RUT. Visible solo para el Usuario municipal. Se elimina junto con nombre_reportante cuando resultado_revision = Validada o Descartada; con Requiere antecedentes se conserva hasta el resultado final.</t>
         </is>
       </c>
     </row>
@@ -20306,8 +20393,10 @@
       <c r="E187" s="41" t="s">
         <v>1088</v>
       </c>
-      <c r="F187" s="33" t="s">
-        <v>1089</v>
+      <c r="F187" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Resultado administrativo de la verificación municipal del reporte. Validada: el reporte requiere atención. Descartada: no corresponde atenderlo. Requiere antecedentes: la información disponible no basta para decidir y es necesario que el Inspector confirme en terreno el estado del árbol; no implica pedir información al reportante.</t>
+        </is>
       </c>
       <c r="G187" s="33" t="s">
         <v>357</v>
@@ -20327,7 +20416,7 @@
       </c>
       <c r="L187" s="42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Debe utilizar valores de un catálogo controlado.</t>
+          <t xml:space="preserve">Debe utilizar valores de un catálogo controlado. Requiere antecedentes es un resultado intermedio: el Usuario municipal crea una OT de Inspección del árbol vinculada mediante id_incidencia y, con el resultado de esa inspección, registra Validada o Descartada. Al registrar Validada o Descartada se eliminan nombre_reportante y rut_reportante.</t>
         </is>
       </c>
     </row>
@@ -20892,7 +20981,7 @@
       </c>
       <c r="L202" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Posterior a fecha_inspeccion. Mostrar el rango sugerido; al llegar la fecha de inicio, enviarla al calendario del módulo para agendarla. Si el Inspector la modifica, exigir justificacion_ajuste_fecha.</t>
+          <t xml:space="preserve">Posterior a fecha_inspeccion. Mostrar el rango sugerido. Al llegar la fecha de inicio, SIVU la muestra como recordatorio en la lista de próximas inspecciones del proyecto, desde la cual el Usuario municipal crea y programa la OT; SIVU no agenda automáticamente. Si el Inspector la modifica, exigir justificacion_ajuste_fecha.</t>
         </is>
       </c>
     </row>
@@ -20954,7 +21043,7 @@
       </c>
       <c r="L203" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Igual o posterior a fecha_inspeccion. Mostrar el rango sugerido; al llegar la fecha de inicio, enviarla al calendario del módulo para agendarla. Si el Inspector la modifica, exigir justificacion_ajuste_fecha.</t>
+          <t xml:space="preserve">Igual o posterior a fecha_inspeccion. Mostrar el rango sugerido. Al llegar la fecha de inicio, SIVU la muestra como recordatorio en la lista de próximos monitoreos del proyecto, desde la cual el Usuario municipal crea y programa la OT; SIVU no agenda automáticamente. Si el Inspector la modifica, exigir justificacion_ajuste_fecha.</t>
         </is>
       </c>
     </row>
@@ -21176,149 +21265,234 @@
       </c>
       <c r="D209" s="33" t="inlineStr">
         <is>
+          <t xml:space="preserve">Sistema / Inspector (solo la anulación)</t>
+        </is>
+      </c>
+      <c r="E209" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Asignación automática según la completitud de los datos obligatorios aplicables de la inspección. El valor Anulado lo registra el Inspector.</t>
+        </is>
+      </c>
+      <c r="F209" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estado del registro de la inspección. Preguardado: falta al menos un dato obligatorio aplicable. Finalizado: todos los datos obligatorios aplicables están registrados. Anulado: inspección finalizada que el Inspector anuló por contener un error; se conserva en el historial y no se considera para la vigencia.</t>
+        </is>
+      </c>
+      <c r="G209" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Categoría</t>
+        </is>
+      </c>
+      <c r="H209" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Preguardado / Finalizado / Anulado</t>
+        </is>
+      </c>
+      <c r="I209" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Obligatorio</t>
+        </is>
+      </c>
+      <c r="J209" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Finalizado cuando están completos todos los campos obligatorios y los condicionales activados de la inspección, de su REGISTRO_EVALUACION y de los datos técnicos del árbol registrados en ella; en otro caso, Preguardado. Anulado solo desde Finalizado, cuando el Inspector registra motivo_anulacion.</t>
+        </is>
+      </c>
+      <c r="K209" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Al guardar la inspección.</t>
+        </is>
+      </c>
+      <c r="L209" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No editable manualmente, salvo la anulación por el Inspector. Valor inicial: Preguardado. Una inspección Preguardado o Anulado no modifica la evaluación vigente del árbol. Mientras alguna inspección vinculada esté Preguardado, la OT no puede pasar a estado_ot = Completada. Una medición pendiente no equivale a cero ni a No presenta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="210" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A210" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INSPECCION</t>
+        </is>
+      </c>
+      <c r="B210" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">motivo_anulacion</t>
+        </is>
+      </c>
+      <c r="C210" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="D210" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Inspector</t>
+        </is>
+      </c>
+      <c r="E210" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Descripción libre del Inspector al anular la inspección.</t>
+        </is>
+      </c>
+      <c r="F210" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fundamento de la anulación de una inspección finalizada que contiene un error.</t>
+        </is>
+      </c>
+      <c r="G210" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Texto</t>
+        </is>
+      </c>
+      <c r="H210" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No aplica</t>
+        </is>
+      </c>
+      <c r="I210" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Condicional</t>
+        </is>
+      </c>
+      <c r="J210" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No aplica.</t>
+        </is>
+      </c>
+      <c r="K210" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">estado_registro = Anulado</t>
+        </is>
+      </c>
+      <c r="L210" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Texto libre, no vacío. Solo el Inspector anula. No editable después de registrar la anulación.</t>
+        </is>
+      </c>
+    </row>
+    <row r="211" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A211" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INSPECCION</t>
+        </is>
+      </c>
+      <c r="B211" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">anulado_por</t>
+        </is>
+      </c>
+      <c r="C211" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vinculado por plataforma</t>
+        </is>
+      </c>
+      <c r="D211" s="33" t="inlineStr">
+        <is>
           <t xml:space="preserve">Sistema</t>
         </is>
       </c>
-      <c r="E209" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Asignación automática según la completitud de los datos obligatorios aplicables de la inspección.</t>
-        </is>
-      </c>
-      <c r="F209" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Estado de completitud del registro de la inspección. Preguardado: falta al menos un dato obligatorio aplicable. Finalizado: todos los datos obligatorios aplicables están registrados.</t>
-        </is>
-      </c>
-      <c r="G209" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Categoría</t>
-        </is>
-      </c>
-      <c r="H209" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Preguardado / Finalizado</t>
-        </is>
-      </c>
-      <c r="I209" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Obligatorio</t>
-        </is>
-      </c>
-      <c r="J209" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Finalizado cuando están completos todos los campos obligatorios y los condicionales activados de la inspección, de su REGISTRO_EVALUACION y de los datos técnicos del árbol registrados en ella; en otro caso, Preguardado.</t>
-        </is>
-      </c>
-      <c r="K209" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Al guardar la inspección.</t>
-        </is>
-      </c>
-      <c r="L209" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No editable manualmente. Valor inicial: Preguardado. Una inspección Preguardado no modifica la evaluación vigente del árbol. Mientras alguna inspección vinculada esté Preguardado, la OT no puede pasar a estado_ot = Completada. Una medición pendiente no equivale a cero ni a No presenta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="210" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A210" s="41" t="s">
-        <v>790</v>
-      </c>
-      <c r="B210" s="41" t="s">
-        <v>198</v>
-      </c>
-      <c r="C210" s="33" t="s">
-        <v>318</v>
-      </c>
-      <c r="D210" s="33" t="s">
-        <v>319</v>
-      </c>
-      <c r="E210" s="41" t="s">
-        <v>320</v>
-      </c>
-      <c r="F210" s="33" t="s">
-        <v>791</v>
-      </c>
-      <c r="G210" s="33" t="s">
-        <v>322</v>
-      </c>
-      <c r="H210" s="33" t="s">
-        <v>792</v>
-      </c>
-      <c r="I210" s="33" t="s">
-        <v>324</v>
-      </c>
-      <c r="K210" s="8"/>
-      <c r="L210" s="8" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="211" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A211" s="41" t="s">
-        <v>790</v>
-      </c>
-      <c r="B211" s="41" t="s">
-        <v>177</v>
-      </c>
-      <c r="C211" s="33" t="s">
-        <v>326</v>
-      </c>
-      <c r="D211" s="33" t="s">
-        <v>319</v>
-      </c>
-      <c r="E211" s="41" t="s">
-        <v>328</v>
-      </c>
-      <c r="F211" s="33" t="s">
-        <v>793</v>
-      </c>
-      <c r="G211" s="33" t="s">
-        <v>322</v>
-      </c>
-      <c r="H211" s="33" t="s">
-        <v>323</v>
-      </c>
-      <c r="I211" s="33" t="s">
-        <v>324</v>
-      </c>
-      <c r="K211" s="8"/>
+      <c r="E211" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Usuario autenticado que anula la inspección.</t>
+        </is>
+      </c>
+      <c r="F211" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Inspector que anuló la inspección.</t>
+        </is>
+      </c>
+      <c r="G211" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Identificador (texto)</t>
+        </is>
+      </c>
+      <c r="H211" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No aplica</t>
+        </is>
+      </c>
+      <c r="I211" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Condicional</t>
+        </is>
+      </c>
+      <c r="J211" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No aplica.</t>
+        </is>
+      </c>
+      <c r="K211" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">estado_registro = Anulado</t>
+        </is>
+      </c>
       <c r="L211" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Referencia válida a ORDENES DE TRABAJO con Tipo_ot = Mantenimiento. Una OT puede tener varios registros de MANTENIMIENTO: si una ejecución es rechazada, la corrección se registra como un nuevo registro y se conservan los anteriores.</t>
+          <t xml:space="preserve">Referencia válida a USUARIOS con rol Inspector. Conservar autoría histórica.</t>
         </is>
       </c>
     </row>
     <row r="212" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A212" s="41" t="s">
-        <v>790</v>
-      </c>
-      <c r="B212" s="41" t="s">
-        <v>0</v>
-      </c>
-      <c r="C212" s="33" t="s">
-        <v>326</v>
-      </c>
-      <c r="D212" s="33" t="s">
-        <v>319</v>
-      </c>
-      <c r="E212" s="41" t="s">
-        <v>746</v>
-      </c>
-      <c r="F212" s="33" t="s">
-        <v>795</v>
-      </c>
-      <c r="G212" s="33" t="s">
-        <v>322</v>
-      </c>
-      <c r="H212" s="33" t="s">
-        <v>323</v>
-      </c>
-      <c r="I212" s="33" t="s">
-        <v>324</v>
-      </c>
-      <c r="K212" s="8"/>
-      <c r="L212" s="8" t="s">
-        <v>748</v>
+      <c r="A212" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INSPECCION</t>
+        </is>
+      </c>
+      <c r="B212" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fecha_anulacion</t>
+        </is>
+      </c>
+      <c r="C212" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sistema</t>
+        </is>
+      </c>
+      <c r="D212" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sistema</t>
+        </is>
+      </c>
+      <c r="E212" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fecha y hora asignadas por el sistema al registrar la anulación.</t>
+        </is>
+      </c>
+      <c r="F212" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Momento en que la inspección fue anulada.</t>
+        </is>
+      </c>
+      <c r="G212" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fecha y hora</t>
+        </is>
+      </c>
+      <c r="H212" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dd/mm/aaaa HH:mm</t>
+        </is>
+      </c>
+      <c r="I212" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Condicional</t>
+        </is>
+      </c>
+      <c r="J212" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No aplica.</t>
+        </is>
+      </c>
+      <c r="K212" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">estado_registro = Anulado</t>
+        </is>
+      </c>
+      <c r="L212" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Igual o posterior a fecha_registro. No editable.</t>
+        </is>
       </c>
     </row>
     <row r="213" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -21326,32 +21500,32 @@
         <v>790</v>
       </c>
       <c r="B213" s="41" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C213" s="33" t="s">
-        <v>276</v>
+        <v>318</v>
       </c>
       <c r="D213" s="33" t="s">
-        <v>261</v>
+        <v>319</v>
       </c>
       <c r="E213" s="41" t="s">
-        <v>749</v>
+        <v>320</v>
       </c>
       <c r="F213" s="33" t="s">
-        <v>796</v>
+        <v>791</v>
       </c>
       <c r="G213" s="33" t="s">
-        <v>335</v>
+        <v>322</v>
       </c>
       <c r="H213" s="33" t="s">
-        <v>336</v>
+        <v>792</v>
       </c>
       <c r="I213" s="33" t="s">
         <v>324</v>
       </c>
       <c r="K213" s="8"/>
       <c r="L213" s="8" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
     </row>
     <row r="214" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -21359,19 +21533,19 @@
         <v>790</v>
       </c>
       <c r="B214" s="41" t="s">
-        <v>200</v>
+        <v>177</v>
       </c>
       <c r="C214" s="33" t="s">
         <v>326</v>
       </c>
       <c r="D214" s="33" t="s">
-        <v>261</v>
+        <v>319</v>
       </c>
       <c r="E214" s="41" t="s">
-        <v>797</v>
+        <v>328</v>
       </c>
       <c r="F214" s="33" t="s">
-        <v>798</v>
+        <v>793</v>
       </c>
       <c r="G214" s="33" t="s">
         <v>322</v>
@@ -21383,8 +21557,10 @@
         <v>324</v>
       </c>
       <c r="K214" s="8"/>
-      <c r="L214" s="8" t="s">
-        <v>799</v>
+      <c r="L214" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Referencia válida a ORDENES DE TRABAJO con Tipo_ot = Mantenimiento. Una OT puede tener varios registros de MANTENIMIENTO: si una ejecución es rechazada, la corrección se registra como un nuevo registro y se conservan los anteriores.</t>
+        </is>
       </c>
     </row>
     <row r="215" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -21392,32 +21568,32 @@
         <v>790</v>
       </c>
       <c r="B215" s="41" t="s">
-        <v>201</v>
+        <v>0</v>
       </c>
       <c r="C215" s="33" t="s">
-        <v>276</v>
+        <v>326</v>
       </c>
       <c r="D215" s="33" t="s">
-        <v>261</v>
+        <v>319</v>
       </c>
       <c r="E215" s="41" t="s">
-        <v>721</v>
+        <v>746</v>
       </c>
       <c r="F215" s="33" t="s">
-        <v>800</v>
+        <v>795</v>
       </c>
       <c r="G215" s="33" t="s">
-        <v>357</v>
+        <v>322</v>
       </c>
       <c r="H215" s="33" t="s">
-        <v>801</v>
+        <v>323</v>
       </c>
       <c r="I215" s="33" t="s">
         <v>324</v>
       </c>
       <c r="K215" s="8"/>
       <c r="L215" s="8" t="s">
-        <v>802</v>
+        <v>748</v>
       </c>
     </row>
     <row r="216" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -21425,7 +21601,7 @@
         <v>790</v>
       </c>
       <c r="B216" s="41" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="C216" s="33" t="s">
         <v>276</v>
@@ -21434,25 +21610,23 @@
         <v>261</v>
       </c>
       <c r="E216" s="41" t="s">
-        <v>803</v>
+        <v>749</v>
       </c>
       <c r="F216" s="33" t="s">
-        <v>804</v>
+        <v>796</v>
       </c>
       <c r="G216" s="33" t="s">
-        <v>357</v>
+        <v>335</v>
       </c>
       <c r="H216" s="33" t="s">
-        <v>805</v>
+        <v>336</v>
       </c>
       <c r="I216" s="33" t="s">
-        <v>363</v>
-      </c>
-      <c r="K216" s="8" t="s">
-        <v>806</v>
-      </c>
+        <v>324</v>
+      </c>
+      <c r="K216" s="8"/>
       <c r="L216" s="8" t="s">
-        <v>807</v>
+        <v>337</v>
       </c>
     </row>
     <row r="217" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -21460,40 +21634,32 @@
         <v>790</v>
       </c>
       <c r="B217" s="41" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="C217" s="33" t="s">
-        <v>276</v>
+        <v>326</v>
       </c>
       <c r="D217" s="33" t="s">
         <v>261</v>
       </c>
-      <c r="E217" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Selección desde lista.</t>
-        </is>
+      <c r="E217" s="41" t="s">
+        <v>797</v>
       </c>
       <c r="F217" s="33" t="s">
-        <v>809</v>
-      </c>
-      <c r="G217" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Categoría</t>
-        </is>
-      </c>
-      <c r="H217" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ejecutado completamente / Ejecutado parcialmente / No ejecutado</t>
-        </is>
+        <v>798</v>
+      </c>
+      <c r="G217" s="33" t="s">
+        <v>322</v>
+      </c>
+      <c r="H217" s="33" t="s">
+        <v>323</v>
       </c>
       <c r="I217" s="33" t="s">
         <v>324</v>
       </c>
       <c r="K217" s="8"/>
-      <c r="L217" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Seleccionar una opción de la lista. El cierre automático de la OT solo procede si resultado = Ejecutado completamente; en otro caso, la OT permanece En ejecución.</t>
-        </is>
+      <c r="L217" s="8" t="s">
+        <v>799</v>
       </c>
     </row>
     <row r="218" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -21501,7 +21667,7 @@
         <v>790</v>
       </c>
       <c r="B218" s="41" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
       <c r="C218" s="33" t="s">
         <v>276</v>
@@ -21510,23 +21676,23 @@
         <v>261</v>
       </c>
       <c r="E218" s="41" t="s">
-        <v>811</v>
+        <v>721</v>
       </c>
       <c r="F218" s="33" t="s">
-        <v>812</v>
+        <v>800</v>
       </c>
       <c r="G218" s="33" t="s">
-        <v>343</v>
+        <v>357</v>
       </c>
       <c r="H218" s="33" t="s">
-        <v>323</v>
+        <v>801</v>
       </c>
       <c r="I218" s="33" t="s">
-        <v>439</v>
+        <v>324</v>
       </c>
       <c r="K218" s="8"/>
       <c r="L218" s="8" t="s">
-        <v>730</v>
+        <v>802</v>
       </c>
     </row>
     <row r="219" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -21534,7 +21700,7 @@
         <v>790</v>
       </c>
       <c r="B219" s="41" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C219" s="33" t="s">
         <v>276</v>
@@ -21543,29 +21709,33 @@
         <v>261</v>
       </c>
       <c r="E219" s="41" t="s">
-        <v>721</v>
+        <v>803</v>
       </c>
       <c r="F219" s="33" t="s">
-        <v>813</v>
+        <v>804</v>
       </c>
       <c r="G219" s="33" t="s">
         <v>357</v>
       </c>
       <c r="H219" s="33" t="s">
-        <v>358</v>
+        <v>805</v>
       </c>
       <c r="I219" s="33" t="s">
-        <v>324</v>
-      </c>
-      <c r="K219" s="8"/>
-      <c r="L219" s="8"/>
+        <v>363</v>
+      </c>
+      <c r="K219" s="8" t="s">
+        <v>806</v>
+      </c>
+      <c r="L219" s="8" t="s">
+        <v>807</v>
+      </c>
     </row>
     <row r="220" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A220" s="41" t="s">
         <v>790</v>
       </c>
       <c r="B220" s="41" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C220" s="33" t="s">
         <v>276</v>
@@ -21573,26 +21743,32 @@
       <c r="D220" s="33" t="s">
         <v>261</v>
       </c>
-      <c r="E220" s="41" t="s">
-        <v>814</v>
+      <c r="E220" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Selección desde lista.</t>
+        </is>
       </c>
       <c r="F220" s="33" t="s">
-        <v>815</v>
-      </c>
-      <c r="G220" s="33" t="s">
-        <v>335</v>
-      </c>
-      <c r="H220" s="33" t="s">
-        <v>336</v>
+        <v>809</v>
+      </c>
+      <c r="G220" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Categoría</t>
+        </is>
+      </c>
+      <c r="H220" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ejecutado completamente / Ejecutado parcialmente / No ejecutado</t>
+        </is>
       </c>
       <c r="I220" s="33" t="s">
-        <v>363</v>
-      </c>
-      <c r="K220" s="8" t="s">
-        <v>816</v>
-      </c>
-      <c r="L220" s="8" t="s">
-        <v>817</v>
+        <v>324</v>
+      </c>
+      <c r="K220" s="8"/>
+      <c r="L220" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Seleccionar una opción de la lista. El cierre automático de la OT solo procede si resultado = Ejecutado completamente; en otro caso, la OT permanece En ejecución.</t>
+        </is>
       </c>
     </row>
     <row r="221" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -21600,7 +21776,7 @@
         <v>790</v>
       </c>
       <c r="B221" s="41" t="s">
-        <v>163</v>
+        <v>188</v>
       </c>
       <c r="C221" s="33" t="s">
         <v>276</v>
@@ -21609,27 +21785,23 @@
         <v>261</v>
       </c>
       <c r="E221" s="41" t="s">
-        <v>733</v>
+        <v>811</v>
       </c>
       <c r="F221" s="33" t="s">
-        <v>818</v>
+        <v>812</v>
       </c>
       <c r="G221" s="33" t="s">
-        <v>735</v>
+        <v>343</v>
       </c>
       <c r="H221" s="33" t="s">
-        <v>736</v>
-      </c>
-      <c r="I221" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Obligatorio</t>
-        </is>
+        <v>323</v>
+      </c>
+      <c r="I221" s="33" t="s">
+        <v>439</v>
       </c>
       <c r="K221" s="8"/>
-      <c r="L221" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Obligatoria para completar la OT. Conservar las imágenes vinculadas a cada registro de ejecución.</t>
-        </is>
+      <c r="L221" s="8" t="s">
+        <v>730</v>
       </c>
     </row>
     <row r="222" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -21637,85 +21809,65 @@
         <v>790</v>
       </c>
       <c r="B222" s="41" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C222" s="33" t="s">
         <v>276</v>
       </c>
-      <c r="D222" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sistema / Inspector</t>
-        </is>
+      <c r="D222" s="33" t="s">
+        <v>261</v>
       </c>
       <c r="E222" s="41" t="s">
         <v>721</v>
       </c>
-      <c r="F222" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Estado de la revisión de la acción ejecutada, realizada por el Inspector.</t>
-        </is>
+      <c r="F222" s="33" t="s">
+        <v>813</v>
       </c>
       <c r="G222" s="33" t="s">
         <v>357</v>
       </c>
       <c r="H222" s="33" t="s">
-        <v>821</v>
-      </c>
-      <c r="I222" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Condicional</t>
-        </is>
-      </c>
-      <c r="K222" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">requiere_revision_inspector = Sí en la orden de trabajo.</t>
-        </is>
-      </c>
-      <c r="L222" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Valor inicial: Pendiente de revisión, asignado por el Sistema. Aprobado o Rechazado lo registra el Inspector. Si requiere_revision_inspector = No, desactivar y dejar vacío.</t>
-        </is>
-      </c>
+        <v>358</v>
+      </c>
+      <c r="I222" s="33" t="s">
+        <v>324</v>
+      </c>
+      <c r="K222" s="8"/>
+      <c r="L222" s="8"/>
     </row>
     <row r="223" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A223" s="41" t="s">
         <v>790</v>
       </c>
       <c r="B223" s="41" t="s">
-        <v>165</v>
+        <v>205</v>
       </c>
       <c r="C223" s="33" t="s">
-        <v>326</v>
-      </c>
-      <c r="D223" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Inspector</t>
-        </is>
+        <v>276</v>
+      </c>
+      <c r="D223" s="33" t="s">
+        <v>261</v>
       </c>
       <c r="E223" s="41" t="s">
-        <v>823</v>
-      </c>
-      <c r="F223" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Inspector que revisa la acción ejecutada.</t>
-        </is>
+        <v>814</v>
+      </c>
+      <c r="F223" s="33" t="s">
+        <v>815</v>
       </c>
       <c r="G223" s="33" t="s">
-        <v>322</v>
+        <v>335</v>
       </c>
       <c r="H223" s="33" t="s">
-        <v>323</v>
+        <v>336</v>
       </c>
       <c r="I223" s="33" t="s">
         <v>363</v>
       </c>
       <c r="K223" s="8" t="s">
-        <v>825</v>
-      </c>
-      <c r="L223" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Referencia válida a USUARIOS con rol Inspector.</t>
-        </is>
+        <v>816</v>
+      </c>
+      <c r="L223" s="8" t="s">
+        <v>817</v>
       </c>
     </row>
     <row r="224" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -21723,36 +21875,36 @@
         <v>790</v>
       </c>
       <c r="B224" s="41" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C224" s="33" t="s">
         <v>276</v>
       </c>
-      <c r="D224" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Inspector</t>
-        </is>
+      <c r="D224" s="33" t="s">
+        <v>261</v>
       </c>
       <c r="E224" s="41" t="s">
-        <v>827</v>
+        <v>733</v>
       </c>
       <c r="F224" s="33" t="s">
-        <v>828</v>
+        <v>818</v>
       </c>
       <c r="G224" s="33" t="s">
-        <v>335</v>
+        <v>735</v>
       </c>
       <c r="H224" s="33" t="s">
-        <v>336</v>
-      </c>
-      <c r="I224" s="33" t="s">
-        <v>363</v>
-      </c>
-      <c r="K224" s="8" t="s">
-        <v>825</v>
-      </c>
-      <c r="L224" s="8" t="s">
-        <v>829</v>
+        <v>736</v>
+      </c>
+      <c r="I224" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Obligatorio</t>
+        </is>
+      </c>
+      <c r="K224" s="8"/>
+      <c r="L224" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Obligatoria para completar la OT. Conservar las imágenes vinculadas a cada registro de ejecución.</t>
+        </is>
       </c>
     </row>
     <row r="225" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -21760,45 +21912,55 @@
         <v>790</v>
       </c>
       <c r="B225" s="41" t="s">
-        <v>167</v>
+        <v>206</v>
       </c>
       <c r="C225" s="33" t="s">
         <v>276</v>
       </c>
       <c r="D225" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Inspector</t>
+          <t xml:space="preserve">Sistema / Inspector</t>
         </is>
       </c>
       <c r="E225" s="41" t="s">
-        <v>830</v>
-      </c>
-      <c r="F225" s="33" t="s">
-        <v>831</v>
+        <v>721</v>
+      </c>
+      <c r="F225" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estado de la revisión de la acción ejecutada, realizada por el Inspector.</t>
+        </is>
       </c>
       <c r="G225" s="33" t="s">
-        <v>343</v>
+        <v>357</v>
       </c>
       <c r="H225" s="33" t="s">
-        <v>323</v>
-      </c>
-      <c r="I225" s="33" t="s">
-        <v>363</v>
-      </c>
-      <c r="K225" s="8" t="s">
-        <v>832</v>
-      </c>
-      <c r="L225" s="8"/>
+        <v>821</v>
+      </c>
+      <c r="I225" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Condicional</t>
+        </is>
+      </c>
+      <c r="K225" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">requiere_revision_inspector = Sí en la orden de trabajo.</t>
+        </is>
+      </c>
+      <c r="L225" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Valor inicial: Pendiente de revisión, asignado por el Sistema. Aprobado o Rechazado lo registra el Inspector. Si requiere_revision_inspector = No, desactivar y dejar vacío.</t>
+        </is>
+      </c>
     </row>
     <row r="226" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A226" s="41" t="s">
         <v>790</v>
       </c>
       <c r="B226" s="41" t="s">
-        <v>207</v>
+        <v>165</v>
       </c>
       <c r="C226" s="33" t="s">
-        <v>276</v>
+        <v>326</v>
       </c>
       <c r="D226" s="33" t="inlineStr">
         <is>
@@ -21806,16 +21968,18 @@
         </is>
       </c>
       <c r="E226" s="41" t="s">
-        <v>721</v>
-      </c>
-      <c r="F226" s="33" t="s">
-        <v>833</v>
+        <v>823</v>
+      </c>
+      <c r="F226" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Inspector que revisa la acción ejecutada.</t>
+        </is>
       </c>
       <c r="G226" s="33" t="s">
-        <v>357</v>
+        <v>322</v>
       </c>
       <c r="H226" s="33" t="s">
-        <v>358</v>
+        <v>323</v>
       </c>
       <c r="I226" s="33" t="s">
         <v>363</v>
@@ -21823,14 +21987,18 @@
       <c r="K226" s="8" t="s">
         <v>825</v>
       </c>
-      <c r="L226" s="8"/>
+      <c r="L226" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Referencia válida a USUARIOS con rol Inspector.</t>
+        </is>
+      </c>
     </row>
     <row r="227" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A227" s="41" t="s">
         <v>790</v>
       </c>
       <c r="B227" s="41" t="s">
-        <v>208</v>
+        <v>164</v>
       </c>
       <c r="C227" s="33" t="s">
         <v>276</v>
@@ -21841,10 +22009,10 @@
         </is>
       </c>
       <c r="E227" s="41" t="s">
-        <v>834</v>
+        <v>827</v>
       </c>
       <c r="F227" s="33" t="s">
-        <v>835</v>
+        <v>828</v>
       </c>
       <c r="G227" s="33" t="s">
         <v>335</v>
@@ -21856,150 +22024,117 @@
         <v>363</v>
       </c>
       <c r="K227" s="8" t="s">
+        <v>825</v>
+      </c>
+      <c r="L227" s="8" t="s">
+        <v>829</v>
+      </c>
+    </row>
+    <row r="228" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A228" s="41" t="s">
+        <v>790</v>
+      </c>
+      <c r="B228" s="41" t="s">
+        <v>167</v>
+      </c>
+      <c r="C228" s="33" t="s">
+        <v>276</v>
+      </c>
+      <c r="D228" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Inspector</t>
+        </is>
+      </c>
+      <c r="E228" s="41" t="s">
+        <v>830</v>
+      </c>
+      <c r="F228" s="33" t="s">
+        <v>831</v>
+      </c>
+      <c r="G228" s="33" t="s">
+        <v>343</v>
+      </c>
+      <c r="H228" s="33" t="s">
+        <v>323</v>
+      </c>
+      <c r="I228" s="33" t="s">
+        <v>363</v>
+      </c>
+      <c r="K228" s="8" t="s">
+        <v>832</v>
+      </c>
+      <c r="L228" s="8"/>
+    </row>
+    <row r="229" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A229" s="41" t="s">
+        <v>790</v>
+      </c>
+      <c r="B229" s="41" t="s">
+        <v>207</v>
+      </c>
+      <c r="C229" s="33" t="s">
+        <v>276</v>
+      </c>
+      <c r="D229" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Inspector</t>
+        </is>
+      </c>
+      <c r="E229" s="41" t="s">
+        <v>721</v>
+      </c>
+      <c r="F229" s="33" t="s">
+        <v>833</v>
+      </c>
+      <c r="G229" s="33" t="s">
+        <v>357</v>
+      </c>
+      <c r="H229" s="33" t="s">
+        <v>358</v>
+      </c>
+      <c r="I229" s="33" t="s">
+        <v>363</v>
+      </c>
+      <c r="K229" s="8" t="s">
+        <v>825</v>
+      </c>
+      <c r="L229" s="8"/>
+    </row>
+    <row r="230" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A230" s="41" t="s">
+        <v>790</v>
+      </c>
+      <c r="B230" s="41" t="s">
+        <v>208</v>
+      </c>
+      <c r="C230" s="33" t="s">
+        <v>276</v>
+      </c>
+      <c r="D230" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Inspector</t>
+        </is>
+      </c>
+      <c r="E230" s="41" t="s">
+        <v>834</v>
+      </c>
+      <c r="F230" s="33" t="s">
+        <v>835</v>
+      </c>
+      <c r="G230" s="33" t="s">
+        <v>335</v>
+      </c>
+      <c r="H230" s="33" t="s">
+        <v>336</v>
+      </c>
+      <c r="I230" s="33" t="s">
+        <v>363</v>
+      </c>
+      <c r="K230" s="8" t="s">
         <v>836</v>
       </c>
-      <c r="L227" s="8" t="s">
+      <c r="L230" s="8" t="s">
         <v>837</v>
-      </c>
-    </row>
-    <row r="228" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A228" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ORDENES DE TRABAJO</t>
-        </is>
-      </c>
-      <c r="B228" s="41" t="s">
-        <v>220</v>
-      </c>
-      <c r="C228" s="33" t="s">
-        <v>318</v>
-      </c>
-      <c r="D228" s="33" t="s">
-        <v>319</v>
-      </c>
-      <c r="E228" s="41" t="s">
-        <v>320</v>
-      </c>
-      <c r="F228" s="33" t="s">
-        <v>839</v>
-      </c>
-      <c r="G228" s="33" t="s">
-        <v>322</v>
-      </c>
-      <c r="H228" s="33" t="s">
-        <v>840</v>
-      </c>
-      <c r="I228" s="33" t="s">
-        <v>324</v>
-      </c>
-      <c r="K228" s="8"/>
-      <c r="L228" s="8" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="229" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A229" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ORDENES DE TRABAJO</t>
-        </is>
-      </c>
-      <c r="B229" s="41" t="s">
-        <v>221</v>
-      </c>
-      <c r="C229" s="33" t="s">
-        <v>326</v>
-      </c>
-      <c r="D229" s="33" t="s">
-        <v>715</v>
-      </c>
-      <c r="E229" s="41" t="s">
-        <v>328</v>
-      </c>
-      <c r="F229" s="33" t="s">
-        <v>841</v>
-      </c>
-      <c r="G229" s="33" t="s">
-        <v>322</v>
-      </c>
-      <c r="H229" s="33" t="s">
-        <v>323</v>
-      </c>
-      <c r="I229" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Condicional</t>
-        </is>
-      </c>
-      <c r="K229" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Accion_solicitada distinta de Levantamiento.</t>
-        </is>
-      </c>
-      <c r="L229" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Referencia válida a ARBOLES. En OT de Levantamiento, dejar vacío; los árboles registrados o evaluados se vinculan mediante INSPECCION.id_arbol.</t>
-        </is>
-      </c>
-    </row>
-    <row r="230" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A230" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ORDENES DE TRABAJO</t>
-        </is>
-      </c>
-      <c r="B230" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">id_incidencia</t>
-        </is>
-      </c>
-      <c r="C230" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vinculado por plataforma</t>
-        </is>
-      </c>
-      <c r="D230" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sistema / Usuario municipal</t>
-        </is>
-      </c>
-      <c r="E230" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vinculación a la incidencia que origina la orden de trabajo.</t>
-        </is>
-      </c>
-      <c r="F230" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Incidencia reportada que origina la orden de trabajo.</t>
-        </is>
-      </c>
-      <c r="G230" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Identificador (texto)</t>
-        </is>
-      </c>
-      <c r="H230" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No aplica</t>
-        </is>
-      </c>
-      <c r="I230" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Condicional</t>
-        </is>
-      </c>
-      <c r="J230" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No aplica.</t>
-        </is>
-      </c>
-      <c r="K230" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cuando la orden de trabajo se origina en una incidencia.</t>
-        </is>
-      </c>
-      <c r="L230" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Referencia válida a INCIDENCIA.</t>
-        </is>
       </c>
     </row>
     <row r="231" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -22009,32 +22144,32 @@
         </is>
       </c>
       <c r="B231" s="41" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="C231" s="33" t="s">
-        <v>276</v>
+        <v>318</v>
       </c>
       <c r="D231" s="33" t="s">
-        <v>257</v>
+        <v>319</v>
       </c>
       <c r="E231" s="41" t="s">
-        <v>721</v>
+        <v>320</v>
       </c>
       <c r="F231" s="33" t="s">
-        <v>842</v>
+        <v>839</v>
       </c>
       <c r="G231" s="33" t="s">
-        <v>357</v>
+        <v>322</v>
       </c>
       <c r="H231" s="33" t="s">
-        <v>843</v>
+        <v>840</v>
       </c>
       <c r="I231" s="33" t="s">
         <v>324</v>
       </c>
       <c r="K231" s="8"/>
       <c r="L231" s="8" t="s">
-        <v>844</v>
+        <v>325</v>
       </c>
     </row>
     <row r="232" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -22044,36 +22179,40 @@
         </is>
       </c>
       <c r="B232" s="41" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="C232" s="33" t="s">
-        <v>845</v>
+        <v>326</v>
       </c>
       <c r="D232" s="33" t="s">
-        <v>257</v>
+        <v>715</v>
       </c>
       <c r="E232" s="41" t="s">
-        <v>846</v>
+        <v>328</v>
       </c>
       <c r="F232" s="33" t="s">
-        <v>847</v>
+        <v>841</v>
       </c>
       <c r="G232" s="33" t="s">
-        <v>848</v>
-      </c>
-      <c r="H232" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Inspección: Evaluación inicial; Reevaluación; Evaluación instrumental; Monitoreo; Levantamiento. Mantenimiento: Poda; Riego; Descompactación; Manejo fitosanitario; Tala_retiro; Reparación_alcorque; Soporte_tutorado; Otra_Intervención.</t>
-        </is>
-      </c>
-      <c r="I232" s="33" t="s">
-        <v>324</v>
-      </c>
-      <c r="K232" s="8" t="s">
-        <v>850</v>
-      </c>
-      <c r="L232" s="8" t="s">
-        <v>851</v>
+        <v>322</v>
+      </c>
+      <c r="H232" s="33" t="s">
+        <v>323</v>
+      </c>
+      <c r="I232" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Condicional</t>
+        </is>
+      </c>
+      <c r="K232" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accion_solicitada distinta de Levantamiento.</t>
+        </is>
+      </c>
+      <c r="L232" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Referencia válida a ARBOLES. En OT de Levantamiento, dejar vacío; los árboles registrados o evaluados se vinculan mediante INSPECCION.id_arbol.</t>
+        </is>
       </c>
     </row>
     <row r="233" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -22082,37 +22221,60 @@
           <t xml:space="preserve">ORDENES DE TRABAJO</t>
         </is>
       </c>
-      <c r="B233" s="41" t="s">
-        <v>224</v>
-      </c>
-      <c r="C233" s="33" t="s">
-        <v>845</v>
-      </c>
-      <c r="D233" s="33" t="s">
-        <v>257</v>
-      </c>
-      <c r="E233" s="41" t="s">
-        <v>852</v>
-      </c>
-      <c r="F233" s="33" t="s">
-        <v>853</v>
-      </c>
-      <c r="G233" s="33" t="s">
-        <v>848</v>
+      <c r="B233" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">id_incidencia</t>
+        </is>
+      </c>
+      <c r="C233" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vinculado por plataforma</t>
+        </is>
+      </c>
+      <c r="D233" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sistema / Usuario municipal</t>
+        </is>
+      </c>
+      <c r="E233" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vinculación a la incidencia que origina la orden de trabajo.</t>
+        </is>
+      </c>
+      <c r="F233" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Incidencia reportada que origina la orden de trabajo.</t>
+        </is>
+      </c>
+      <c r="G233" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Identificador (texto)</t>
+        </is>
       </c>
       <c r="H233" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reevaluación: Seguimiento; Post_intervención. Evaluación instrumental: Tomografía_sónica; Resistografía; Otra. Monitoreo: Fitosanitario; Estructural; Vitalidad. Poda: Sanitaria; Formación; Despeje; Reducción. Riego: Programado; Emergencia. Descompactación: Manual; Mecánica. Manejo fitosanitario: Preventivo; Correctivo; Retiro_residuos. Tala_retiro: Tala; Retiro_tocón.</t>
-        </is>
-      </c>
-      <c r="I233" s="33" t="s">
-        <v>363</v>
-      </c>
-      <c r="K233" s="8" t="s">
-        <v>855</v>
-      </c>
-      <c r="L233" s="8" t="s">
-        <v>856</v>
+          <t xml:space="preserve">No aplica</t>
+        </is>
+      </c>
+      <c r="I233" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Condicional</t>
+        </is>
+      </c>
+      <c r="J233" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No aplica.</t>
+        </is>
+      </c>
+      <c r="K233" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cuando la orden de trabajo se origina en una incidencia.</t>
+        </is>
+      </c>
+      <c r="L233" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Referencia válida a INCIDENCIA.</t>
+        </is>
       </c>
     </row>
     <row r="234" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -22122,7 +22284,7 @@
         </is>
       </c>
       <c r="B234" s="41" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="C234" s="33" t="s">
         <v>276</v>
@@ -22131,23 +22293,23 @@
         <v>257</v>
       </c>
       <c r="E234" s="41" t="s">
-        <v>857</v>
+        <v>721</v>
       </c>
       <c r="F234" s="33" t="s">
-        <v>858</v>
+        <v>842</v>
       </c>
       <c r="G234" s="33" t="s">
-        <v>343</v>
+        <v>357</v>
       </c>
       <c r="H234" s="33" t="s">
-        <v>323</v>
+        <v>843</v>
       </c>
       <c r="I234" s="33" t="s">
-        <v>439</v>
+        <v>324</v>
       </c>
       <c r="K234" s="8"/>
       <c r="L234" s="8" t="s">
-        <v>730</v>
+        <v>844</v>
       </c>
     </row>
     <row r="235" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -22157,34 +22319,36 @@
         </is>
       </c>
       <c r="B235" s="41" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="C235" s="33" t="s">
-        <v>276</v>
+        <v>845</v>
       </c>
       <c r="D235" s="33" t="s">
         <v>257</v>
       </c>
       <c r="E235" s="41" t="s">
-        <v>721</v>
+        <v>846</v>
       </c>
       <c r="F235" s="33" t="s">
-        <v>859</v>
+        <v>847</v>
       </c>
       <c r="G235" s="33" t="s">
-        <v>357</v>
-      </c>
-      <c r="H235" s="33" t="s">
-        <v>770</v>
+        <v>848</v>
+      </c>
+      <c r="H235" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Inspección: Evaluación inicial; Reevaluación; Evaluación instrumental; Monitoreo; Levantamiento. Mantenimiento: Poda; Riego; Descompactación; Manejo fitosanitario; Tala_retiro; Reparación_alcorque; Soporte_tutorado; Otra_Intervención.</t>
+        </is>
       </c>
       <c r="I235" s="33" t="s">
         <v>324</v>
       </c>
-      <c r="K235" s="8"/>
-      <c r="L235" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Si el árbol tiene una evaluación vigente, proponer por defecto su clasificacion_prioridad; el Usuario municipal puede modificarla.</t>
-        </is>
+      <c r="K235" s="8" t="s">
+        <v>850</v>
+      </c>
+      <c r="L235" s="8" t="s">
+        <v>851</v>
       </c>
     </row>
     <row r="236" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -22194,36 +22358,36 @@
         </is>
       </c>
       <c r="B236" s="41" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="C236" s="33" t="s">
-        <v>276</v>
-      </c>
-      <c r="D236" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Usuario municipal / Sistema</t>
-        </is>
+        <v>845</v>
+      </c>
+      <c r="D236" s="33" t="s">
+        <v>257</v>
       </c>
       <c r="E236" s="41" t="s">
-        <v>738</v>
+        <v>852</v>
       </c>
       <c r="F236" s="33" t="s">
-        <v>861</v>
+        <v>853</v>
       </c>
       <c r="G236" s="33" t="s">
-        <v>357</v>
-      </c>
-      <c r="H236" s="33" t="s">
-        <v>862</v>
+        <v>848</v>
+      </c>
+      <c r="H236" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reevaluación: Seguimiento; Post_intervención. Evaluación instrumental: Tomografía_sónica; Resistografía; Otra. Monitoreo: Fitosanitario; Estructural; Vitalidad. Poda: Sanitaria; Formación; Despeje; Reducción. Riego: Programado; Emergencia. Descompactación: Manual; Mecánica. Manejo fitosanitario: Preventivo; Correctivo; Retiro_residuos. Tala_retiro: Tala; Retiro_tocón.</t>
+        </is>
       </c>
       <c r="I236" s="33" t="s">
-        <v>324</v>
-      </c>
-      <c r="K236" s="8"/>
-      <c r="L236" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Valor inicial: Pendiente. No permitir Completada mientras alguna inspección vinculada tenga estado_registro = Preguardado. Al pasar a Completada, registrar fecha_completada_ot. En OT de Mantenimiento, el Sistema asigna Completada: si requiere_revision_inspector = No, al registrarse la ejecución con resultado = Ejecutado completamente y la evidencia fotográfica; si requiere_revision_inspector = Sí, cuando estado_revision = Aprobado. Si estado_revision = Rechazado, la OT vuelve a En ejecución.</t>
-        </is>
+        <v>363</v>
+      </c>
+      <c r="K236" s="8" t="s">
+        <v>855</v>
+      </c>
+      <c r="L236" s="8" t="s">
+        <v>856</v>
       </c>
     </row>
     <row r="237" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -22233,32 +22397,32 @@
         </is>
       </c>
       <c r="B237" s="41" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="C237" s="33" t="s">
-        <v>319</v>
+        <v>276</v>
       </c>
       <c r="D237" s="33" t="s">
-        <v>319</v>
+        <v>257</v>
       </c>
       <c r="E237" s="41" t="s">
-        <v>864</v>
+        <v>857</v>
       </c>
       <c r="F237" s="33" t="s">
-        <v>865</v>
+        <v>858</v>
       </c>
       <c r="G237" s="33" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
       <c r="H237" s="33" t="s">
-        <v>336</v>
+        <v>323</v>
       </c>
       <c r="I237" s="33" t="s">
-        <v>324</v>
+        <v>439</v>
       </c>
       <c r="K237" s="8"/>
       <c r="L237" s="8" t="s">
-        <v>337</v>
+        <v>730</v>
       </c>
     </row>
     <row r="238" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -22268,7 +22432,7 @@
         </is>
       </c>
       <c r="B238" s="41" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="C238" s="33" t="s">
         <v>276</v>
@@ -22277,25 +22441,25 @@
         <v>257</v>
       </c>
       <c r="E238" s="41" t="s">
-        <v>866</v>
+        <v>721</v>
       </c>
       <c r="F238" s="33" t="s">
-        <v>867</v>
+        <v>859</v>
       </c>
       <c r="G238" s="33" t="s">
-        <v>335</v>
+        <v>357</v>
       </c>
       <c r="H238" s="33" t="s">
-        <v>336</v>
+        <v>770</v>
       </c>
       <c r="I238" s="33" t="s">
-        <v>363</v>
-      </c>
-      <c r="K238" s="8" t="s">
-        <v>868</v>
-      </c>
-      <c r="L238" s="8" t="s">
-        <v>869</v>
+        <v>324</v>
+      </c>
+      <c r="K238" s="8"/>
+      <c r="L238" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Si el árbol tiene una evaluación vigente, proponer por defecto su clasificacion_prioridad; el Usuario municipal puede modificarla.</t>
+        </is>
       </c>
     </row>
     <row r="239" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -22304,59 +22468,36 @@
           <t xml:space="preserve">ORDENES DE TRABAJO</t>
         </is>
       </c>
-      <c r="B239" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">fecha_completada_ot</t>
-        </is>
-      </c>
-      <c r="C239" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sistema</t>
-        </is>
+      <c r="B239" s="41" t="s">
+        <v>227</v>
+      </c>
+      <c r="C239" s="33" t="s">
+        <v>276</v>
       </c>
       <c r="D239" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sistema</t>
-        </is>
-      </c>
-      <c r="E239" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fecha asignada por el sistema cuando estado_ot cambia a Completada.</t>
-        </is>
-      </c>
-      <c r="F239" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fecha en que se completa la orden de trabajo. Determina la evaluación vigente del árbol.</t>
-        </is>
-      </c>
-      <c r="G239" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fecha</t>
-        </is>
-      </c>
-      <c r="H239" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">dd/mm/aaaa</t>
-        </is>
-      </c>
-      <c r="I239" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Condicional</t>
-        </is>
-      </c>
-      <c r="J239" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No aplica.</t>
-        </is>
-      </c>
-      <c r="K239" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">estado_ot = Completada</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Usuario municipal / Sistema</t>
+        </is>
+      </c>
+      <c r="E239" s="41" t="s">
+        <v>738</v>
+      </c>
+      <c r="F239" s="33" t="s">
+        <v>861</v>
+      </c>
+      <c r="G239" s="33" t="s">
+        <v>357</v>
+      </c>
+      <c r="H239" s="33" t="s">
+        <v>862</v>
+      </c>
+      <c r="I239" s="33" t="s">
+        <v>324</v>
+      </c>
+      <c r="K239" s="8"/>
       <c r="L239" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">No editable manualmente. Igual o posterior a fecha_creacion_OT. La evaluación vigente corresponde a la OT completada más recientemente según esta fecha, aunque su fecha_inspeccion sea anterior a la de otra inspección.</t>
+          <t xml:space="preserve">Valor inicial: Pendiente. No permitir Completada mientras alguna inspección vinculada tenga estado_registro = Preguardado. Al pasar a Completada, registrar fecha_completada_ot. En OT de Mantenimiento, el Sistema asigna Completada: si requiere_revision_inspector = No, al registrarse la ejecución con resultado = Ejecutado completamente y la evidencia fotográfica; si requiere_revision_inspector = Sí, cuando estado_revision = Aprobado. Si estado_revision = Rechazado, la OT vuelve a En ejecución.</t>
         </is>
       </c>
     </row>
@@ -22366,37 +22507,33 @@
           <t xml:space="preserve">ORDENES DE TRABAJO</t>
         </is>
       </c>
-      <c r="B240" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ot_creado_por</t>
-        </is>
+      <c r="B240" s="41" t="s">
+        <v>228</v>
       </c>
       <c r="C240" s="33" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
       <c r="D240" s="33" t="s">
         <v>319</v>
       </c>
       <c r="E240" s="41" t="s">
-        <v>870</v>
+        <v>864</v>
       </c>
       <c r="F240" s="33" t="s">
-        <v>871</v>
+        <v>865</v>
       </c>
       <c r="G240" s="33" t="s">
-        <v>322</v>
+        <v>335</v>
       </c>
       <c r="H240" s="33" t="s">
-        <v>323</v>
+        <v>336</v>
       </c>
       <c r="I240" s="33" t="s">
         <v>324</v>
       </c>
       <c r="K240" s="8"/>
-      <c r="L240" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Referencia válida a USUARIOS.</t>
-        </is>
+      <c r="L240" s="8" t="s">
+        <v>337</v>
       </c>
     </row>
     <row r="241" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -22406,7 +22543,7 @@
         </is>
       </c>
       <c r="B241" s="41" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="C241" s="33" t="s">
         <v>276</v>
@@ -22415,23 +22552,25 @@
         <v>257</v>
       </c>
       <c r="E241" s="41" t="s">
-        <v>873</v>
+        <v>866</v>
       </c>
       <c r="F241" s="33" t="s">
-        <v>874</v>
+        <v>867</v>
       </c>
       <c r="G241" s="33" t="s">
-        <v>322</v>
+        <v>335</v>
       </c>
       <c r="H241" s="33" t="s">
-        <v>323</v>
+        <v>336</v>
       </c>
       <c r="I241" s="33" t="s">
-        <v>324</v>
-      </c>
-      <c r="K241" s="8"/>
+        <v>363</v>
+      </c>
+      <c r="K241" s="8" t="s">
+        <v>868</v>
+      </c>
       <c r="L241" s="8" t="s">
-        <v>875</v>
+        <v>869</v>
       </c>
     </row>
     <row r="242" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -22442,37 +22581,37 @@
       </c>
       <c r="B242" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">requiere_revision_inspector</t>
+          <t xml:space="preserve">fecha_completada_ot</t>
         </is>
       </c>
       <c r="C242" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manual</t>
+          <t xml:space="preserve">Sistema</t>
         </is>
       </c>
       <c r="D242" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Usuario municipal</t>
+          <t xml:space="preserve">Sistema</t>
         </is>
       </c>
       <c r="E242" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Selección al crear la orden de trabajo.</t>
+          <t xml:space="preserve">Fecha asignada por el sistema cuando estado_ot cambia a Completada.</t>
         </is>
       </c>
       <c r="F242" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Indica si la ejecución de la acción de mantenimiento debe ser aprobada o rechazada por el Inspector.</t>
+          <t xml:space="preserve">Fecha en que se completa la orden de trabajo. Determina la evaluación vigente del árbol.</t>
         </is>
       </c>
       <c r="G242" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Categoría</t>
+          <t xml:space="preserve">Fecha</t>
         </is>
       </c>
       <c r="H242" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sí / No</t>
+          <t xml:space="preserve">dd/mm/aaaa</t>
         </is>
       </c>
       <c r="I242" s="33" t="inlineStr">
@@ -22482,17 +22621,17 @@
       </c>
       <c r="J242" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Valor inicial: No. Si subtipo_accion = Tala o Retiro_tocón, el Sistema asigna Sí y no permite modificarlo.</t>
+          <t xml:space="preserve">No aplica.</t>
         </is>
       </c>
       <c r="K242" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tipo_ot = Mantenimiento</t>
+          <t xml:space="preserve">estado_ot = Completada</t>
         </is>
       </c>
       <c r="L242" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sí: la OT se completa cuando el Inspector registra estado_revision = Aprobado. No: la OT se completa automáticamente al registrarse en MANTENIMIENTO la ejecución con resultado = Ejecutado completamente y la evidencia fotográfica. Si cambia Tipo_ot, Accion_solicitada o subtipo_accion, volver a aplicar la regla.</t>
+          <t xml:space="preserve">No editable manualmente. Igual o posterior a fecha_creacion_OT. La evaluación vigente corresponde a la OT completada más recientemente según esta fecha, aunque su fecha_inspeccion sea anterior a la de otra inspección.</t>
         </is>
       </c>
     </row>
@@ -22502,143 +22641,177 @@
           <t xml:space="preserve">ORDENES DE TRABAJO</t>
         </is>
       </c>
-      <c r="B243" s="41" t="s">
-        <v>188</v>
+      <c r="B243" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ot_creado_por</t>
+        </is>
       </c>
       <c r="C243" s="33" t="s">
-        <v>276</v>
+        <v>326</v>
       </c>
       <c r="D243" s="33" t="s">
-        <v>257</v>
+        <v>319</v>
       </c>
       <c r="E243" s="41" t="s">
-        <v>857</v>
-      </c>
-      <c r="F243" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Indicaciones complementarias para ejecutar la orden. En OT de Levantamiento, descripción del área de trabajo.</t>
-        </is>
+        <v>870</v>
+      </c>
+      <c r="F243" s="33" t="s">
+        <v>871</v>
       </c>
       <c r="G243" s="33" t="s">
-        <v>343</v>
+        <v>322</v>
       </c>
       <c r="H243" s="33" t="s">
         <v>323</v>
       </c>
       <c r="I243" s="33" t="s">
-        <v>363</v>
-      </c>
-      <c r="K243" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Accion_solicitada o subtipo_accion = Otra / Otra_Intervención, o Accion_solicitada = Levantamiento</t>
-        </is>
-      </c>
+        <v>324</v>
+      </c>
+      <c r="K243" s="8"/>
       <c r="L243" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obligatorio para especificar acciones o subtipos «Otra» y para describir el área de trabajo de una OT de Levantamiento; opcional en los demás casos.</t>
+          <t xml:space="preserve">Referencia válida a USUARIOS.</t>
         </is>
       </c>
     </row>
     <row r="244" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A244" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">USUARIOS</t>
+          <t xml:space="preserve">ORDENES DE TRABAJO</t>
         </is>
       </c>
       <c r="B244" s="41" t="s">
-        <v>244</v>
+        <v>231</v>
       </c>
       <c r="C244" s="33" t="s">
-        <v>318</v>
+        <v>276</v>
       </c>
       <c r="D244" s="33" t="s">
-        <v>319</v>
+        <v>257</v>
       </c>
       <c r="E244" s="41" t="s">
-        <v>1099</v>
+        <v>873</v>
       </c>
       <c r="F244" s="33" t="s">
-        <v>1100</v>
+        <v>874</v>
       </c>
       <c r="G244" s="33" t="s">
-        <v>343</v>
+        <v>322</v>
       </c>
       <c r="H244" s="33" t="s">
-        <v>1101</v>
+        <v>323</v>
       </c>
       <c r="I244" s="33" t="s">
         <v>324</v>
       </c>
-      <c r="L244" s="33" t="s">
-        <v>1102</v>
+      <c r="K244" s="8"/>
+      <c r="L244" s="8" t="s">
+        <v>875</v>
       </c>
     </row>
     <row r="245" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A245" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">USUARIOS</t>
-        </is>
-      </c>
-      <c r="B245" s="41" t="s">
-        <v>245</v>
-      </c>
-      <c r="C245" s="33" t="s">
-        <v>276</v>
-      </c>
-      <c r="D245" s="33" t="s">
-        <v>252</v>
-      </c>
-      <c r="E245" s="41" t="s">
-        <v>1103</v>
-      </c>
-      <c r="F245" s="33" t="s">
-        <v>1104</v>
-      </c>
-      <c r="G245" s="33" t="s">
-        <v>343</v>
-      </c>
-      <c r="H245" s="33" t="s">
-        <v>1105</v>
-      </c>
-      <c r="I245" s="33" t="s">
-        <v>324</v>
-      </c>
-      <c r="L245" s="33" t="s">
-        <v>1106</v>
+          <t xml:space="preserve">ORDENES DE TRABAJO</t>
+        </is>
+      </c>
+      <c r="B245" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">requiere_revision_inspector</t>
+        </is>
+      </c>
+      <c r="C245" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="D245" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Usuario municipal</t>
+        </is>
+      </c>
+      <c r="E245" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Selección al crear la orden de trabajo.</t>
+        </is>
+      </c>
+      <c r="F245" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Indica si la ejecución de la acción de mantenimiento debe ser aprobada o rechazada por el Inspector.</t>
+        </is>
+      </c>
+      <c r="G245" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Categoría</t>
+        </is>
+      </c>
+      <c r="H245" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sí / No</t>
+        </is>
+      </c>
+      <c r="I245" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Condicional</t>
+        </is>
+      </c>
+      <c r="J245" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Valor inicial: No. Si subtipo_accion = Tala o Retiro_tocón, el Sistema asigna Sí y no permite modificarlo.</t>
+        </is>
+      </c>
+      <c r="K245" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tipo_ot = Mantenimiento</t>
+        </is>
+      </c>
+      <c r="L245" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sí: la OT se completa cuando el Inspector registra estado_revision = Aprobado. No: la OT se completa automáticamente al registrarse en MANTENIMIENTO la ejecución con resultado = Ejecutado completamente y la evidencia fotográfica. Si cambia Tipo_ot, Accion_solicitada o subtipo_accion, volver a aplicar la regla.</t>
+        </is>
       </c>
     </row>
     <row r="246" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A246" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">USUARIOS</t>
+          <t xml:space="preserve">ORDENES DE TRABAJO</t>
         </is>
       </c>
       <c r="B246" s="41" t="s">
-        <v>246</v>
+        <v>188</v>
       </c>
       <c r="C246" s="33" t="s">
         <v>276</v>
       </c>
       <c r="D246" s="33" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="E246" s="41" t="s">
-        <v>1107</v>
-      </c>
-      <c r="F246" s="41" t="s">
-        <v>1108</v>
+        <v>857</v>
+      </c>
+      <c r="F246" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Indicaciones complementarias para ejecutar la orden. En OT de Levantamiento, descripción del área de trabajo.</t>
+        </is>
       </c>
       <c r="G246" s="33" t="s">
-        <v>246</v>
+        <v>343</v>
       </c>
       <c r="H246" s="33" t="s">
-        <v>1109</v>
+        <v>323</v>
       </c>
       <c r="I246" s="33" t="s">
-        <v>324</v>
-      </c>
-      <c r="L246" s="33" t="s">
-        <v>1110</v>
+        <v>363</v>
+      </c>
+      <c r="K246" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accion_solicitada o subtipo_accion = Otra / Otra_Intervención, o Accion_solicitada = Levantamiento</t>
+        </is>
+      </c>
+      <c r="L246" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Obligatorio para especificar acciones o subtipos «Otra» y para describir el área de trabajo de una OT de Levantamiento; opcional en los demás casos.</t>
+        </is>
       </c>
     </row>
     <row r="247" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -22648,31 +22821,31 @@
         </is>
       </c>
       <c r="B247" s="41" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="C247" s="33" t="s">
-        <v>276</v>
+        <v>318</v>
       </c>
       <c r="D247" s="33" t="s">
-        <v>252</v>
+        <v>319</v>
       </c>
       <c r="E247" s="41" t="s">
-        <v>1111</v>
+        <v>1099</v>
       </c>
       <c r="F247" s="33" t="s">
-        <v>1112</v>
+        <v>1100</v>
       </c>
       <c r="G247" s="33" t="s">
-        <v>357</v>
+        <v>343</v>
       </c>
       <c r="H247" s="33" t="s">
-        <v>1113</v>
+        <v>1101</v>
       </c>
       <c r="I247" s="33" t="s">
         <v>324</v>
       </c>
       <c r="L247" s="33" t="s">
-        <v>1114</v>
+        <v>1102</v>
       </c>
     </row>
     <row r="248" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -22682,7 +22855,7 @@
         </is>
       </c>
       <c r="B248" s="41" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="C248" s="33" t="s">
         <v>276</v>
@@ -22691,111 +22864,100 @@
         <v>252</v>
       </c>
       <c r="E248" s="41" t="s">
-        <v>1115</v>
+        <v>1103</v>
       </c>
       <c r="F248" s="33" t="s">
-        <v>1116</v>
+        <v>1104</v>
       </c>
       <c r="G248" s="33" t="s">
-        <v>357</v>
+        <v>343</v>
       </c>
       <c r="H248" s="33" t="s">
-        <v>358</v>
+        <v>1105</v>
       </c>
       <c r="I248" s="33" t="s">
         <v>324</v>
       </c>
-      <c r="J248" s="33" t="s">
-        <v>1117</v>
-      </c>
       <c r="L248" s="33" t="s">
-        <v>1118</v>
+        <v>1106</v>
       </c>
     </row>
     <row r="249" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A249" s="41" t="s">
-        <v>1150</v>
+      <c r="A249" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">USUARIOS</t>
+        </is>
       </c>
       <c r="B249" s="41" t="s">
-        <v>1157</v>
+        <v>246</v>
       </c>
       <c r="C249" s="33" t="s">
-        <v>318</v>
+        <v>276</v>
       </c>
       <c r="D249" s="33" t="s">
-        <v>319</v>
+        <v>252</v>
       </c>
       <c r="E249" s="41" t="s">
-        <v>1159</v>
-      </c>
-      <c r="F249" s="33" t="s">
-        <v>1160</v>
+        <v>1107</v>
+      </c>
+      <c r="F249" s="41" t="s">
+        <v>1108</v>
       </c>
       <c r="G249" s="33" t="s">
-        <v>322</v>
+        <v>246</v>
       </c>
       <c r="H249" s="33" t="s">
-        <v>323</v>
+        <v>1109</v>
       </c>
       <c r="I249" s="33" t="s">
         <v>324</v>
       </c>
-      <c r="J249" s="33" t="s">
-        <v>1161</v>
-      </c>
-      <c r="K249" s="33" t="s">
-        <v>1152</v>
-      </c>
       <c r="L249" s="33" t="s">
-        <v>1162</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="250" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A250" s="41" t="s">
-        <v>1150</v>
+      <c r="A250" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">USUARIOS</t>
+        </is>
       </c>
       <c r="B250" s="41" t="s">
-        <v>1</v>
+        <v>247</v>
       </c>
       <c r="C250" s="33" t="s">
-        <v>326</v>
+        <v>276</v>
       </c>
       <c r="D250" s="33" t="s">
-        <v>319</v>
+        <v>252</v>
       </c>
       <c r="E250" s="41" t="s">
-        <v>1163</v>
+        <v>1111</v>
       </c>
       <c r="F250" s="33" t="s">
-        <v>1164</v>
+        <v>1112</v>
       </c>
       <c r="G250" s="33" t="s">
-        <v>322</v>
+        <v>357</v>
       </c>
       <c r="H250" s="33" t="s">
-        <v>323</v>
+        <v>1113</v>
       </c>
       <c r="I250" s="33" t="s">
         <v>324</v>
       </c>
-      <c r="J250" s="33" t="s">
-        <v>1151</v>
-      </c>
-      <c r="K250" s="33" t="s">
-        <v>1152</v>
-      </c>
-      <c r="L250" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Debe referenciar un proyecto existente. El Administrador debe tener autorización para gestionarlo. Un único sector por proyecto.</t>
-        </is>
+      <c r="L250" s="33" t="s">
+        <v>1114</v>
       </c>
     </row>
     <row r="251" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A251" s="41" t="s">
-        <v>1150</v>
+      <c r="A251" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">USUARIOS</t>
+        </is>
       </c>
       <c r="B251" s="41" t="s">
-        <v>1158</v>
+        <v>248</v>
       </c>
       <c r="C251" s="33" t="s">
         <v>276</v>
@@ -22804,32 +22966,25 @@
         <v>252</v>
       </c>
       <c r="E251" s="41" t="s">
-        <v>1166</v>
-      </c>
-      <c r="F251" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nombre visible de la delimitación territorial del proyecto, utilizada para consultar indicadores territoriales.</t>
-        </is>
+        <v>1115</v>
+      </c>
+      <c r="F251" s="33" t="s">
+        <v>1116</v>
       </c>
       <c r="G251" s="33" t="s">
-        <v>343</v>
+        <v>357</v>
       </c>
       <c r="H251" s="33" t="s">
-        <v>323</v>
+        <v>358</v>
       </c>
       <c r="I251" s="33" t="s">
         <v>324</v>
       </c>
       <c r="J251" s="33" t="s">
-        <v>1151</v>
-      </c>
-      <c r="K251" s="33" t="s">
-        <v>1168</v>
-      </c>
-      <c r="L251" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No vacío. Su modificación no altera id_sector.</t>
-        </is>
+        <v>1117</v>
+      </c>
+      <c r="L251" s="33" t="s">
+        <v>1118</v>
       </c>
     </row>
     <row r="252" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -22837,37 +22992,37 @@
         <v>1150</v>
       </c>
       <c r="B252" s="41" t="s">
-        <v>1153</v>
+        <v>1157</v>
       </c>
       <c r="C252" s="33" t="s">
-        <v>1154</v>
+        <v>318</v>
       </c>
       <c r="D252" s="33" t="s">
-        <v>252</v>
-      </c>
-      <c r="E252" s="60" t="s">
-        <v>1170</v>
+        <v>319</v>
+      </c>
+      <c r="E252" s="41" t="s">
+        <v>1159</v>
       </c>
       <c r="F252" s="33" t="s">
-        <v>1171</v>
+        <v>1160</v>
       </c>
       <c r="G252" s="33" t="s">
-        <v>1155</v>
+        <v>322</v>
       </c>
       <c r="H252" s="33" t="s">
-        <v>1172</v>
+        <v>323</v>
       </c>
       <c r="I252" s="33" t="s">
         <v>324</v>
       </c>
       <c r="J252" s="33" t="s">
-        <v>1173</v>
+        <v>1161</v>
       </c>
       <c r="K252" s="33" t="s">
-        <v>1174</v>
+        <v>1152</v>
       </c>
       <c r="L252" s="33" t="s">
-        <v>1175</v>
+        <v>1162</v>
       </c>
     </row>
     <row r="253" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -22875,410 +23030,344 @@
         <v>1150</v>
       </c>
       <c r="B253" s="41" t="s">
-        <v>1156</v>
+        <v>1</v>
       </c>
       <c r="C253" s="33" t="s">
-        <v>419</v>
+        <v>326</v>
       </c>
       <c r="D253" s="33" t="s">
         <v>319</v>
       </c>
       <c r="E253" s="41" t="s">
-        <v>1176</v>
+        <v>1163</v>
       </c>
       <c r="F253" s="33" t="s">
-        <v>1177</v>
+        <v>1164</v>
       </c>
       <c r="G253" s="33" t="s">
-        <v>347</v>
+        <v>322</v>
       </c>
       <c r="H253" s="33" t="s">
-        <v>567</v>
+        <v>323</v>
       </c>
       <c r="I253" s="33" t="s">
-        <v>1178</v>
+        <v>324</v>
       </c>
       <c r="J253" s="33" t="s">
-        <v>1179</v>
+        <v>1151</v>
       </c>
       <c r="K253" s="33" t="s">
-        <v>1180</v>
-      </c>
-      <c r="L253" s="33" t="s">
-        <v>1181</v>
+        <v>1152</v>
+      </c>
+      <c r="L253" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Debe referenciar un proyecto existente. El Administrador debe tener autorización para gestionarlo. Un único sector por proyecto.</t>
+        </is>
       </c>
     </row>
     <row r="254" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A254" s="41" t="s">
-        <v>1210</v>
+        <v>1150</v>
       </c>
       <c r="B254" s="41" t="s">
-        <v>10</v>
+        <v>1158</v>
       </c>
       <c r="C254" s="33" t="s">
         <v>276</v>
       </c>
       <c r="D254" s="33" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="E254" s="41" t="s">
-        <v>1214</v>
-      </c>
-      <c r="F254" s="33" t="s">
-        <v>1215</v>
+        <v>1166</v>
+      </c>
+      <c r="F254" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nombre visible de la delimitación territorial del proyecto, utilizada para consultar indicadores territoriales.</t>
+        </is>
       </c>
       <c r="G254" s="33" t="s">
         <v>343</v>
       </c>
       <c r="H254" s="33" t="s">
-        <v>1211</v>
+        <v>323</v>
       </c>
       <c r="I254" s="33" t="s">
-        <v>1216</v>
+        <v>324</v>
       </c>
       <c r="J254" s="33" t="s">
         <v>1151</v>
       </c>
       <c r="K254" s="33" t="s">
-        <v>1217</v>
-      </c>
-      <c r="L254" s="33" t="s">
-        <v>1218</v>
+        <v>1168</v>
+      </c>
+      <c r="L254" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No vacío. Su modificación no altera id_sector.</t>
+        </is>
       </c>
     </row>
     <row r="255" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A255" s="41" t="s">
-        <v>1210</v>
+        <v>1150</v>
       </c>
       <c r="B255" s="41" t="s">
-        <v>1208</v>
+        <v>1153</v>
       </c>
       <c r="C255" s="33" t="s">
-        <v>276</v>
+        <v>1154</v>
       </c>
       <c r="D255" s="33" t="s">
-        <v>259</v>
-      </c>
-      <c r="E255" s="41" t="s">
-        <v>1219</v>
+        <v>252</v>
+      </c>
+      <c r="E255" s="60" t="s">
+        <v>1170</v>
       </c>
       <c r="F255" s="33" t="s">
-        <v>1220</v>
+        <v>1171</v>
       </c>
       <c r="G255" s="33" t="s">
-        <v>343</v>
+        <v>1155</v>
       </c>
       <c r="H255" s="33" t="s">
-        <v>1212</v>
+        <v>1172</v>
       </c>
       <c r="I255" s="33" t="s">
-        <v>1221</v>
+        <v>324</v>
       </c>
       <c r="J255" s="33" t="s">
-        <v>1222</v>
+        <v>1173</v>
       </c>
       <c r="K255" s="33" t="s">
-        <v>1223</v>
+        <v>1174</v>
       </c>
       <c r="L255" s="33" t="s">
-        <v>1224</v>
+        <v>1175</v>
       </c>
     </row>
     <row r="256" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A256" s="41" t="s">
+        <v>1150</v>
+      </c>
+      <c r="B256" s="41" t="s">
+        <v>1156</v>
+      </c>
+      <c r="C256" s="33" t="s">
+        <v>419</v>
+      </c>
+      <c r="D256" s="33" t="s">
+        <v>319</v>
+      </c>
+      <c r="E256" s="41" t="s">
+        <v>1176</v>
+      </c>
+      <c r="F256" s="33" t="s">
+        <v>1177</v>
+      </c>
+      <c r="G256" s="33" t="s">
+        <v>347</v>
+      </c>
+      <c r="H256" s="33" t="s">
+        <v>567</v>
+      </c>
+      <c r="I256" s="33" t="s">
+        <v>1178</v>
+      </c>
+      <c r="J256" s="33" t="s">
+        <v>1179</v>
+      </c>
+      <c r="K256" s="33" t="s">
+        <v>1180</v>
+      </c>
+      <c r="L256" s="33" t="s">
+        <v>1181</v>
+      </c>
+    </row>
+    <row r="257" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A257" s="41" t="s">
         <v>1210</v>
       </c>
-      <c r="B256" s="41" t="s">
+      <c r="B257" s="41" t="s">
+        <v>10</v>
+      </c>
+      <c r="C257" s="33" t="s">
+        <v>276</v>
+      </c>
+      <c r="D257" s="33" t="s">
+        <v>259</v>
+      </c>
+      <c r="E257" s="41" t="s">
+        <v>1214</v>
+      </c>
+      <c r="F257" s="33" t="s">
+        <v>1215</v>
+      </c>
+      <c r="G257" s="33" t="s">
+        <v>343</v>
+      </c>
+      <c r="H257" s="33" t="s">
+        <v>1211</v>
+      </c>
+      <c r="I257" s="33" t="s">
+        <v>1216</v>
+      </c>
+      <c r="J257" s="33" t="s">
+        <v>1151</v>
+      </c>
+      <c r="K257" s="33" t="s">
+        <v>1217</v>
+      </c>
+      <c r="L257" s="33" t="s">
+        <v>1218</v>
+      </c>
+    </row>
+    <row r="258" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A258" s="41" t="s">
+        <v>1210</v>
+      </c>
+      <c r="B258" s="41" t="s">
+        <v>1208</v>
+      </c>
+      <c r="C258" s="33" t="s">
+        <v>276</v>
+      </c>
+      <c r="D258" s="33" t="s">
+        <v>259</v>
+      </c>
+      <c r="E258" s="41" t="s">
+        <v>1219</v>
+      </c>
+      <c r="F258" s="33" t="s">
+        <v>1220</v>
+      </c>
+      <c r="G258" s="33" t="s">
+        <v>343</v>
+      </c>
+      <c r="H258" s="33" t="s">
+        <v>1212</v>
+      </c>
+      <c r="I258" s="33" t="s">
+        <v>1221</v>
+      </c>
+      <c r="J258" s="33" t="s">
+        <v>1222</v>
+      </c>
+      <c r="K258" s="33" t="s">
+        <v>1223</v>
+      </c>
+      <c r="L258" s="33" t="s">
+        <v>1224</v>
+      </c>
+    </row>
+    <row r="259" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A259" s="41" t="s">
+        <v>1210</v>
+      </c>
+      <c r="B259" s="41" t="s">
         <v>1209</v>
       </c>
-      <c r="C256" s="33" t="s">
+      <c r="C259" s="33" t="s">
         <v>276</v>
       </c>
-      <c r="D256" s="33" t="s">
+      <c r="D259" s="33" t="s">
         <v>259</v>
       </c>
-      <c r="E256" s="41" t="s">
+      <c r="E259" s="41" t="s">
         <v>1225</v>
       </c>
-      <c r="F256" s="33" t="s">
+      <c r="F259" s="33" t="s">
         <v>1226</v>
       </c>
-      <c r="G256" s="33" t="s">
+      <c r="G259" s="33" t="s">
         <v>343</v>
       </c>
-      <c r="H256" s="33" t="s">
+      <c r="H259" s="33" t="s">
         <v>1213</v>
       </c>
-      <c r="I256" s="33" t="s">
+      <c r="I259" s="33" t="s">
         <v>1221</v>
       </c>
-      <c r="J256" s="33" t="s">
+      <c r="J259" s="33" t="s">
         <v>1227</v>
       </c>
-      <c r="K256" s="33" t="s">
+      <c r="K259" s="33" t="s">
         <v>1223</v>
       </c>
-      <c r="L256" s="33" t="s">
+      <c r="L259" s="33" t="s">
         <v>1228</v>
-      </c>
-    </row>
-    <row r="257" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A257" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CATALOGO_ESPECIES</t>
-        </is>
-      </c>
-      <c r="B257" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">origen_biogeografico</t>
-        </is>
-      </c>
-      <c r="C257" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Manual</t>
-        </is>
-      </c>
-      <c r="D257" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Inspector</t>
-        </is>
-      </c>
-      <c r="E257" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Asignación según la distribución natural de la especie respecto de Chile, consultando el Catálogo de las plantas vasculares de Chile (Rodríguez et al., 2018) o su versión en línea vigente.</t>
-        </is>
-      </c>
-      <c r="F257" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Clasificación de la especie según su procedencia biogeográfica respecto del territorio chileno. Endémica: especie nativa cuya distribución natural está restringida a Chile. Nativa: especie nativa de Chile cuya distribución natural no se restringe al país. Introducida: especie exótica presente en Chile fuera de su distribución natural.</t>
-        </is>
-      </c>
-      <c r="G257" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Categoría</t>
-        </is>
-      </c>
-      <c r="H257" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nativa / Endémica / Introducida</t>
-        </is>
-      </c>
-      <c r="I257" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Obligatorio para completar la clasificación del catálogo</t>
-        </is>
-      </c>
-      <c r="J257" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">La plataforma lo vincula al árbol mediante especie_cientifica.</t>
-        </is>
-      </c>
-      <c r="K257" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Al completar o actualizar la clasificación de la especie.</t>
-        </is>
-      </c>
-      <c r="L257" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Categorías excluyentes: una especie endémica no se registra como Nativa. Considerar la distribución natural de la especie respecto de Chile, no el lugar de plantación ni el origen del ejemplar. Si aún no se conoce, dejar nulo; no inventarlo ni bloquear el registro del árbol. Se muestra en la ficha del árbol mediante especie_cientifica; no se ingresa por ejemplar ni se duplica en ARBOLES. Si el árbol no tiene especie_cientifica vigente, se informa como Origen no determinado.</t>
-        </is>
-      </c>
-    </row>
-    <row r="258" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A258" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CATALOGO_ESPECIES</t>
-        </is>
-      </c>
-      <c r="B258" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">persistencia_follaje</t>
-        </is>
-      </c>
-      <c r="C258" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Manual</t>
-        </is>
-      </c>
-      <c r="D258" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Inspector</t>
-        </is>
-      </c>
-      <c r="E258" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Asignación según fuentes botánicas de referencia al incorporar o completar la especie en el catálogo.</t>
-        </is>
-      </c>
-      <c r="F258" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Comportamiento habitual del follaje de la especie a lo largo del año. Perennifolia: conserva follaje funcional durante todo el año, con renovación gradual. Caducifolia: pierde la totalidad del follaje durante la estación desfavorable. Semicaducifolia: pierde parcialmente el follaje, o lo pierde por un período breve, según las condiciones climáticas del año.</t>
-        </is>
-      </c>
-      <c r="G258" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Categoría</t>
-        </is>
-      </c>
-      <c r="H258" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Perennifolia / Caducifolia / Semicaducifolia</t>
-        </is>
-      </c>
-      <c r="I258" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Obligatorio para completar la clasificación del catálogo</t>
-        </is>
-      </c>
-      <c r="J258" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">La plataforma la vincula al árbol mediante especie_cientifica.</t>
-        </is>
-      </c>
-      <c r="K258" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Al completar o actualizar la clasificación de la especie.</t>
-        </is>
-      </c>
-      <c r="L258" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Corresponde al comportamiento habitual de la especie, no a la condición observada en el ejemplar. Si las fuentes describen un comportamiento variable, registrar el habitual en las condiciones climáticas de Valparaíso. Si aún no se conoce, dejar nulo; no inventarla ni bloquear el registro del árbol. No duplicar en ARBOLES. Si el árbol no tiene especie_cientifica vigente, no mostrar valor.</t>
-        </is>
-      </c>
-    </row>
-    <row r="259" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A259" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CATALOGO_ESPECIES</t>
-        </is>
-      </c>
-      <c r="B259" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tipo_hoja</t>
-        </is>
-      </c>
-      <c r="C259" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Manual</t>
-        </is>
-      </c>
-      <c r="D259" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Inspector</t>
-        </is>
-      </c>
-      <c r="E259" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Asignación según fuentes botánicas de referencia al incorporar o completar la especie en el catálogo.</t>
-        </is>
-      </c>
-      <c r="F259" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Morfología predominante de las hojas adultas de la especie. Latifoliada: lámina ancha y plana. Acicular: hoja alargada y angosta, en forma de aguja. Escuamiforme: hoja reducida a escamas adosadas a la ramilla. Palmera: hoja de palmera, palmada o pinnada.</t>
-        </is>
-      </c>
-      <c r="G259" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Categoría</t>
-        </is>
-      </c>
-      <c r="H259" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Latifoliada / Acicular / Escuamiforme / Palmera</t>
-        </is>
-      </c>
-      <c r="I259" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Obligatorio para completar la clasificación del catálogo</t>
-        </is>
-      </c>
-      <c r="J259" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">La plataforma lo vincula al árbol mediante especie_cientifica.</t>
-        </is>
-      </c>
-      <c r="K259" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Al completar o actualizar la clasificación de la especie.</t>
-        </is>
-      </c>
-      <c r="L259" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Seleccionar una única categoría según el follaje adulto; no considerar el follaje juvenil. Si la morfología no coincide exactamente con una categoría, asignar la más cercana: las estructuras planas que cumplen función foliar, como los filodios, se clasifican como Latifoliada; las hojas reducidas a escamas sobre ramillas verdes se clasifican como Escuamiforme. Si aún no se conoce, dejar nulo; no inventarlo ni bloquear el registro del árbol. No duplicar en ARBOLES. Si el árbol no tiene especie_cientifica vigente, no mostrar valor.</t>
-        </is>
       </c>
     </row>
     <row r="260" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A260" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">PROYECTOS</t>
+          <t xml:space="preserve">CATALOGO_ESPECIES</t>
         </is>
       </c>
       <c r="B260" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">id_proyecto</t>
+          <t xml:space="preserve">origen_biogeografico</t>
         </is>
       </c>
       <c r="C260" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Generado por plataforma</t>
+          <t xml:space="preserve">Manual</t>
         </is>
       </c>
       <c r="D260" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sistema</t>
+          <t xml:space="preserve">Inspector</t>
         </is>
       </c>
       <c r="E260" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Asignación automática al crear el proyecto.</t>
+          <t xml:space="preserve">Asignación según la distribución natural de la especie respecto de Chile, consultando el Catálogo de las plantas vasculares de Chile (Rodríguez et al., 2018) o su versión en línea vigente.</t>
         </is>
       </c>
       <c r="F260" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Identificador único y estable del proyecto, que separa inventarios, delimitación territorial y acceso de usuarios.</t>
+          <t xml:space="preserve">Clasificación de la especie según su procedencia biogeográfica respecto del territorio chileno. Endémica: especie nativa cuya distribución natural está restringida a Chile. Nativa: especie nativa de Chile cuya distribución natural no se restringe al país. Introducida: especie exótica presente en Chile fuera de su distribución natural.</t>
         </is>
       </c>
       <c r="G260" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Identificador (texto)</t>
+          <t xml:space="preserve">Categoría</t>
         </is>
       </c>
       <c r="H260" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">No aplica</t>
+          <t xml:space="preserve">Nativa / Endémica / Introducida</t>
         </is>
       </c>
       <c r="I260" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obligatorio</t>
+          <t xml:space="preserve">Obligatorio para completar la clasificación del catálogo</t>
         </is>
       </c>
       <c r="J260" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Asignación automática única.</t>
+          <t xml:space="preserve">La plataforma lo vincula al árbol mediante especie_cientifica.</t>
         </is>
       </c>
       <c r="K260" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Al crear el proyecto.</t>
+          <t xml:space="preserve">Al completar o actualizar la clasificación de la especie.</t>
         </is>
       </c>
       <c r="L260" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">No editable. Solo el Administrador puede crear proyectos.</t>
+          <t xml:space="preserve">Categorías excluyentes: una especie endémica no se registra como Nativa. Considerar la distribución natural de la especie respecto de Chile, no el lugar de plantación ni el origen del ejemplar. Si aún no se conoce, dejar nulo; no inventarlo ni bloquear el registro del árbol. Se muestra en la ficha del árbol mediante especie_cientifica; no se ingresa por ejemplar ni se duplica en ARBOLES. Si el árbol no tiene especie_cientifica vigente, se informa como Origen no determinado.</t>
         </is>
       </c>
     </row>
     <row r="261" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A261" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">PROYECTOS</t>
+          <t xml:space="preserve">CATALOGO_ESPECIES</t>
         </is>
       </c>
       <c r="B261" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">nombre_proyecto</t>
+          <t xml:space="preserve">persistencia_follaje</t>
         </is>
       </c>
       <c r="C261" s="33" t="inlineStr">
@@ -23288,169 +23377,355 @@
       </c>
       <c r="D261" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Administrador</t>
+          <t xml:space="preserve">Inspector</t>
         </is>
       </c>
       <c r="E261" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ingreso del nombre al crear o editar el proyecto.</t>
+          <t xml:space="preserve">Asignación según fuentes botánicas de referencia al incorporar o completar la especie en el catálogo.</t>
         </is>
       </c>
       <c r="F261" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nombre visible del proyecto.</t>
+          <t xml:space="preserve">Comportamiento habitual del follaje de la especie a lo largo del año. Perennifolia: conserva follaje funcional durante todo el año, con renovación gradual. Caducifolia: pierde la totalidad del follaje durante la estación desfavorable. Semicaducifolia: pierde parcialmente el follaje, o lo pierde por un período breve, según las condiciones climáticas del año.</t>
         </is>
       </c>
       <c r="G261" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Texto</t>
+          <t xml:space="preserve">Categoría</t>
         </is>
       </c>
       <c r="H261" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">No aplica</t>
+          <t xml:space="preserve">Perennifolia / Caducifolia / Semicaducifolia</t>
         </is>
       </c>
       <c r="I261" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obligatorio</t>
+          <t xml:space="preserve">Obligatorio para completar la clasificación del catálogo</t>
         </is>
       </c>
       <c r="J261" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">No aplica.</t>
+          <t xml:space="preserve">La plataforma la vincula al árbol mediante especie_cientifica.</t>
         </is>
       </c>
       <c r="K261" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Al crear o editar el proyecto.</t>
+          <t xml:space="preserve">Al completar o actualizar la clasificación de la especie.</t>
         </is>
       </c>
       <c r="L261" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">No vacío. Su modificación no altera id_proyecto.</t>
+          <t xml:space="preserve">Corresponde al comportamiento habitual de la especie, no a la condición observada en el ejemplar. Si las fuentes describen un comportamiento variable, registrar el habitual en las condiciones climáticas de Valparaíso. Si aún no se conoce, dejar nulo; no inventarla ni bloquear el registro del árbol. No duplicar en ARBOLES. Si el árbol no tiene especie_cientifica vigente, no mostrar valor.</t>
         </is>
       </c>
     </row>
     <row r="262" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A262" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">MIEMBROS_PROYECTO</t>
+          <t xml:space="preserve">CATALOGO_ESPECIES</t>
         </is>
       </c>
       <c r="B262" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">id_proyecto</t>
+          <t xml:space="preserve">tipo_hoja</t>
         </is>
       </c>
       <c r="C262" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vinculado por plataforma</t>
+          <t xml:space="preserve">Manual</t>
         </is>
       </c>
       <c r="D262" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Administrador</t>
+          <t xml:space="preserve">Inspector</t>
         </is>
       </c>
       <c r="E262" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Selección del proyecto al asignar un miembro.</t>
+          <t xml:space="preserve">Asignación según fuentes botánicas de referencia al incorporar o completar la especie en el catálogo.</t>
         </is>
       </c>
       <c r="F262" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proyecto al que se asigna el usuario.</t>
+          <t xml:space="preserve">Morfología predominante de las hojas adultas de la especie. Latifoliada: lámina ancha y plana. Acicular: hoja alargada y angosta, en forma de aguja. Escuamiforme: hoja reducida a escamas adosadas a la ramilla. Palmera: hoja de palmera, palmada o pinnada.</t>
         </is>
       </c>
       <c r="G262" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Identificador (texto)</t>
+          <t xml:space="preserve">Categoría</t>
         </is>
       </c>
       <c r="H262" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">No aplica</t>
+          <t xml:space="preserve">Latifoliada / Acicular / Escuamiforme / Palmera</t>
         </is>
       </c>
       <c r="I262" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obligatorio</t>
+          <t xml:space="preserve">Obligatorio para completar la clasificación del catálogo</t>
         </is>
       </c>
       <c r="J262" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">No aplica.</t>
+          <t xml:space="preserve">La plataforma lo vincula al árbol mediante especie_cientifica.</t>
         </is>
       </c>
       <c r="K262" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Al asignar un usuario a un proyecto.</t>
+          <t xml:space="preserve">Al completar o actualizar la clasificación de la especie.</t>
         </is>
       </c>
       <c r="L262" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Referencia válida a PROYECTOS. Un usuario puede pertenecer a varios proyectos; no repetir la misma combinación id_proyecto e id_usuario.</t>
+          <t xml:space="preserve">Seleccionar una única categoría según el follaje adulto; no considerar el follaje juvenil. Si la morfología no coincide exactamente con una categoría, asignar la más cercana: las estructuras planas que cumplen función foliar, como los filodios, se clasifican como Latifoliada; las hojas reducidas a escamas sobre ramillas verdes se clasifican como Escuamiforme. Si aún no se conoce, dejar nulo; no inventarlo ni bloquear el registro del árbol. No duplicar en ARBOLES. Si el árbol no tiene especie_cientifica vigente, no mostrar valor.</t>
         </is>
       </c>
     </row>
     <row r="263" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A263" s="41" t="inlineStr">
         <is>
+          <t xml:space="preserve">PROYECTOS</t>
+        </is>
+      </c>
+      <c r="B263" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">id_proyecto</t>
+        </is>
+      </c>
+      <c r="C263" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Generado por plataforma</t>
+        </is>
+      </c>
+      <c r="D263" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sistema</t>
+        </is>
+      </c>
+      <c r="E263" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Asignación automática al crear el proyecto.</t>
+        </is>
+      </c>
+      <c r="F263" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Identificador único y estable del proyecto, que separa inventarios, delimitación territorial y acceso de usuarios.</t>
+        </is>
+      </c>
+      <c r="G263" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Identificador (texto)</t>
+        </is>
+      </c>
+      <c r="H263" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No aplica</t>
+        </is>
+      </c>
+      <c r="I263" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Obligatorio</t>
+        </is>
+      </c>
+      <c r="J263" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Asignación automática única.</t>
+        </is>
+      </c>
+      <c r="K263" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Al crear el proyecto.</t>
+        </is>
+      </c>
+      <c r="L263" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No editable. Solo el Administrador puede crear proyectos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="264" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A264" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PROYECTOS</t>
+        </is>
+      </c>
+      <c r="B264" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nombre_proyecto</t>
+        </is>
+      </c>
+      <c r="C264" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="D264" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Administrador</t>
+        </is>
+      </c>
+      <c r="E264" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ingreso del nombre al crear o editar el proyecto.</t>
+        </is>
+      </c>
+      <c r="F264" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nombre visible del proyecto.</t>
+        </is>
+      </c>
+      <c r="G264" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Texto</t>
+        </is>
+      </c>
+      <c r="H264" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No aplica</t>
+        </is>
+      </c>
+      <c r="I264" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Obligatorio</t>
+        </is>
+      </c>
+      <c r="J264" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No aplica.</t>
+        </is>
+      </c>
+      <c r="K264" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Al crear o editar el proyecto.</t>
+        </is>
+      </c>
+      <c r="L264" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No vacío. Su modificación no altera id_proyecto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="265" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A265" s="41" t="inlineStr">
+        <is>
           <t xml:space="preserve">MIEMBROS_PROYECTO</t>
         </is>
       </c>
-      <c r="B263" s="41" t="inlineStr">
+      <c r="B265" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">id_proyecto</t>
+        </is>
+      </c>
+      <c r="C265" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vinculado por plataforma</t>
+        </is>
+      </c>
+      <c r="D265" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Administrador</t>
+        </is>
+      </c>
+      <c r="E265" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Selección del proyecto al asignar un miembro.</t>
+        </is>
+      </c>
+      <c r="F265" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proyecto al que se asigna el usuario.</t>
+        </is>
+      </c>
+      <c r="G265" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Identificador (texto)</t>
+        </is>
+      </c>
+      <c r="H265" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No aplica</t>
+        </is>
+      </c>
+      <c r="I265" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Obligatorio</t>
+        </is>
+      </c>
+      <c r="J265" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No aplica.</t>
+        </is>
+      </c>
+      <c r="K265" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Al asignar un usuario a un proyecto.</t>
+        </is>
+      </c>
+      <c r="L265" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Referencia válida a PROYECTOS. Un usuario puede pertenecer a varios proyectos; no repetir la misma combinación id_proyecto e id_usuario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="266" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A266" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIEMBROS_PROYECTO</t>
+        </is>
+      </c>
+      <c r="B266" s="41" t="inlineStr">
         <is>
           <t xml:space="preserve">id_usuario</t>
         </is>
       </c>
-      <c r="C263" s="33" t="inlineStr">
+      <c r="C266" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">Vinculado por plataforma</t>
         </is>
       </c>
-      <c r="D263" s="33" t="inlineStr">
+      <c r="D266" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">Administrador</t>
         </is>
       </c>
-      <c r="E263" s="41" t="inlineStr">
+      <c r="E266" s="41" t="inlineStr">
         <is>
           <t xml:space="preserve">Selección del usuario al asignarlo al proyecto.</t>
         </is>
       </c>
-      <c r="F263" s="33" t="inlineStr">
+      <c r="F266" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">Usuario con acceso al proyecto.</t>
         </is>
       </c>
-      <c r="G263" s="33" t="inlineStr">
+      <c r="G266" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">Identificador (texto)</t>
         </is>
       </c>
-      <c r="H263" s="33" t="inlineStr">
+      <c r="H266" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">No aplica</t>
         </is>
       </c>
-      <c r="I263" s="33" t="inlineStr">
+      <c r="I266" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">Obligatorio</t>
         </is>
       </c>
-      <c r="J263" s="33" t="inlineStr">
+      <c r="J266" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">No aplica.</t>
         </is>
       </c>
-      <c r="K263" s="33" t="inlineStr">
+      <c r="K266" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">Al asignar un usuario a un proyecto.</t>
         </is>
       </c>
-      <c r="L263" s="33" t="inlineStr">
+      <c r="L266" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">Referencia válida a USUARIOS con activo = Sí. El rol del usuario se mantiene en USUARIOS.Rol.</t>
         </is>

</xml_diff>

<commit_message>
[CC-030] Excel: IN-RSU-05 pasa a Moderada
Con afectacion_fisica_red_subterranea = Sí y
compromete_funcionalidad_red_subterranea = No determinado, la categoría
parcial de M04 pasa de Leve (1) a Moderada (2): el mínimo por el daño
físico confirmado, nunca inferior a IN-RSU-04. Decisión de la autora
(2026-10-20), observación de la verificación final de AM-08. IN-RAE no
cambia.

Solo el Excel (REGLAS_INDICADORES F97 y G97). Sin cambios de código,
migraciones, RLS ni Supabase.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/excel/Base de Datos Valpo Verde.xlsx
+++ b/docs/excel/Base de Datos Valpo Verde.xlsx
@@ -11367,12 +11367,12 @@
       </c>
       <c r="F97" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leve</t>
+          <t xml:space="preserve">Moderada</t>
         </is>
       </c>
       <c r="G97" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[AM-08] Excel: 2.0.0 publicada en VERSION; cuentas ficticias en USUARIOS
- VERSION, fila 5: estado "publicada", fecha_publicacion y
  fecha_aprobacion 2026-10-20, aprobado_por marybaxmann, tag_git
  metodologia-v2.0.0; observaciones con IN-RSU-05 (CC-030, PR #29).
  Aprobación expresa de la autora, 2026-10-20.
- USUARIOS: nombres y correos reales reemplazados por cuentas ficticias
  (dominio reservado example.org), sin hipervínculos; se vacían en la tabla
  interna de textos los valores personales que ya no usa ninguna celda.

Solo el Excel. Sin cambios de código, migraciones, RLS ni Supabase.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/excel/Base de Datos Valpo Verde.xlsx
+++ b/docs/excel/Base de Datos Valpo Verde.xlsx
@@ -878,10 +878,10 @@
     <t>USR-001</t>
   </si>
   <si>
-    <t>Valentina Jiménez</t>
-  </si>
-  <si>
-    <t>valejimenezvpjc@gmail.com</t>
+    <t/>
+  </si>
+  <si>
+    <t/>
   </si>
   <si>
     <t>Administrador</t>
@@ -890,25 +890,25 @@
     <t>USR-002</t>
   </si>
   <si>
-    <t>Mariajosé Baxmann</t>
-  </si>
-  <si>
-    <t>baxmannmariajose@gmail.com</t>
-  </si>
-  <si>
-    <t>baxmannroman12@gmail.com</t>
+    <t/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t/>
   </si>
   <si>
     <t>Usuario municipal</t>
   </si>
   <si>
-    <t>valazjc@gmail.com</t>
+    <t/>
   </si>
   <si>
     <t>Inspector</t>
   </si>
   <si>
-    <t>valentina.jimenezc@estudiantes.uv.cl</t>
+    <t/>
   </si>
   <si>
     <t>Encargado de mantención</t>
@@ -11623,7 +11623,12 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">aprobación de publicación pendiente</t>
+          <t xml:space="preserve">publicada</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-20</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
@@ -11631,6 +11636,21 @@
           <t xml:space="preserve">CC-024, CC-026, CC-027, CC-028, CC-029, CC-030, CC-031, CC-032, CC-034, CC-035, CC-036, CC-037, CC-039</t>
         </is>
       </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">marybaxmann</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-20</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">metodologia-v2.0.0</t>
+        </is>
+      </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">2.0.0 en preparación (fuente única desde CC-028)</t>
@@ -11638,7 +11658,7 @@
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Incluye AM-10: textos de CC-031, CC-032, CC-036 y CC-037; rango_edad_estimada_anios opcional (CC-039) y referencia estacional de la defoliación en caducifolias (AM-11). El Excel maestro es la única fuente (CC-028) y los diagramas no forman parte del paquete (CC-030). INDICES sigue en propuesta (DM-09). Todas las reglas de REGLAS_INDICADORES son vigentes en esta versión (PR-011 v3.0). Al publicar, la autora completa fecha_publicacion, aprobado_por, fecha_aprobacion y tag_git, y cambia el estado a publicada.</t>
+          <t xml:space="preserve">Incluye AM-10: textos de CC-031, CC-032, CC-036 y CC-037; rango_edad_estimada_anios opcional (CC-039) y referencia estacional de la defoliación en caducifolias (AM-11). El Excel maestro es la única fuente (CC-028) y los diagramas no forman parte del paquete (CC-030). INDICES sigue en propuesta (DM-09). Todas las reglas de REGLAS_INDICADORES son vigentes en esta versión (PR-011 v3.0). Incluye también IN-RSU-05 = Moderada (CC-030, PR #29). Primera versión publicada, el 2026-10-20 (AM-08).</t>
         </is>
       </c>
     </row>
@@ -12826,11 +12846,15 @@
       <c r="A2" t="s">
         <v>249</v>
       </c>
-      <c r="B2" t="s">
-        <v>250</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>251</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Administrador de ejemplo 1</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">admin1@example.org</t>
+        </is>
       </c>
       <c r="D2" t="s">
         <v>252</v>
@@ -12843,11 +12867,15 @@
       <c r="A3" t="s">
         <v>253</v>
       </c>
-      <c r="B3" t="s">
-        <v>254</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>255</v>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Administrador de ejemplo 2</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">admin2@example.org</t>
+        </is>
       </c>
       <c r="D3" t="s">
         <v>252</v>
@@ -12860,11 +12888,15 @@
       <c r="A4" t="s">
         <v>219</v>
       </c>
-      <c r="B4" t="s">
-        <v>254</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>256</v>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Usuario municipal de ejemplo</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">municipal@example.org</t>
+        </is>
       </c>
       <c r="D4" t="s">
         <v>257</v>
@@ -12877,11 +12909,15 @@
       <c r="A5" t="s">
         <v>192</v>
       </c>
-      <c r="B5" t="s">
-        <v>250</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>258</v>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Inspector de ejemplo</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">inspector@example.org</t>
+        </is>
       </c>
       <c r="D5" t="s">
         <v>259</v>
@@ -12894,11 +12930,15 @@
       <c r="A6" t="s">
         <v>212</v>
       </c>
-      <c r="B6" t="s">
-        <v>250</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>260</v>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Encargado de mantención de ejemplo</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mantencion@example.org</t>
+        </is>
       </c>
       <c r="D6" t="s">
         <v>261</v>
@@ -12908,13 +12948,6 @@
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" xr:uid="{00000000-0004-0000-0600-000000000000}"/>
-    <hyperlink ref="C3" r:id="rId2" xr:uid="{00000000-0004-0000-0600-000001000000}"/>
-    <hyperlink ref="C4" r:id="rId3" xr:uid="{00000000-0004-0000-0600-000002000000}"/>
-    <hyperlink ref="C5" r:id="rId4" xr:uid="{00000000-0004-0000-0600-000003000000}"/>
-    <hyperlink ref="C6" r:id="rId5" xr:uid="{00000000-0004-0000-0600-000004000000}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
[CC-042] Excel: estado_proyecto (Activo / Cerrado) en PROYECTOS
- DICCIONARIO_CAMPOS: fila nueva 265 (estado_proyecto); MIEMBROS_PROYECTO
  pasa a D-266 y D-267.
- PROYECTOS: cabecera C1.
- REGLAS_GENERALES fila 27 (Proyectos): proyecto Cerrado en solo consulta;
  no se cierra con OT abiertas ni incidencias Ingresada o En revisión;
  reabrible; solo el Administrador.
- VERSION fila 6: 2.0.1 en preparación (PATCH, rule_version sigue 2.0).
- registro-cambios: índice y ficha de CC-042.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/excel/Base de Datos Valpo Verde.xlsx
+++ b/docs/excel/Base de Datos Valpo Verde.xlsx
@@ -7135,7 +7135,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -7716,6 +7716,28 @@
         </is>
       </c>
     </row>
+    <row r="27" spans="1:4">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proyectos</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Un proyecto con estado_proyecto = Cerrado queda en solo consulta: se pueden ver sus árboles, mapa, fichas, indicadores e historial, pero no se registran árboles ni se crean OT, inspecciones, mantenimientos o incidencias, y el formulario QR de sus árboles no recibe incidencias. La delimitación del sector no se modifica; el Administrador puede seguir gestionando los miembros. Solo el Administrador cierra o reabre un proyecto, y no puede cerrarlo mientras alguna OT esté Pendiente, Programada o En ejecución o alguna incidencia esté Ingresada o En revisión.</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">estado_proyecto; estado_ot; estado_incidencia</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PROYECTOS; ARBOLES; ORDENES DE TRABAJO; INSPECCION; MANTENIMIENTO; INCIDENCIA; SECTORES; MIEMBROS_PROYECTO</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -7723,14 +7745,15 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="40" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:3">
       <c r="A1" t="inlineStr">
         <is>
           <t>id_proyecto</t>
@@ -7739,6 +7762,11 @@
       <c r="B1" t="inlineStr">
         <is>
           <t>nombre_proyecto</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>estado_proyecto</t>
         </is>
       </c>
     </row>
@@ -11457,7 +11485,7 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -11659,6 +11687,38 @@
       <c r="J5" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Incluye AM-10: textos de CC-031, CC-032, CC-036 y CC-037; rango_edad_estimada_anios opcional (CC-039) y referencia estacional de la defoliación en caducifolias (AM-11). El Excel maestro es la única fuente (CC-028) y los diagramas no forman parte del paquete (CC-030). INDICES sigue en propuesta (DM-09). Todas las reglas de REGLAS_INDICADORES son vigentes en esta versión (PR-011 v3.0). Incluye también IN-RSU-05 = Moderada (CC-030, PR #29). Primera versión publicada, el 2026-10-20 (AM-08).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2.0.1</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2.0</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">en preparación</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CC-042</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2.0.0</t>
+        </is>
+      </c>
+      <c r="J6" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PATCH: agrega PROYECTOS.estado_proyecto (Activo / Cerrado) y su regla en REGLAS_GENERALES (Proyectos). El campo no participa en ninguna regla de cálculo: no cambia resultados y rule_version sigue siendo 2.0. NO publicada.</t>
         </is>
       </c>
     </row>
@@ -13155,7 +13215,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M266"/>
+  <dimension ref="A1:M267"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="24" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7" style="41" customWidth="1"/>
@@ -23640,45 +23700,45 @@
         </is>
       </c>
     </row>
-    <row r="265" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A265" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">MIEMBROS_PROYECTO</t>
+          <t xml:space="preserve">PROYECTOS</t>
         </is>
       </c>
       <c r="B265" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">id_proyecto</t>
+          <t xml:space="preserve">estado_proyecto</t>
         </is>
       </c>
       <c r="C265" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vinculado por plataforma</t>
+          <t xml:space="preserve">Manual</t>
         </is>
       </c>
       <c r="D265" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Administrador</t>
+          <t xml:space="preserve">Administrador / Sistema</t>
         </is>
       </c>
       <c r="E265" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Selección del proyecto al asignar un miembro.</t>
+          <t xml:space="preserve">Valor inicial asignado por la plataforma al crear el proyecto; el Administrador lo cambia al cerrar o reabrir el proyecto.</t>
         </is>
       </c>
       <c r="F265" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proyecto al que se asigna el usuario.</t>
+          <t xml:space="preserve">Situación del proyecto. Activo: permite registrar y gestionar árboles, OT, inspecciones, mantenimientos e incidencias. Cerrado: el proyecto queda en solo consulta.</t>
         </is>
       </c>
       <c r="G265" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Identificador (texto)</t>
+          <t xml:space="preserve">Categoría</t>
         </is>
       </c>
       <c r="H265" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">No aplica</t>
+          <t xml:space="preserve">Activo / Cerrado</t>
         </is>
       </c>
       <c r="I265" s="33" t="inlineStr">
@@ -23693,12 +23753,12 @@
       </c>
       <c r="K265" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Al asignar un usuario a un proyecto.</t>
+          <t xml:space="preserve">Al crear el proyecto y al cerrarlo o reabrirlo.</t>
         </is>
       </c>
       <c r="L265" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Referencia válida a PROYECTOS. Un usuario puede pertenecer a varios proyectos; no repetir la misma combinación id_proyecto e id_usuario.</t>
+          <t xml:space="preserve">Valor inicial: Activo. Solo el Administrador cierra o reabre el proyecto. No permitir Cerrado mientras alguna OT del proyecto tenga estado_ot = Pendiente, Programada o En ejecución, o alguna incidencia de sus árboles tenga estado_incidencia = Ingresada o En revisión. Un proyecto Cerrado puede reabrirse (Activo). El cambio de estado no altera id_proyecto ni el historial.</t>
         </is>
       </c>
     </row>
@@ -23710,55 +23770,117 @@
       </c>
       <c r="B266" s="41" t="inlineStr">
         <is>
+          <t xml:space="preserve">id_proyecto</t>
+        </is>
+      </c>
+      <c r="C266" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vinculado por plataforma</t>
+        </is>
+      </c>
+      <c r="D266" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Administrador</t>
+        </is>
+      </c>
+      <c r="E266" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Selección del proyecto al asignar un miembro.</t>
+        </is>
+      </c>
+      <c r="F266" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proyecto al que se asigna el usuario.</t>
+        </is>
+      </c>
+      <c r="G266" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Identificador (texto)</t>
+        </is>
+      </c>
+      <c r="H266" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No aplica</t>
+        </is>
+      </c>
+      <c r="I266" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Obligatorio</t>
+        </is>
+      </c>
+      <c r="J266" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No aplica.</t>
+        </is>
+      </c>
+      <c r="K266" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Al asignar un usuario a un proyecto.</t>
+        </is>
+      </c>
+      <c r="L266" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Referencia válida a PROYECTOS. Un usuario puede pertenecer a varios proyectos; no repetir la misma combinación id_proyecto e id_usuario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="267" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A267" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MIEMBROS_PROYECTO</t>
+        </is>
+      </c>
+      <c r="B267" s="41" t="inlineStr">
+        <is>
           <t xml:space="preserve">id_usuario</t>
         </is>
       </c>
-      <c r="C266" s="33" t="inlineStr">
+      <c r="C267" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">Vinculado por plataforma</t>
         </is>
       </c>
-      <c r="D266" s="33" t="inlineStr">
+      <c r="D267" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">Administrador</t>
         </is>
       </c>
-      <c r="E266" s="41" t="inlineStr">
+      <c r="E267" s="41" t="inlineStr">
         <is>
           <t xml:space="preserve">Selección del usuario al asignarlo al proyecto.</t>
         </is>
       </c>
-      <c r="F266" s="33" t="inlineStr">
+      <c r="F267" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">Usuario con acceso al proyecto.</t>
         </is>
       </c>
-      <c r="G266" s="33" t="inlineStr">
+      <c r="G267" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">Identificador (texto)</t>
         </is>
       </c>
-      <c r="H266" s="33" t="inlineStr">
+      <c r="H267" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">No aplica</t>
         </is>
       </c>
-      <c r="I266" s="33" t="inlineStr">
+      <c r="I267" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">Obligatorio</t>
         </is>
       </c>
-      <c r="J266" s="33" t="inlineStr">
+      <c r="J267" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">No aplica.</t>
         </is>
       </c>
-      <c r="K266" s="33" t="inlineStr">
+      <c r="K267" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">Al asignar un usuario a un proyecto.</t>
         </is>
       </c>
-      <c r="L266" s="33" t="inlineStr">
+      <c r="L267" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">Referencia válida a USUARIOS con activo = Sí. El rol del usuario se mantiene en USUARIOS.Rol.</t>
         </is>

</xml_diff>

<commit_message>
[CC-042] Cierre del proyecto permitido con OT o incidencias abiertas (quedan congeladas)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/excel/Base de Datos Valpo Verde.xlsx
+++ b/docs/excel/Base de Datos Valpo Verde.xlsx
@@ -7724,7 +7724,7 @@
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Un proyecto con estado_proyecto = Cerrado queda en solo consulta: se pueden ver sus árboles, mapa, fichas, indicadores e historial, pero no se registran árboles ni se crean OT, inspecciones, mantenimientos o incidencias, y el formulario QR de sus árboles no recibe incidencias. La delimitación del sector no se modifica; el Administrador puede seguir gestionando los miembros. Solo el Administrador cierra o reabre un proyecto, y no puede cerrarlo mientras alguna OT esté Pendiente, Programada o En ejecución o alguna incidencia esté Ingresada o En revisión.</t>
+          <t xml:space="preserve">Un proyecto con estado_proyecto = Cerrado queda en solo consulta: se pueden ver sus árboles, mapa, fichas, indicadores e historial, pero no se registran árboles ni se crean OT, inspecciones, mantenimientos o incidencias, y el formulario QR de sus árboles no recibe incidencias. La delimitación del sector no se modifica; el Administrador puede seguir gestionando los miembros. Solo el Administrador cierra o reabre un proyecto. Puede cerrarse aunque existan OT o incidencias abiertas: mientras el proyecto está Cerrado, esas OT e incidencias se conservan en su estado y no avanzan hasta que el proyecto se reabra.</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
@@ -23758,7 +23758,7 @@
       </c>
       <c r="L265" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Valor inicial: Activo. Solo el Administrador cierra o reabre el proyecto. No permitir Cerrado mientras alguna OT del proyecto tenga estado_ot = Pendiente, Programada o En ejecución, o alguna incidencia de sus árboles tenga estado_incidencia = Ingresada o En revisión. Un proyecto Cerrado puede reabrirse (Activo). El cambio de estado no altera id_proyecto ni el historial.</t>
+          <t xml:space="preserve">Valor inicial: Activo. Solo el Administrador cierra o reabre el proyecto. Puede cerrarse aunque existan OT o incidencias abiertas: mientras el proyecto está Cerrado, esas OT e incidencias se conservan en su estado y no avanzan hasta que el proyecto se reabra. Un proyecto Cerrado puede reabrirse (Activo). El cambio de estado no altera id_proyecto ni el historial.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[AM-12] Excel: textos de CC-040; versión en preparación 2.1.0
- REGLAS_GENERALES fila 28 (Preguardado y finalización): alcance de la
  evaluación según tipo_inspeccion_realizada, evaluación vigente campo por
  campo, fotografías por tipo, campos por subtipo de Monitoreo, cavidades
  internas Sí/No en la instrumental, No determinado si falta un valor
  vigente y ajustes descartados en el recálculo.
- DICCIONARIO_CAMPOS: D-209 J y L (estado_registro); D-27 I y K
  (fotografias_arbol).
- VERSION fila 6: 2.0.1 → 2.1.0, rule_version 2.1, CC-040 y CC-042.
- Export regenerado; verificar_14_9.py sin hallazgos.
- registro-cambios (CC-040, CC-042), roadmap (AM-12) y diseño de la Fase 3.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/excel/Base de Datos Valpo Verde.xlsx
+++ b/docs/excel/Base de Datos Valpo Verde.xlsx
@@ -7135,7 +7135,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -7735,6 +7735,28 @@
       <c r="D27" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">PROYECTOS; ARBOLES; ORDENES DE TRABAJO; INSPECCION; MANTENIMIENTO; INCIDENCIA; SECTORES; MIEMBROS_PROYECTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Preguardado y finalización</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La evaluación que se exige para finalizar depende de tipo_inspeccion_realizada. Evaluación inicial, Reevaluación y Levantamiento: evaluación completa (todos los campos Obligatorios y los Condicionales activados de ARBOLES y REGISTRO_EVALUACION). Evaluación instrumental: solo los campos de cavidad basal y de tronco; resuelve el No determinado de Requiere evaluación instrumental. Monitoreo: solo los campos de su subtipo (Fitosanitario, Estructural o Vitalidad). En una inspección parcial, los campos registrados reemplazan el valor vigente del árbol al completar la OT; los demás conservan su valor vigente anterior. El historial no se sobrescribe: cada valor queda vinculado a la inspección que lo registró. Las clasificaciones se calculan con los valores vigentes resultantes: para cada campo, el último valor entre las inspecciones no anuladas de OT completadas. Las cuatro vistas fotográficas del árbol se exigen solo en Evaluación inicial, Reevaluación y Levantamiento; la Evaluación instrumental no considera fotografías y en el Monitoreo no son obligatorias. Campos por subtipo de Monitoreo: Fitosanitario = defoliacion_estimada_pct, clorosis_pct, necrosis_pct, muerte_regresiva_copa_pct y presenta_exudaciones; Estructural = las entradas de R01, R02 y R03; Vitalidad = clasificacion_vitalidad. En la Evaluación instrumental, cavidad_basal_interna y cavidad_interna_tronco solo admiten Sí o No. Si falta un valor vigente que una clasificación necesita, esa clasificación queda No determinado. Si al recalcular la evaluación vigente el valor calculado cambia, el ajuste del Inspector se descarta y queda marcado para su revisión.</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tipo_inspeccion_realizada; subtipo_inspeccion; estado_registro; fotografias_arbol; campos de cavidad; campos de cada subtipo de Monitoreo</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INSPECCION; REGISTRO_EVALUACION; ARBOLES</t>
         </is>
       </c>
     </row>
@@ -11693,12 +11715,12 @@
     <row r="6" spans="1:10">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">2.0.1</t>
+          <t xml:space="preserve">2.1.0</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">2.0</t>
+          <t xml:space="preserve">2.1</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
@@ -11708,7 +11730,7 @@
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">CC-042</t>
+          <t xml:space="preserve">CC-040, CC-042</t>
         </is>
       </c>
       <c r="I6" s="7" t="inlineStr">
@@ -11718,7 +11740,7 @@
       </c>
       <c r="J6" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">PATCH: agrega PROYECTOS.estado_proyecto (Activo / Cerrado) y su regla en REGLAS_GENERALES (Proyectos). El campo no participa en ninguna regla de cálculo: no cambia resultados y rule_version sigue siendo 2.0. NO publicada.</t>
+          <t xml:space="preserve">MINOR: CC-040 cambia los valores con que se calculan las clasificaciones (alcance de la evaluación según el tipo de inspección, evaluación vigente compuesta campo por campo, campos por subtipo de Monitoreo, cavidades internas Sí/No en la instrumental y ajustes del Inspector en el recálculo; REGLAS_GENERALES fila 28, D-209 y D-27; AM-12). Incluye CC-042: PROYECTOS.estado_proyecto (Activo / Cerrado) y REGLAS_GENERALES fila 27. NO publicada.</t>
         </is>
       </c>
     </row>
@@ -14257,14 +14279,18 @@
       <c r="H27" s="50" t="s">
         <v>1438</v>
       </c>
-      <c r="I27" s="50" t="s">
-        <v>1439</v>
+      <c r="I27" s="50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Obligatorio para finalizar la Evaluación inicial, la Reevaluación y el Levantamiento</t>
+        </is>
       </c>
       <c r="J27" s="50" t="s">
         <v>1440</v>
       </c>
-      <c r="K27" s="50" t="s">
-        <v>1441</v>
+      <c r="K27" s="50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">En la inspección de Evaluación inicial, Reevaluación o Levantamiento mediante OT. No aplica en la Evaluación instrumental; en el Monitoreo no es obligatoria.</t>
+        </is>
       </c>
       <c r="L27" s="50" t="s">
         <v>1442</v>
@@ -21388,7 +21414,7 @@
       </c>
       <c r="J209" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Finalizado cuando están completos todos los campos obligatorios y los condicionales activados de la inspección, de su REGISTRO_EVALUACION y de los datos técnicos del árbol registrados en ella; en otro caso, Preguardado. Anulado solo desde Finalizado, cuando el Inspector registra motivo_anulacion.</t>
+          <t xml:space="preserve">Finalizado cuando están completos todos los campos obligatorios y los condicionales activados que exige el tipo de inspección (REGLAS_GENERALES, Preguardado y finalización): evaluación completa en Evaluación inicial, Reevaluación y Levantamiento; campos de cavidad en Evaluación instrumental; campos de su subtipo en Monitoreo. En otro caso, Preguardado. Anulado solo desde Finalizado, cuando el Inspector registra motivo_anulacion.</t>
         </is>
       </c>
       <c r="K209" s="8" t="inlineStr">
@@ -21398,7 +21424,7 @@
       </c>
       <c r="L209" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">No editable manualmente, salvo la anulación por el Inspector. Valor inicial: Preguardado. Una inspección Preguardado o Anulado no modifica la evaluación vigente del árbol. Mientras alguna inspección vinculada esté Preguardado, la OT no puede pasar a estado_ot = Completada. Una medición pendiente no equivale a cero ni a No presenta.</t>
+          <t xml:space="preserve">No editable manualmente, salvo la anulación por el Inspector. Valor inicial: Preguardado. Una inspección Preguardado o Anulado no modifica la evaluación vigente del árbol. Una inspección parcial solo reemplaza los valores vigentes de los campos que registra. Mientras alguna inspección vinculada esté Preguardado, la OT no puede pasar a estado_ot = Completada. Una medición pendiente no equivale a cero ni a No presenta.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[AM-13] Excel: 2.1.0 publicada en VERSION (2026-10-21)
VERSION fila 6: estado publicada, fecha_publicacion y fecha_aprobacion 2026-10-21, aprobado_por marybaxmann, tag_git metodologia-v2.1.0. Export de VERSION regenerado; verificar_14_9.py sin hallazgos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/excel/Base de Datos Valpo Verde.xlsx
+++ b/docs/excel/Base de Datos Valpo Verde.xlsx
@@ -11725,7 +11725,12 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">en preparación</t>
+          <t xml:space="preserve">publicada</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-21</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
@@ -11733,6 +11738,21 @@
           <t xml:space="preserve">CC-040, CC-042</t>
         </is>
       </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">marybaxmann</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-21</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">metodologia-v2.1.0</t>
+        </is>
+      </c>
       <c r="I6" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">2.0.0</t>
@@ -11740,7 +11760,7 @@
       </c>
       <c r="J6" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">MINOR: CC-040 cambia los valores con que se calculan las clasificaciones (alcance de la evaluación según el tipo de inspección, evaluación vigente compuesta campo por campo, campos por subtipo de Monitoreo, cavidades internas Sí/No en la instrumental y ajustes del Inspector en el recálculo; REGLAS_GENERALES fila 28, D-209 y D-27; AM-12). Incluye CC-042: PROYECTOS.estado_proyecto (Activo / Cerrado) y REGLAS_GENERALES fila 27. NO publicada.</t>
+          <t xml:space="preserve">MINOR: CC-040 cambia los valores con que se calculan las clasificaciones (alcance de la evaluación según el tipo de inspección, evaluación vigente compuesta campo por campo, campos por subtipo de Monitoreo, cavidades internas Sí/No en la instrumental y ajustes del Inspector en el recálculo; REGLAS_GENERALES fila 28, D-209 y D-27; AM-12). Incluye CC-042: PROYECTOS.estado_proyecto (Activo / Cerrado) y REGLAS_GENERALES fila 27. Publicada el 2026-10-21 (AM-13), antes de la Fase 4.</t>
         </is>
       </c>
     </row>

</xml_diff>